<commit_message>
Ajoute l’envoi Resend et affine FeexPay
Ajoute des gabarits d’e-mails transactionnels et un pilote Resend configurable, avec une adresse d’équipe dédiée aux demandes. Filtre aussi les moyens de paiement FeexPay selon le choix du client et met à jour les domaines configurés.
</commit_message>
<xml_diff>
--- a/Recette E-Masterclass BigFive — clôture 15-10.xlsx
+++ b/Recette E-Masterclass BigFive — clôture 15-10.xlsx
@@ -1654,6 +1654,7 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
@@ -3165,7 +3166,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:B1179"/>
+  <dimension ref="A1:B1179"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" style="31" min="1" max="1"/>
@@ -3186,6 +3187,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="B4" s="59" t="inlineStr">
         <is>
@@ -3200,6 +3202,37 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
+    <row r="7"/>
+    <row r="8"/>
+    <row r="9"/>
+    <row r="10"/>
+    <row r="11"/>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
     <row r="37">
       <c r="B37" s="59" t="inlineStr">
         <is>
@@ -3214,6 +3247,33 @@
         </is>
       </c>
     </row>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
+    <row r="60"/>
+    <row r="61"/>
+    <row r="62"/>
+    <row r="63"/>
+    <row r="64"/>
+    <row r="65"/>
     <row r="66">
       <c r="B66" s="59" t="inlineStr">
         <is>
@@ -3228,6 +3288,36 @@
         </is>
       </c>
     </row>
+    <row r="68"/>
+    <row r="69"/>
+    <row r="70"/>
+    <row r="71"/>
+    <row r="72"/>
+    <row r="73"/>
+    <row r="74"/>
+    <row r="75"/>
+    <row r="76"/>
+    <row r="77"/>
+    <row r="78"/>
+    <row r="79"/>
+    <row r="80"/>
+    <row r="81"/>
+    <row r="82"/>
+    <row r="83"/>
+    <row r="84"/>
+    <row r="85"/>
+    <row r="86"/>
+    <row r="87"/>
+    <row r="88"/>
+    <row r="89"/>
+    <row r="90"/>
+    <row r="91"/>
+    <row r="92"/>
+    <row r="93"/>
+    <row r="94"/>
+    <row r="95"/>
+    <row r="96"/>
+    <row r="97"/>
     <row r="98">
       <c r="B98" s="59" t="inlineStr">
         <is>
@@ -3242,6 +3332,32 @@
         </is>
       </c>
     </row>
+    <row r="100"/>
+    <row r="101"/>
+    <row r="102"/>
+    <row r="103"/>
+    <row r="104"/>
+    <row r="105"/>
+    <row r="106"/>
+    <row r="107"/>
+    <row r="108"/>
+    <row r="109"/>
+    <row r="110"/>
+    <row r="111"/>
+    <row r="112"/>
+    <row r="113"/>
+    <row r="114"/>
+    <row r="115"/>
+    <row r="116"/>
+    <row r="117"/>
+    <row r="118"/>
+    <row r="119"/>
+    <row r="120"/>
+    <row r="121"/>
+    <row r="122"/>
+    <row r="123"/>
+    <row r="124"/>
+    <row r="125"/>
     <row r="126">
       <c r="B126" s="59" t="inlineStr">
         <is>
@@ -3256,6 +3372,33 @@
         </is>
       </c>
     </row>
+    <row r="128"/>
+    <row r="129"/>
+    <row r="130"/>
+    <row r="131"/>
+    <row r="132"/>
+    <row r="133"/>
+    <row r="134"/>
+    <row r="135"/>
+    <row r="136"/>
+    <row r="137"/>
+    <row r="138"/>
+    <row r="139"/>
+    <row r="140"/>
+    <row r="141"/>
+    <row r="142"/>
+    <row r="143"/>
+    <row r="144"/>
+    <row r="145"/>
+    <row r="146"/>
+    <row r="147"/>
+    <row r="148"/>
+    <row r="149"/>
+    <row r="150"/>
+    <row r="151"/>
+    <row r="152"/>
+    <row r="153"/>
+    <row r="154"/>
     <row r="155">
       <c r="B155" s="59" t="inlineStr">
         <is>
@@ -3270,6 +3413,63 @@
         </is>
       </c>
     </row>
+    <row r="157"/>
+    <row r="158"/>
+    <row r="159"/>
+    <row r="160"/>
+    <row r="161"/>
+    <row r="162"/>
+    <row r="163"/>
+    <row r="164"/>
+    <row r="165"/>
+    <row r="166"/>
+    <row r="167"/>
+    <row r="168"/>
+    <row r="169"/>
+    <row r="170"/>
+    <row r="171"/>
+    <row r="172"/>
+    <row r="173"/>
+    <row r="174"/>
+    <row r="175"/>
+    <row r="176"/>
+    <row r="177"/>
+    <row r="178"/>
+    <row r="179"/>
+    <row r="180"/>
+    <row r="181"/>
+    <row r="182"/>
+    <row r="183"/>
+    <row r="184"/>
+    <row r="185"/>
+    <row r="186"/>
+    <row r="187"/>
+    <row r="188"/>
+    <row r="189"/>
+    <row r="190"/>
+    <row r="191"/>
+    <row r="192"/>
+    <row r="193"/>
+    <row r="194"/>
+    <row r="195"/>
+    <row r="196"/>
+    <row r="197"/>
+    <row r="198"/>
+    <row r="199"/>
+    <row r="200"/>
+    <row r="201"/>
+    <row r="202"/>
+    <row r="203"/>
+    <row r="204"/>
+    <row r="205"/>
+    <row r="206"/>
+    <row r="207"/>
+    <row r="208"/>
+    <row r="209"/>
+    <row r="210"/>
+    <row r="211"/>
+    <row r="212"/>
+    <row r="213"/>
     <row r="214">
       <c r="B214" s="59" t="inlineStr">
         <is>
@@ -3284,6 +3484,33 @@
         </is>
       </c>
     </row>
+    <row r="216"/>
+    <row r="217"/>
+    <row r="218"/>
+    <row r="219"/>
+    <row r="220"/>
+    <row r="221"/>
+    <row r="222"/>
+    <row r="223"/>
+    <row r="224"/>
+    <row r="225"/>
+    <row r="226"/>
+    <row r="227"/>
+    <row r="228"/>
+    <row r="229"/>
+    <row r="230"/>
+    <row r="231"/>
+    <row r="232"/>
+    <row r="233"/>
+    <row r="234"/>
+    <row r="235"/>
+    <row r="236"/>
+    <row r="237"/>
+    <row r="238"/>
+    <row r="239"/>
+    <row r="240"/>
+    <row r="241"/>
+    <row r="242"/>
     <row r="243">
       <c r="B243" s="59" t="inlineStr">
         <is>
@@ -3298,6 +3525,38 @@
         </is>
       </c>
     </row>
+    <row r="245"/>
+    <row r="246"/>
+    <row r="247"/>
+    <row r="248"/>
+    <row r="249"/>
+    <row r="250"/>
+    <row r="251"/>
+    <row r="252"/>
+    <row r="253"/>
+    <row r="254"/>
+    <row r="255"/>
+    <row r="256"/>
+    <row r="257"/>
+    <row r="258"/>
+    <row r="259"/>
+    <row r="260"/>
+    <row r="261"/>
+    <row r="262"/>
+    <row r="263"/>
+    <row r="264"/>
+    <row r="265"/>
+    <row r="266"/>
+    <row r="267"/>
+    <row r="268"/>
+    <row r="269"/>
+    <row r="270"/>
+    <row r="271"/>
+    <row r="272"/>
+    <row r="273"/>
+    <row r="274"/>
+    <row r="275"/>
+    <row r="276"/>
     <row r="277">
       <c r="B277" s="59" t="inlineStr">
         <is>
@@ -3312,6 +3571,38 @@
         </is>
       </c>
     </row>
+    <row r="279"/>
+    <row r="280"/>
+    <row r="281"/>
+    <row r="282"/>
+    <row r="283"/>
+    <row r="284"/>
+    <row r="285"/>
+    <row r="286"/>
+    <row r="287"/>
+    <row r="288"/>
+    <row r="289"/>
+    <row r="290"/>
+    <row r="291"/>
+    <row r="292"/>
+    <row r="293"/>
+    <row r="294"/>
+    <row r="295"/>
+    <row r="296"/>
+    <row r="297"/>
+    <row r="298"/>
+    <row r="299"/>
+    <row r="300"/>
+    <row r="301"/>
+    <row r="302"/>
+    <row r="303"/>
+    <row r="304"/>
+    <row r="305"/>
+    <row r="306"/>
+    <row r="307"/>
+    <row r="308"/>
+    <row r="309"/>
+    <row r="310"/>
     <row r="311">
       <c r="B311" s="59" t="inlineStr">
         <is>
@@ -3326,6 +3617,43 @@
         </is>
       </c>
     </row>
+    <row r="313"/>
+    <row r="314"/>
+    <row r="315"/>
+    <row r="316"/>
+    <row r="317"/>
+    <row r="318"/>
+    <row r="319"/>
+    <row r="320"/>
+    <row r="321"/>
+    <row r="322"/>
+    <row r="323"/>
+    <row r="324"/>
+    <row r="325"/>
+    <row r="326"/>
+    <row r="327"/>
+    <row r="328"/>
+    <row r="329"/>
+    <row r="330"/>
+    <row r="331"/>
+    <row r="332"/>
+    <row r="333"/>
+    <row r="334"/>
+    <row r="335"/>
+    <row r="336"/>
+    <row r="337"/>
+    <row r="338"/>
+    <row r="339"/>
+    <row r="340"/>
+    <row r="341"/>
+    <row r="342"/>
+    <row r="343"/>
+    <row r="344"/>
+    <row r="345"/>
+    <row r="346"/>
+    <row r="347"/>
+    <row r="348"/>
+    <row r="349"/>
     <row r="350">
       <c r="B350" s="59" t="inlineStr">
         <is>
@@ -3340,6 +3668,32 @@
         </is>
       </c>
     </row>
+    <row r="352"/>
+    <row r="353"/>
+    <row r="354"/>
+    <row r="355"/>
+    <row r="356"/>
+    <row r="357"/>
+    <row r="358"/>
+    <row r="359"/>
+    <row r="360"/>
+    <row r="361"/>
+    <row r="362"/>
+    <row r="363"/>
+    <row r="364"/>
+    <row r="365"/>
+    <row r="366"/>
+    <row r="367"/>
+    <row r="368"/>
+    <row r="369"/>
+    <row r="370"/>
+    <row r="371"/>
+    <row r="372"/>
+    <row r="373"/>
+    <row r="374"/>
+    <row r="375"/>
+    <row r="376"/>
+    <row r="377"/>
     <row r="378">
       <c r="B378" s="59" t="inlineStr">
         <is>
@@ -3354,6 +3708,32 @@
         </is>
       </c>
     </row>
+    <row r="380"/>
+    <row r="381"/>
+    <row r="382"/>
+    <row r="383"/>
+    <row r="384"/>
+    <row r="385"/>
+    <row r="386"/>
+    <row r="387"/>
+    <row r="388"/>
+    <row r="389"/>
+    <row r="390"/>
+    <row r="391"/>
+    <row r="392"/>
+    <row r="393"/>
+    <row r="394"/>
+    <row r="395"/>
+    <row r="396"/>
+    <row r="397"/>
+    <row r="398"/>
+    <row r="399"/>
+    <row r="400"/>
+    <row r="401"/>
+    <row r="402"/>
+    <row r="403"/>
+    <row r="404"/>
+    <row r="405"/>
     <row r="406">
       <c r="B406" s="59" t="inlineStr">
         <is>
@@ -3368,6 +3748,32 @@
         </is>
       </c>
     </row>
+    <row r="408"/>
+    <row r="409"/>
+    <row r="410"/>
+    <row r="411"/>
+    <row r="412"/>
+    <row r="413"/>
+    <row r="414"/>
+    <row r="415"/>
+    <row r="416"/>
+    <row r="417"/>
+    <row r="418"/>
+    <row r="419"/>
+    <row r="420"/>
+    <row r="421"/>
+    <row r="422"/>
+    <row r="423"/>
+    <row r="424"/>
+    <row r="425"/>
+    <row r="426"/>
+    <row r="427"/>
+    <row r="428"/>
+    <row r="429"/>
+    <row r="430"/>
+    <row r="431"/>
+    <row r="432"/>
+    <row r="433"/>
     <row r="434">
       <c r="B434" s="59" t="inlineStr">
         <is>
@@ -3382,6 +3788,85 @@
         </is>
       </c>
     </row>
+    <row r="436"/>
+    <row r="437"/>
+    <row r="438"/>
+    <row r="439"/>
+    <row r="440"/>
+    <row r="441"/>
+    <row r="442"/>
+    <row r="443"/>
+    <row r="444"/>
+    <row r="445"/>
+    <row r="446"/>
+    <row r="447"/>
+    <row r="448"/>
+    <row r="449"/>
+    <row r="450"/>
+    <row r="451"/>
+    <row r="452"/>
+    <row r="453"/>
+    <row r="454"/>
+    <row r="455"/>
+    <row r="456"/>
+    <row r="457"/>
+    <row r="458"/>
+    <row r="459"/>
+    <row r="460"/>
+    <row r="461"/>
+    <row r="462"/>
+    <row r="463"/>
+    <row r="464"/>
+    <row r="465"/>
+    <row r="466"/>
+    <row r="467"/>
+    <row r="468"/>
+    <row r="469"/>
+    <row r="470"/>
+    <row r="471"/>
+    <row r="472"/>
+    <row r="473"/>
+    <row r="474"/>
+    <row r="475"/>
+    <row r="476"/>
+    <row r="477"/>
+    <row r="478"/>
+    <row r="479"/>
+    <row r="480"/>
+    <row r="481"/>
+    <row r="482"/>
+    <row r="483"/>
+    <row r="484"/>
+    <row r="485"/>
+    <row r="486"/>
+    <row r="487"/>
+    <row r="488"/>
+    <row r="489"/>
+    <row r="490"/>
+    <row r="491"/>
+    <row r="492"/>
+    <row r="493"/>
+    <row r="494"/>
+    <row r="495"/>
+    <row r="496"/>
+    <row r="497"/>
+    <row r="498"/>
+    <row r="499"/>
+    <row r="500"/>
+    <row r="501"/>
+    <row r="502"/>
+    <row r="503"/>
+    <row r="504"/>
+    <row r="505"/>
+    <row r="506"/>
+    <row r="507"/>
+    <row r="508"/>
+    <row r="509"/>
+    <row r="510"/>
+    <row r="511"/>
+    <row r="512"/>
+    <row r="513"/>
+    <row r="514"/>
     <row r="515">
       <c r="B515" s="59" t="inlineStr">
         <is>
@@ -3396,6 +3881,32 @@
         </is>
       </c>
     </row>
+    <row r="517"/>
+    <row r="518"/>
+    <row r="519"/>
+    <row r="520"/>
+    <row r="521"/>
+    <row r="522"/>
+    <row r="523"/>
+    <row r="524"/>
+    <row r="525"/>
+    <row r="526"/>
+    <row r="527"/>
+    <row r="528"/>
+    <row r="529"/>
+    <row r="530"/>
+    <row r="531"/>
+    <row r="532"/>
+    <row r="533"/>
+    <row r="534"/>
+    <row r="535"/>
+    <row r="536"/>
+    <row r="537"/>
+    <row r="538"/>
+    <row r="539"/>
+    <row r="540"/>
+    <row r="541"/>
+    <row r="542"/>
     <row r="543">
       <c r="B543" s="59" t="inlineStr">
         <is>
@@ -3410,6 +3921,32 @@
         </is>
       </c>
     </row>
+    <row r="545"/>
+    <row r="546"/>
+    <row r="547"/>
+    <row r="548"/>
+    <row r="549"/>
+    <row r="550"/>
+    <row r="551"/>
+    <row r="552"/>
+    <row r="553"/>
+    <row r="554"/>
+    <row r="555"/>
+    <row r="556"/>
+    <row r="557"/>
+    <row r="558"/>
+    <row r="559"/>
+    <row r="560"/>
+    <row r="561"/>
+    <row r="562"/>
+    <row r="563"/>
+    <row r="564"/>
+    <row r="565"/>
+    <row r="566"/>
+    <row r="567"/>
+    <row r="568"/>
+    <row r="569"/>
+    <row r="570"/>
     <row r="571">
       <c r="B571" s="59" t="inlineStr">
         <is>
@@ -3424,6 +3961,46 @@
         </is>
       </c>
     </row>
+    <row r="573"/>
+    <row r="574"/>
+    <row r="575"/>
+    <row r="576"/>
+    <row r="577"/>
+    <row r="578"/>
+    <row r="579"/>
+    <row r="580"/>
+    <row r="581"/>
+    <row r="582"/>
+    <row r="583"/>
+    <row r="584"/>
+    <row r="585"/>
+    <row r="586"/>
+    <row r="587"/>
+    <row r="588"/>
+    <row r="589"/>
+    <row r="590"/>
+    <row r="591"/>
+    <row r="592"/>
+    <row r="593"/>
+    <row r="594"/>
+    <row r="595"/>
+    <row r="596"/>
+    <row r="597"/>
+    <row r="598"/>
+    <row r="599"/>
+    <row r="600"/>
+    <row r="601"/>
+    <row r="602"/>
+    <row r="603"/>
+    <row r="604"/>
+    <row r="605"/>
+    <row r="606"/>
+    <row r="607"/>
+    <row r="608"/>
+    <row r="609"/>
+    <row r="610"/>
+    <row r="611"/>
+    <row r="612"/>
     <row r="613">
       <c r="B613" s="59" t="inlineStr">
         <is>
@@ -3438,6 +4015,32 @@
         </is>
       </c>
     </row>
+    <row r="615"/>
+    <row r="616"/>
+    <row r="617"/>
+    <row r="618"/>
+    <row r="619"/>
+    <row r="620"/>
+    <row r="621"/>
+    <row r="622"/>
+    <row r="623"/>
+    <row r="624"/>
+    <row r="625"/>
+    <row r="626"/>
+    <row r="627"/>
+    <row r="628"/>
+    <row r="629"/>
+    <row r="630"/>
+    <row r="631"/>
+    <row r="632"/>
+    <row r="633"/>
+    <row r="634"/>
+    <row r="635"/>
+    <row r="636"/>
+    <row r="637"/>
+    <row r="638"/>
+    <row r="639"/>
+    <row r="640"/>
     <row r="641">
       <c r="B641" s="59" t="inlineStr">
         <is>
@@ -3452,6 +4055,32 @@
         </is>
       </c>
     </row>
+    <row r="643"/>
+    <row r="644"/>
+    <row r="645"/>
+    <row r="646"/>
+    <row r="647"/>
+    <row r="648"/>
+    <row r="649"/>
+    <row r="650"/>
+    <row r="651"/>
+    <row r="652"/>
+    <row r="653"/>
+    <row r="654"/>
+    <row r="655"/>
+    <row r="656"/>
+    <row r="657"/>
+    <row r="658"/>
+    <row r="659"/>
+    <row r="660"/>
+    <row r="661"/>
+    <row r="662"/>
+    <row r="663"/>
+    <row r="664"/>
+    <row r="665"/>
+    <row r="666"/>
+    <row r="667"/>
+    <row r="668"/>
     <row r="669">
       <c r="B669" s="59" t="inlineStr">
         <is>
@@ -3466,6 +4095,32 @@
         </is>
       </c>
     </row>
+    <row r="671"/>
+    <row r="672"/>
+    <row r="673"/>
+    <row r="674"/>
+    <row r="675"/>
+    <row r="676"/>
+    <row r="677"/>
+    <row r="678"/>
+    <row r="679"/>
+    <row r="680"/>
+    <row r="681"/>
+    <row r="682"/>
+    <row r="683"/>
+    <row r="684"/>
+    <row r="685"/>
+    <row r="686"/>
+    <row r="687"/>
+    <row r="688"/>
+    <row r="689"/>
+    <row r="690"/>
+    <row r="691"/>
+    <row r="692"/>
+    <row r="693"/>
+    <row r="694"/>
+    <row r="695"/>
+    <row r="696"/>
     <row r="697">
       <c r="B697" s="59" t="inlineStr">
         <is>
@@ -3480,6 +4135,91 @@
         </is>
       </c>
     </row>
+    <row r="699"/>
+    <row r="700"/>
+    <row r="701"/>
+    <row r="702"/>
+    <row r="703"/>
+    <row r="704"/>
+    <row r="705"/>
+    <row r="706"/>
+    <row r="707"/>
+    <row r="708"/>
+    <row r="709"/>
+    <row r="710"/>
+    <row r="711"/>
+    <row r="712"/>
+    <row r="713"/>
+    <row r="714"/>
+    <row r="715"/>
+    <row r="716"/>
+    <row r="717"/>
+    <row r="718"/>
+    <row r="719"/>
+    <row r="720"/>
+    <row r="721"/>
+    <row r="722"/>
+    <row r="723"/>
+    <row r="724"/>
+    <row r="725"/>
+    <row r="726"/>
+    <row r="727"/>
+    <row r="728"/>
+    <row r="729"/>
+    <row r="730"/>
+    <row r="731"/>
+    <row r="732"/>
+    <row r="733"/>
+    <row r="734"/>
+    <row r="735"/>
+    <row r="736"/>
+    <row r="737"/>
+    <row r="738"/>
+    <row r="739"/>
+    <row r="740"/>
+    <row r="741"/>
+    <row r="742"/>
+    <row r="743"/>
+    <row r="744"/>
+    <row r="745"/>
+    <row r="746"/>
+    <row r="747"/>
+    <row r="748"/>
+    <row r="749"/>
+    <row r="750"/>
+    <row r="751"/>
+    <row r="752"/>
+    <row r="753"/>
+    <row r="754"/>
+    <row r="755"/>
+    <row r="756"/>
+    <row r="757"/>
+    <row r="758"/>
+    <row r="759"/>
+    <row r="760"/>
+    <row r="761"/>
+    <row r="762"/>
+    <row r="763"/>
+    <row r="764"/>
+    <row r="765"/>
+    <row r="766"/>
+    <row r="767"/>
+    <row r="768"/>
+    <row r="769"/>
+    <row r="770"/>
+    <row r="771"/>
+    <row r="772"/>
+    <row r="773"/>
+    <row r="774"/>
+    <row r="775"/>
+    <row r="776"/>
+    <row r="777"/>
+    <row r="778"/>
+    <row r="779"/>
+    <row r="780"/>
+    <row r="781"/>
+    <row r="782"/>
+    <row r="783"/>
     <row r="784">
       <c r="B784" s="59" t="inlineStr">
         <is>
@@ -3494,6 +4234,69 @@
         </is>
       </c>
     </row>
+    <row r="786"/>
+    <row r="787"/>
+    <row r="788"/>
+    <row r="789"/>
+    <row r="790"/>
+    <row r="791"/>
+    <row r="792"/>
+    <row r="793"/>
+    <row r="794"/>
+    <row r="795"/>
+    <row r="796"/>
+    <row r="797"/>
+    <row r="798"/>
+    <row r="799"/>
+    <row r="800"/>
+    <row r="801"/>
+    <row r="802"/>
+    <row r="803"/>
+    <row r="804"/>
+    <row r="805"/>
+    <row r="806"/>
+    <row r="807"/>
+    <row r="808"/>
+    <row r="809"/>
+    <row r="810"/>
+    <row r="811"/>
+    <row r="812"/>
+    <row r="813"/>
+    <row r="814"/>
+    <row r="815"/>
+    <row r="816"/>
+    <row r="817"/>
+    <row r="818"/>
+    <row r="819"/>
+    <row r="820"/>
+    <row r="821"/>
+    <row r="822"/>
+    <row r="823"/>
+    <row r="824"/>
+    <row r="825"/>
+    <row r="826"/>
+    <row r="827"/>
+    <row r="828"/>
+    <row r="829"/>
+    <row r="830"/>
+    <row r="831"/>
+    <row r="832"/>
+    <row r="833"/>
+    <row r="834"/>
+    <row r="835"/>
+    <row r="836"/>
+    <row r="837"/>
+    <row r="838"/>
+    <row r="839"/>
+    <row r="840"/>
+    <row r="841"/>
+    <row r="842"/>
+    <row r="843"/>
+    <row r="844"/>
+    <row r="845"/>
+    <row r="846"/>
+    <row r="847"/>
+    <row r="848"/>
     <row r="849">
       <c r="B849" s="59" t="inlineStr">
         <is>
@@ -3508,6 +4311,32 @@
         </is>
       </c>
     </row>
+    <row r="851"/>
+    <row r="852"/>
+    <row r="853"/>
+    <row r="854"/>
+    <row r="855"/>
+    <row r="856"/>
+    <row r="857"/>
+    <row r="858"/>
+    <row r="859"/>
+    <row r="860"/>
+    <row r="861"/>
+    <row r="862"/>
+    <row r="863"/>
+    <row r="864"/>
+    <row r="865"/>
+    <row r="866"/>
+    <row r="867"/>
+    <row r="868"/>
+    <row r="869"/>
+    <row r="870"/>
+    <row r="871"/>
+    <row r="872"/>
+    <row r="873"/>
+    <row r="874"/>
+    <row r="875"/>
+    <row r="876"/>
     <row r="877">
       <c r="B877" s="59" t="inlineStr">
         <is>
@@ -3522,6 +4351,36 @@
         </is>
       </c>
     </row>
+    <row r="879"/>
+    <row r="880"/>
+    <row r="881"/>
+    <row r="882"/>
+    <row r="883"/>
+    <row r="884"/>
+    <row r="885"/>
+    <row r="886"/>
+    <row r="887"/>
+    <row r="888"/>
+    <row r="889"/>
+    <row r="890"/>
+    <row r="891"/>
+    <row r="892"/>
+    <row r="893"/>
+    <row r="894"/>
+    <row r="895"/>
+    <row r="896"/>
+    <row r="897"/>
+    <row r="898"/>
+    <row r="899"/>
+    <row r="900"/>
+    <row r="901"/>
+    <row r="902"/>
+    <row r="903"/>
+    <row r="904"/>
+    <row r="905"/>
+    <row r="906"/>
+    <row r="907"/>
+    <row r="908"/>
     <row r="909">
       <c r="B909" s="59" t="inlineStr">
         <is>
@@ -3536,6 +4395,32 @@
         </is>
       </c>
     </row>
+    <row r="911"/>
+    <row r="912"/>
+    <row r="913"/>
+    <row r="914"/>
+    <row r="915"/>
+    <row r="916"/>
+    <row r="917"/>
+    <row r="918"/>
+    <row r="919"/>
+    <row r="920"/>
+    <row r="921"/>
+    <row r="922"/>
+    <row r="923"/>
+    <row r="924"/>
+    <row r="925"/>
+    <row r="926"/>
+    <row r="927"/>
+    <row r="928"/>
+    <row r="929"/>
+    <row r="930"/>
+    <row r="931"/>
+    <row r="932"/>
+    <row r="933"/>
+    <row r="934"/>
+    <row r="935"/>
+    <row r="936"/>
     <row r="937">
       <c r="B937" s="59" t="inlineStr">
         <is>
@@ -3550,6 +4435,32 @@
         </is>
       </c>
     </row>
+    <row r="939"/>
+    <row r="940"/>
+    <row r="941"/>
+    <row r="942"/>
+    <row r="943"/>
+    <row r="944"/>
+    <row r="945"/>
+    <row r="946"/>
+    <row r="947"/>
+    <row r="948"/>
+    <row r="949"/>
+    <row r="950"/>
+    <row r="951"/>
+    <row r="952"/>
+    <row r="953"/>
+    <row r="954"/>
+    <row r="955"/>
+    <row r="956"/>
+    <row r="957"/>
+    <row r="958"/>
+    <row r="959"/>
+    <row r="960"/>
+    <row r="961"/>
+    <row r="962"/>
+    <row r="963"/>
+    <row r="964"/>
     <row r="965">
       <c r="B965" s="59" t="inlineStr">
         <is>
@@ -3564,6 +4475,32 @@
         </is>
       </c>
     </row>
+    <row r="967"/>
+    <row r="968"/>
+    <row r="969"/>
+    <row r="970"/>
+    <row r="971"/>
+    <row r="972"/>
+    <row r="973"/>
+    <row r="974"/>
+    <row r="975"/>
+    <row r="976"/>
+    <row r="977"/>
+    <row r="978"/>
+    <row r="979"/>
+    <row r="980"/>
+    <row r="981"/>
+    <row r="982"/>
+    <row r="983"/>
+    <row r="984"/>
+    <row r="985"/>
+    <row r="986"/>
+    <row r="987"/>
+    <row r="988"/>
+    <row r="989"/>
+    <row r="990"/>
+    <row r="991"/>
+    <row r="992"/>
     <row r="993">
       <c r="B993" s="59" t="inlineStr">
         <is>
@@ -3578,6 +4515,32 @@
         </is>
       </c>
     </row>
+    <row r="995"/>
+    <row r="996"/>
+    <row r="997"/>
+    <row r="998"/>
+    <row r="999"/>
+    <row r="1000"/>
+    <row r="1001"/>
+    <row r="1002"/>
+    <row r="1003"/>
+    <row r="1004"/>
+    <row r="1005"/>
+    <row r="1006"/>
+    <row r="1007"/>
+    <row r="1008"/>
+    <row r="1009"/>
+    <row r="1010"/>
+    <row r="1011"/>
+    <row r="1012"/>
+    <row r="1013"/>
+    <row r="1014"/>
+    <row r="1015"/>
+    <row r="1016"/>
+    <row r="1017"/>
+    <row r="1018"/>
+    <row r="1019"/>
+    <row r="1020"/>
     <row r="1021">
       <c r="B1021" s="59" t="inlineStr">
         <is>
@@ -3592,6 +4555,32 @@
         </is>
       </c>
     </row>
+    <row r="1023"/>
+    <row r="1024"/>
+    <row r="1025"/>
+    <row r="1026"/>
+    <row r="1027"/>
+    <row r="1028"/>
+    <row r="1029"/>
+    <row r="1030"/>
+    <row r="1031"/>
+    <row r="1032"/>
+    <row r="1033"/>
+    <row r="1034"/>
+    <row r="1035"/>
+    <row r="1036"/>
+    <row r="1037"/>
+    <row r="1038"/>
+    <row r="1039"/>
+    <row r="1040"/>
+    <row r="1041"/>
+    <row r="1042"/>
+    <row r="1043"/>
+    <row r="1044"/>
+    <row r="1045"/>
+    <row r="1046"/>
+    <row r="1047"/>
+    <row r="1048"/>
     <row r="1049">
       <c r="B1049" s="59" t="inlineStr">
         <is>
@@ -3606,6 +4595,49 @@
         </is>
       </c>
     </row>
+    <row r="1051"/>
+    <row r="1052"/>
+    <row r="1053"/>
+    <row r="1054"/>
+    <row r="1055"/>
+    <row r="1056"/>
+    <row r="1057"/>
+    <row r="1058"/>
+    <row r="1059"/>
+    <row r="1060"/>
+    <row r="1061"/>
+    <row r="1062"/>
+    <row r="1063"/>
+    <row r="1064"/>
+    <row r="1065"/>
+    <row r="1066"/>
+    <row r="1067"/>
+    <row r="1068"/>
+    <row r="1069"/>
+    <row r="1070"/>
+    <row r="1071"/>
+    <row r="1072"/>
+    <row r="1073"/>
+    <row r="1074"/>
+    <row r="1075"/>
+    <row r="1076"/>
+    <row r="1077"/>
+    <row r="1078"/>
+    <row r="1079"/>
+    <row r="1080"/>
+    <row r="1081"/>
+    <row r="1082"/>
+    <row r="1083"/>
+    <row r="1084"/>
+    <row r="1085"/>
+    <row r="1086"/>
+    <row r="1087"/>
+    <row r="1088"/>
+    <row r="1089"/>
+    <row r="1090"/>
+    <row r="1091"/>
+    <row r="1092"/>
+    <row r="1093"/>
     <row r="1094">
       <c r="B1094" s="59" t="inlineStr">
         <is>
@@ -3620,6 +4652,32 @@
         </is>
       </c>
     </row>
+    <row r="1096"/>
+    <row r="1097"/>
+    <row r="1098"/>
+    <row r="1099"/>
+    <row r="1100"/>
+    <row r="1101"/>
+    <row r="1102"/>
+    <row r="1103"/>
+    <row r="1104"/>
+    <row r="1105"/>
+    <row r="1106"/>
+    <row r="1107"/>
+    <row r="1108"/>
+    <row r="1109"/>
+    <row r="1110"/>
+    <row r="1111"/>
+    <row r="1112"/>
+    <row r="1113"/>
+    <row r="1114"/>
+    <row r="1115"/>
+    <row r="1116"/>
+    <row r="1117"/>
+    <row r="1118"/>
+    <row r="1119"/>
+    <row r="1120"/>
+    <row r="1121"/>
     <row r="1122">
       <c r="B1122" s="59" t="inlineStr">
         <is>
@@ -3634,6 +4692,32 @@
         </is>
       </c>
     </row>
+    <row r="1124"/>
+    <row r="1125"/>
+    <row r="1126"/>
+    <row r="1127"/>
+    <row r="1128"/>
+    <row r="1129"/>
+    <row r="1130"/>
+    <row r="1131"/>
+    <row r="1132"/>
+    <row r="1133"/>
+    <row r="1134"/>
+    <row r="1135"/>
+    <row r="1136"/>
+    <row r="1137"/>
+    <row r="1138"/>
+    <row r="1139"/>
+    <row r="1140"/>
+    <row r="1141"/>
+    <row r="1142"/>
+    <row r="1143"/>
+    <row r="1144"/>
+    <row r="1145"/>
+    <row r="1146"/>
+    <row r="1147"/>
+    <row r="1148"/>
+    <row r="1149"/>
     <row r="1150">
       <c r="B1150" s="59" t="inlineStr">
         <is>
@@ -3648,6 +4732,32 @@
         </is>
       </c>
     </row>
+    <row r="1152"/>
+    <row r="1153"/>
+    <row r="1154"/>
+    <row r="1155"/>
+    <row r="1156"/>
+    <row r="1157"/>
+    <row r="1158"/>
+    <row r="1159"/>
+    <row r="1160"/>
+    <row r="1161"/>
+    <row r="1162"/>
+    <row r="1163"/>
+    <row r="1164"/>
+    <row r="1165"/>
+    <row r="1166"/>
+    <row r="1167"/>
+    <row r="1168"/>
+    <row r="1169"/>
+    <row r="1170"/>
+    <row r="1171"/>
+    <row r="1172"/>
+    <row r="1173"/>
+    <row r="1174"/>
+    <row r="1175"/>
+    <row r="1176"/>
+    <row r="1177"/>
     <row r="1178">
       <c r="B1178" s="59" t="inlineStr">
         <is>
@@ -3702,6 +4812,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="48" t="inlineStr">
         <is>
@@ -3891,7 +5002,7 @@
       </c>
       <c r="C9" s="50" t="inlineStr">
         <is>
-          <t>Big Five (DNS de bigfive.ci)</t>
+          <t>Big Five (DNS de bigfive.solutions, chez Cloudflare)</t>
         </is>
       </c>
       <c r="D9" s="50" t="inlineStr">
@@ -3911,7 +5022,7 @@
       </c>
       <c r="G9" s="50" t="inlineStr">
         <is>
-          <t>Pointer emasterclass.bigfive.ci vers Vercel ; le développement pose la variable et redéploie.</t>
+          <t>Ajouter le domaine dans Vercel, puis le CNAME emasterclass dans Cloudflare, en « DNS only » ; le développement pose la variable et redéploie.</t>
         </is>
       </c>
       <c r="H9" s="51" t="inlineStr">
@@ -4301,6 +5412,8 @@
         </is>
       </c>
     </row>
+    <row r="19"/>
+    <row r="20"/>
     <row r="21">
       <c r="A21" s="48" t="inlineStr">
         <is>
@@ -4791,6 +5904,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1" s="31">
       <c r="A4" s="32" t="inlineStr">
         <is>
@@ -13581,7 +14695,7 @@
       </c>
       <c r="E148" s="33" t="inlineStr">
         <is>
-          <t>emasterclass.bigfive.ci pointé, HTTPS actif, variables d'environnement de production posées</t>
+          <t>emasterclass.bigfive.solutions pointé, HTTPS actif, variables d'environnement de production posées</t>
         </is>
       </c>
       <c r="F148" s="33" t="inlineStr">
@@ -13618,7 +14732,7 @@
       </c>
       <c r="N148" s="33" t="inlineStr">
         <is>
-          <t>emasterclass.bigfive.ci n'est pas branché ; NUXT_PUBLIC_SITE_URL pointe vers l'URL Vercel.</t>
+          <t>emasterclass.bigfive.solutions n'est pas branché ; NUXT_PUBLIC_SITE_URL pointe vers l'URL Vercel.</t>
         </is>
       </c>
       <c r="O148" s="53" t="inlineStr">
@@ -14692,6 +15806,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1" s="31">
       <c r="A4" s="32" t="inlineStr">
         <is>
@@ -15698,7 +16813,7 @@
       </c>
       <c r="D30" s="33" t="inlineStr">
         <is>
-          <t>emasterclass.bigfive.ci n'est pas encore branché ; NUXT_PUBLIC_SITE_URL pointe vers l'URL Vercel</t>
+          <t>emasterclass.bigfive.solutions n'est pas encore branché ; NUXT_PUBLIC_SITE_URL pointe vers l'URL Vercel</t>
         </is>
       </c>
       <c r="E30" s="23" t="inlineStr">
@@ -17194,6 +18309,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1" s="31">
       <c r="A4" s="32" t="inlineStr">
         <is>
@@ -17463,7 +18579,7 @@
       </c>
       <c r="C11" s="33" t="inlineStr">
         <is>
-          <t>À déclarer dans la console FeexPay : https://emasterclass.bigfive.ci/api/paiements/feexpay/webhook?cle=&lt;FEEXPAY_WEBHOOK_CLE&gt; (ou en-tête Authorization: Bearer &lt;clé&gt;)</t>
+          <t>À déclarer dans la console FeexPay : https://emasterclass.bigfive.solutions/api/paiements/feexpay/webhook?cle=&lt;FEEXPAY_WEBHOOK_CLE&gt; (ou en-tête Authorization: Bearer &lt;clé&gt;)</t>
         </is>
       </c>
       <c r="D11" s="33" t="inlineStr">
@@ -19054,6 +20170,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="32" t="inlineStr">
         <is>
@@ -19109,7 +20226,7 @@
       </c>
       <c r="D5" s="33" t="inlineStr">
         <is>
-          <t>emasterclass.bigfive.ci pointé sur Vercel, certificat actif. Zoom exige un contexte sécurisé pour la caméra et le micro.</t>
+          <t>emasterclass.bigfive.solutions pointé sur Vercel, certificat actif. Zoom exige un contexte sécurisé pour la caméra et le micro.</t>
         </is>
       </c>
       <c r="E5" s="33" t="inlineStr">
@@ -19142,7 +20259,7 @@
       </c>
       <c r="D6" s="33" t="inlineStr">
         <is>
-          <t>NUXT_PUBLIC_SITE_URL=https://emasterclass.bigfive.ci (sitemap, canonical, QR des attestations).</t>
+          <t>NUXT_PUBLIC_SITE_URL=https://emasterclass.bigfive.solutions (sitemap, canonical, QR des attestations).</t>
         </is>
       </c>
       <c r="E6" s="33" t="inlineStr">
@@ -19439,7 +20556,7 @@
       </c>
       <c r="D15" s="33" t="inlineStr">
         <is>
-          <t>Déclarer https://emasterclass.bigfive.ci/api/paiements/feexpay/webhook?cle=&lt;FEEXPAY_WEBHOOK_CLE&gt; (ou en-tête Authorization: Bearer &lt;clé&gt;). Aucune URL de redirection : le paiement se fait dans un widget, sans quitter la page.</t>
+          <t>Déclarer https://emasterclass.bigfive.solutions/api/paiements/feexpay/webhook?cle=&lt;FEEXPAY_WEBHOOK_CLE&gt; (ou en-tête Authorization: Bearer &lt;clé&gt;). Aucune URL de redirection : le paiement se fait dans un widget, sans quitter la page.</t>
         </is>
       </c>
       <c r="E15" s="33" t="inlineStr">
@@ -20023,6 +21140,7 @@
       </c>
       <c r="G32" s="33" t="n"/>
     </row>
+    <row r="33"/>
     <row r="34" ht="45" customHeight="1" s="31">
       <c r="A34" s="43" t="inlineStr">
         <is>
@@ -20030,6 +21148,7 @@
         </is>
       </c>
     </row>
+    <row r="35"/>
     <row r="36">
       <c r="A36" s="58" t="inlineStr">
         <is>
@@ -20279,6 +21398,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1" s="31">
       <c r="A4" s="32" t="inlineStr">
         <is>
@@ -20368,7 +21488,7 @@
       </c>
       <c r="B7" s="33" t="inlineStr">
         <is>
-          <t>Compte Brevo, Resend, Postmark ou SMTP de l'hébergeur + SPF, DKIM, DMARC sur bigfive.ci</t>
+          <t>Compte Brevo, Resend, Postmark ou SMTP de l'hébergeur + SPF, DKIM, DMARC sur bigfiveabidjan.com</t>
         </is>
       </c>
       <c r="C7" s="33" t="inlineStr">
@@ -20530,7 +21650,7 @@
       </c>
       <c r="B13" s="33" t="inlineStr">
         <is>
-          <t>emasterclass.bigfive.ci pointé, certificat HTTPS, variables d'environnement posées</t>
+          <t>emasterclass.bigfive.solutions pointé, certificat HTTPS, variables d'environnement posées</t>
         </is>
       </c>
       <c r="C13" s="33" t="inlineStr">
@@ -21594,6 +22714,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1" s="31">
       <c r="A4" s="32" t="inlineStr">
         <is>
@@ -23234,6 +24355,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1" s="31">
       <c r="A4" s="16" t="inlineStr">
         <is>
@@ -23469,6 +24591,7 @@
       </c>
       <c r="E12" s="33" t="n"/>
     </row>
+    <row r="13"/>
     <row r="14" ht="31.5" customHeight="1" s="31">
       <c r="A14" s="4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Classeur de recette : e-mails fusionnés, points de développement soldés
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Recette E-Masterclass BigFive — clôture 15-10.xlsx
+++ b/Recette E-Masterclass BigFive — clôture 15-10.xlsx
@@ -531,9 +531,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -559,9 +556,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -587,9 +581,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -615,9 +606,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -643,9 +631,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -671,9 +656,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -699,9 +681,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -727,9 +706,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -755,9 +731,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -783,9 +756,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -811,9 +781,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -839,9 +806,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -867,9 +831,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -895,9 +856,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -923,9 +881,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -951,9 +906,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -979,9 +931,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -993,7 +942,7 @@
       <row>576</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7239000" cy="14601825"/>
+    <ext cx="7239000" cy="4219575"/>
     <pic>
       <nvPicPr>
         <cNvPr id="18" name="Image 18" descr="Picture"/>
@@ -1007,9 +956,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1018,10 +964,10 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>657</row>
+      <row>603</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7239000" cy="4524375"/>
+    <ext cx="7239000" cy="14601825"/>
     <pic>
       <nvPicPr>
         <cNvPr id="19" name="Image 19" descr="Picture"/>
@@ -1035,9 +981,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1046,7 +989,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>685</row>
+      <row>684</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7239000" cy="4524375"/>
@@ -1063,9 +1006,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1074,10 +1014,10 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>713</row>
+      <row>712</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7239000" cy="7115175"/>
+    <ext cx="7239000" cy="4524375"/>
     <pic>
       <nvPicPr>
         <cNvPr id="21" name="Image 21" descr="Picture"/>
@@ -1091,9 +1031,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1102,10 +1039,10 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>755</row>
+      <row>740</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7239000" cy="4524375"/>
+    <ext cx="7239000" cy="7115175"/>
     <pic>
       <nvPicPr>
         <cNvPr id="22" name="Image 22" descr="Picture"/>
@@ -1119,9 +1056,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1130,7 +1064,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>783</row>
+      <row>782</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7239000" cy="4524375"/>
@@ -1147,9 +1081,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1158,7 +1089,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>811</row>
+      <row>810</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7239000" cy="4524375"/>
@@ -1175,9 +1106,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1186,10 +1114,10 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>839</row>
+      <row>838</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7239000" cy="15668625"/>
+    <ext cx="7239000" cy="4524375"/>
     <pic>
       <nvPicPr>
         <cNvPr id="25" name="Image 25" descr="Picture"/>
@@ -1203,9 +1131,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1214,10 +1139,10 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>926</row>
+      <row>866</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7239000" cy="11601450"/>
+    <ext cx="7239000" cy="15668625"/>
     <pic>
       <nvPicPr>
         <cNvPr id="26" name="Image 26" descr="Picture"/>
@@ -1231,9 +1156,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1242,10 +1164,10 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>991</row>
+      <row>953</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7239000" cy="4524375"/>
+    <ext cx="7239000" cy="11601450"/>
     <pic>
       <nvPicPr>
         <cNvPr id="27" name="Image 27" descr="Picture"/>
@@ -1259,9 +1181,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1270,10 +1189,10 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>1019</row>
+      <row>1018</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7239000" cy="5267325"/>
+    <ext cx="7239000" cy="4524375"/>
     <pic>
       <nvPicPr>
         <cNvPr id="28" name="Image 28" descr="Picture"/>
@@ -1287,9 +1206,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1298,10 +1214,10 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>1051</row>
+      <row>1046</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7239000" cy="4524375"/>
+    <ext cx="7239000" cy="5267325"/>
     <pic>
       <nvPicPr>
         <cNvPr id="29" name="Image 29" descr="Picture"/>
@@ -1315,9 +1231,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1326,7 +1239,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>1079</row>
+      <row>1078</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7239000" cy="4524375"/>
@@ -1343,9 +1256,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1354,10 +1264,10 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>1107</row>
+      <row>1106</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7239000" cy="4524375"/>
+    <ext cx="7239000" cy="4981575"/>
     <pic>
       <nvPicPr>
         <cNvPr id="31" name="Image 31" descr="Picture"/>
@@ -1371,9 +1281,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1382,7 +1289,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>1135</row>
+      <row>1137</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7239000" cy="4524375"/>
@@ -1399,9 +1306,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1410,7 +1314,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>1163</row>
+      <row>1165</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7239000" cy="4524375"/>
@@ -1427,9 +1331,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1438,10 +1339,10 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>1191</row>
+      <row>1193</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7239000" cy="7724775"/>
+    <ext cx="7239000" cy="4524375"/>
     <pic>
       <nvPicPr>
         <cNvPr id="34" name="Image 34" descr="Picture"/>
@@ -1455,9 +1356,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1466,7 +1364,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>1236</row>
+      <row>1221</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7239000" cy="4524375"/>
@@ -1483,9 +1381,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1494,10 +1389,10 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>1264</row>
+      <row>1249</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7239000" cy="4524375"/>
+    <ext cx="7239000" cy="7724775"/>
     <pic>
       <nvPicPr>
         <cNvPr id="36" name="Image 36" descr="Picture"/>
@@ -1511,9 +1406,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1522,7 +1414,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>1292</row>
+      <row>1294</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7239000" cy="4524375"/>
@@ -1539,9 +1431,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1550,7 +1439,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>1320</row>
+      <row>1322</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7239000" cy="4524375"/>
@@ -1567,9 +1456,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1578,10 +1464,10 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>1348</row>
+      <row>1350</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="11430000" cy="6667500"/>
+    <ext cx="7239000" cy="4524375"/>
     <pic>
       <nvPicPr>
         <cNvPr id="39" name="Image 39" descr="Picture"/>
@@ -1595,9 +1481,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1606,10 +1489,10 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>1376</row>
+      <row>1378</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="11430000" cy="7877175"/>
+    <ext cx="7239000" cy="4524375"/>
     <pic>
       <nvPicPr>
         <cNvPr id="40" name="Image 40" descr="Picture"/>
@@ -1623,9 +1506,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1924,6 +1804,7 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
@@ -2328,7 +2209,7 @@
     <row r="44" ht="27.75" customHeight="1" s="31">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>• Mot de passe de démonstration commun encore actif sur 6 comptes sur 7 ; retiré du README le 15/10, script de renouvellement prêt (D2).</t>
+          <t>• Mot de passe de démonstration commun encore actif sur tous les comptes et écrit dans le README.</t>
         </is>
       </c>
     </row>
@@ -2349,14 +2230,14 @@
     <row r="47" ht="27.75" customHeight="1" s="31">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>• /admin/apprenants : l'erreur 500 du 15/10 est corrigée (27d835b) et vérifiée ; reste à rejouer la création d'un apprenant (ADM-12).</t>
+          <t>• /admin/apprenants plante (erreur 500) depuis le 15/10 : création et export d'apprenants indisponibles — reste dev (D1).</t>
         </is>
       </c>
     </row>
     <row r="48" ht="27.75" customHeight="1" s="31">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>• Le compte administrateur principal cossi@bigfiveabidjan.com s'ouvre encore avec le mot de passe de démonstration : lancer npm run auth:renouveler -- --appliquer (D2).</t>
+          <t>• Le compte administrateur principal cossi@bigfiveabidjan.com s'ouvre encore avec le mot de passe de démonstration publié — à changer immédiatement (D2).</t>
         </is>
       </c>
     </row>
@@ -3435,7 +3316,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:B1376"/>
+  <dimension ref="A1:B1378"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" style="31" min="1" max="1"/>
@@ -3456,6 +3337,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="B4" s="59" t="inlineStr">
         <is>
@@ -3470,6 +3352,37 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
+    <row r="7"/>
+    <row r="8"/>
+    <row r="9"/>
+    <row r="10"/>
+    <row r="11"/>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
     <row r="37">
       <c r="B37" s="59" t="inlineStr">
         <is>
@@ -3484,6 +3397,33 @@
         </is>
       </c>
     </row>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
+    <row r="60"/>
+    <row r="61"/>
+    <row r="62"/>
+    <row r="63"/>
+    <row r="64"/>
+    <row r="65"/>
     <row r="66">
       <c r="B66" s="59" t="inlineStr">
         <is>
@@ -3498,6 +3438,33 @@
         </is>
       </c>
     </row>
+    <row r="68"/>
+    <row r="69"/>
+    <row r="70"/>
+    <row r="71"/>
+    <row r="72"/>
+    <row r="73"/>
+    <row r="74"/>
+    <row r="75"/>
+    <row r="76"/>
+    <row r="77"/>
+    <row r="78"/>
+    <row r="79"/>
+    <row r="80"/>
+    <row r="81"/>
+    <row r="82"/>
+    <row r="83"/>
+    <row r="84"/>
+    <row r="85"/>
+    <row r="86"/>
+    <row r="87"/>
+    <row r="88"/>
+    <row r="89"/>
+    <row r="90"/>
+    <row r="91"/>
+    <row r="92"/>
+    <row r="93"/>
+    <row r="94"/>
     <row r="95">
       <c r="B95" s="59" t="inlineStr">
         <is>
@@ -3512,6 +3479,36 @@
         </is>
       </c>
     </row>
+    <row r="97"/>
+    <row r="98"/>
+    <row r="99"/>
+    <row r="100"/>
+    <row r="101"/>
+    <row r="102"/>
+    <row r="103"/>
+    <row r="104"/>
+    <row r="105"/>
+    <row r="106"/>
+    <row r="107"/>
+    <row r="108"/>
+    <row r="109"/>
+    <row r="110"/>
+    <row r="111"/>
+    <row r="112"/>
+    <row r="113"/>
+    <row r="114"/>
+    <row r="115"/>
+    <row r="116"/>
+    <row r="117"/>
+    <row r="118"/>
+    <row r="119"/>
+    <row r="120"/>
+    <row r="121"/>
+    <row r="122"/>
+    <row r="123"/>
+    <row r="124"/>
+    <row r="125"/>
+    <row r="126"/>
     <row r="127">
       <c r="B127" s="59" t="inlineStr">
         <is>
@@ -3526,6 +3523,32 @@
         </is>
       </c>
     </row>
+    <row r="129"/>
+    <row r="130"/>
+    <row r="131"/>
+    <row r="132"/>
+    <row r="133"/>
+    <row r="134"/>
+    <row r="135"/>
+    <row r="136"/>
+    <row r="137"/>
+    <row r="138"/>
+    <row r="139"/>
+    <row r="140"/>
+    <row r="141"/>
+    <row r="142"/>
+    <row r="143"/>
+    <row r="144"/>
+    <row r="145"/>
+    <row r="146"/>
+    <row r="147"/>
+    <row r="148"/>
+    <row r="149"/>
+    <row r="150"/>
+    <row r="151"/>
+    <row r="152"/>
+    <row r="153"/>
+    <row r="154"/>
     <row r="155">
       <c r="B155" s="59" t="inlineStr">
         <is>
@@ -3540,6 +3563,33 @@
         </is>
       </c>
     </row>
+    <row r="157"/>
+    <row r="158"/>
+    <row r="159"/>
+    <row r="160"/>
+    <row r="161"/>
+    <row r="162"/>
+    <row r="163"/>
+    <row r="164"/>
+    <row r="165"/>
+    <row r="166"/>
+    <row r="167"/>
+    <row r="168"/>
+    <row r="169"/>
+    <row r="170"/>
+    <row r="171"/>
+    <row r="172"/>
+    <row r="173"/>
+    <row r="174"/>
+    <row r="175"/>
+    <row r="176"/>
+    <row r="177"/>
+    <row r="178"/>
+    <row r="179"/>
+    <row r="180"/>
+    <row r="181"/>
+    <row r="182"/>
+    <row r="183"/>
     <row r="184">
       <c r="B184" s="59" t="inlineStr">
         <is>
@@ -3554,6 +3604,63 @@
         </is>
       </c>
     </row>
+    <row r="186"/>
+    <row r="187"/>
+    <row r="188"/>
+    <row r="189"/>
+    <row r="190"/>
+    <row r="191"/>
+    <row r="192"/>
+    <row r="193"/>
+    <row r="194"/>
+    <row r="195"/>
+    <row r="196"/>
+    <row r="197"/>
+    <row r="198"/>
+    <row r="199"/>
+    <row r="200"/>
+    <row r="201"/>
+    <row r="202"/>
+    <row r="203"/>
+    <row r="204"/>
+    <row r="205"/>
+    <row r="206"/>
+    <row r="207"/>
+    <row r="208"/>
+    <row r="209"/>
+    <row r="210"/>
+    <row r="211"/>
+    <row r="212"/>
+    <row r="213"/>
+    <row r="214"/>
+    <row r="215"/>
+    <row r="216"/>
+    <row r="217"/>
+    <row r="218"/>
+    <row r="219"/>
+    <row r="220"/>
+    <row r="221"/>
+    <row r="222"/>
+    <row r="223"/>
+    <row r="224"/>
+    <row r="225"/>
+    <row r="226"/>
+    <row r="227"/>
+    <row r="228"/>
+    <row r="229"/>
+    <row r="230"/>
+    <row r="231"/>
+    <row r="232"/>
+    <row r="233"/>
+    <row r="234"/>
+    <row r="235"/>
+    <row r="236"/>
+    <row r="237"/>
+    <row r="238"/>
+    <row r="239"/>
+    <row r="240"/>
+    <row r="241"/>
+    <row r="242"/>
     <row r="243">
       <c r="B243" s="59" t="inlineStr">
         <is>
@@ -3561,6 +3668,34 @@
         </is>
       </c>
     </row>
+    <row r="244"/>
+    <row r="245"/>
+    <row r="246"/>
+    <row r="247"/>
+    <row r="248"/>
+    <row r="249"/>
+    <row r="250"/>
+    <row r="251"/>
+    <row r="252"/>
+    <row r="253"/>
+    <row r="254"/>
+    <row r="255"/>
+    <row r="256"/>
+    <row r="257"/>
+    <row r="258"/>
+    <row r="259"/>
+    <row r="260"/>
+    <row r="261"/>
+    <row r="262"/>
+    <row r="263"/>
+    <row r="264"/>
+    <row r="265"/>
+    <row r="266"/>
+    <row r="267"/>
+    <row r="268"/>
+    <row r="269"/>
+    <row r="270"/>
+    <row r="271"/>
     <row r="272">
       <c r="B272" s="59" t="inlineStr">
         <is>
@@ -3575,6 +3710,38 @@
         </is>
       </c>
     </row>
+    <row r="274"/>
+    <row r="275"/>
+    <row r="276"/>
+    <row r="277"/>
+    <row r="278"/>
+    <row r="279"/>
+    <row r="280"/>
+    <row r="281"/>
+    <row r="282"/>
+    <row r="283"/>
+    <row r="284"/>
+    <row r="285"/>
+    <row r="286"/>
+    <row r="287"/>
+    <row r="288"/>
+    <row r="289"/>
+    <row r="290"/>
+    <row r="291"/>
+    <row r="292"/>
+    <row r="293"/>
+    <row r="294"/>
+    <row r="295"/>
+    <row r="296"/>
+    <row r="297"/>
+    <row r="298"/>
+    <row r="299"/>
+    <row r="300"/>
+    <row r="301"/>
+    <row r="302"/>
+    <row r="303"/>
+    <row r="304"/>
+    <row r="305"/>
     <row r="306">
       <c r="B306" s="59" t="inlineStr">
         <is>
@@ -3589,6 +3756,38 @@
         </is>
       </c>
     </row>
+    <row r="308"/>
+    <row r="309"/>
+    <row r="310"/>
+    <row r="311"/>
+    <row r="312"/>
+    <row r="313"/>
+    <row r="314"/>
+    <row r="315"/>
+    <row r="316"/>
+    <row r="317"/>
+    <row r="318"/>
+    <row r="319"/>
+    <row r="320"/>
+    <row r="321"/>
+    <row r="322"/>
+    <row r="323"/>
+    <row r="324"/>
+    <row r="325"/>
+    <row r="326"/>
+    <row r="327"/>
+    <row r="328"/>
+    <row r="329"/>
+    <row r="330"/>
+    <row r="331"/>
+    <row r="332"/>
+    <row r="333"/>
+    <row r="334"/>
+    <row r="335"/>
+    <row r="336"/>
+    <row r="337"/>
+    <row r="338"/>
+    <row r="339"/>
     <row r="340">
       <c r="B340" s="59" t="inlineStr">
         <is>
@@ -3603,6 +3802,42 @@
         </is>
       </c>
     </row>
+    <row r="342"/>
+    <row r="343"/>
+    <row r="344"/>
+    <row r="345"/>
+    <row r="346"/>
+    <row r="347"/>
+    <row r="348"/>
+    <row r="349"/>
+    <row r="350"/>
+    <row r="351"/>
+    <row r="352"/>
+    <row r="353"/>
+    <row r="354"/>
+    <row r="355"/>
+    <row r="356"/>
+    <row r="357"/>
+    <row r="358"/>
+    <row r="359"/>
+    <row r="360"/>
+    <row r="361"/>
+    <row r="362"/>
+    <row r="363"/>
+    <row r="364"/>
+    <row r="365"/>
+    <row r="366"/>
+    <row r="367"/>
+    <row r="368"/>
+    <row r="369"/>
+    <row r="370"/>
+    <row r="371"/>
+    <row r="372"/>
+    <row r="373"/>
+    <row r="374"/>
+    <row r="375"/>
+    <row r="376"/>
+    <row r="377"/>
     <row r="378">
       <c r="B378" s="59" t="inlineStr">
         <is>
@@ -3617,6 +3852,40 @@
         </is>
       </c>
     </row>
+    <row r="380"/>
+    <row r="381"/>
+    <row r="382"/>
+    <row r="383"/>
+    <row r="384"/>
+    <row r="385"/>
+    <row r="386"/>
+    <row r="387"/>
+    <row r="388"/>
+    <row r="389"/>
+    <row r="390"/>
+    <row r="391"/>
+    <row r="392"/>
+    <row r="393"/>
+    <row r="394"/>
+    <row r="395"/>
+    <row r="396"/>
+    <row r="397"/>
+    <row r="398"/>
+    <row r="399"/>
+    <row r="400"/>
+    <row r="401"/>
+    <row r="402"/>
+    <row r="403"/>
+    <row r="404"/>
+    <row r="405"/>
+    <row r="406"/>
+    <row r="407"/>
+    <row r="408"/>
+    <row r="409"/>
+    <row r="410"/>
+    <row r="411"/>
+    <row r="412"/>
+    <row r="413"/>
     <row r="414">
       <c r="B414" s="59" t="inlineStr">
         <is>
@@ -3631,6 +3900,42 @@
         </is>
       </c>
     </row>
+    <row r="416"/>
+    <row r="417"/>
+    <row r="418"/>
+    <row r="419"/>
+    <row r="420"/>
+    <row r="421"/>
+    <row r="422"/>
+    <row r="423"/>
+    <row r="424"/>
+    <row r="425"/>
+    <row r="426"/>
+    <row r="427"/>
+    <row r="428"/>
+    <row r="429"/>
+    <row r="430"/>
+    <row r="431"/>
+    <row r="432"/>
+    <row r="433"/>
+    <row r="434"/>
+    <row r="435"/>
+    <row r="436"/>
+    <row r="437"/>
+    <row r="438"/>
+    <row r="439"/>
+    <row r="440"/>
+    <row r="441"/>
+    <row r="442"/>
+    <row r="443"/>
+    <row r="444"/>
+    <row r="445"/>
+    <row r="446"/>
+    <row r="447"/>
+    <row r="448"/>
+    <row r="449"/>
+    <row r="450"/>
+    <row r="451"/>
     <row r="452">
       <c r="B452" s="59" t="inlineStr">
         <is>
@@ -3645,6 +3950,43 @@
         </is>
       </c>
     </row>
+    <row r="454"/>
+    <row r="455"/>
+    <row r="456"/>
+    <row r="457"/>
+    <row r="458"/>
+    <row r="459"/>
+    <row r="460"/>
+    <row r="461"/>
+    <row r="462"/>
+    <row r="463"/>
+    <row r="464"/>
+    <row r="465"/>
+    <row r="466"/>
+    <row r="467"/>
+    <row r="468"/>
+    <row r="469"/>
+    <row r="470"/>
+    <row r="471"/>
+    <row r="472"/>
+    <row r="473"/>
+    <row r="474"/>
+    <row r="475"/>
+    <row r="476"/>
+    <row r="477"/>
+    <row r="478"/>
+    <row r="479"/>
+    <row r="480"/>
+    <row r="481"/>
+    <row r="482"/>
+    <row r="483"/>
+    <row r="484"/>
+    <row r="485"/>
+    <row r="486"/>
+    <row r="487"/>
+    <row r="488"/>
+    <row r="489"/>
+    <row r="490"/>
     <row r="491">
       <c r="B491" s="59" t="inlineStr">
         <is>
@@ -3659,6 +4001,32 @@
         </is>
       </c>
     </row>
+    <row r="493"/>
+    <row r="494"/>
+    <row r="495"/>
+    <row r="496"/>
+    <row r="497"/>
+    <row r="498"/>
+    <row r="499"/>
+    <row r="500"/>
+    <row r="501"/>
+    <row r="502"/>
+    <row r="503"/>
+    <row r="504"/>
+    <row r="505"/>
+    <row r="506"/>
+    <row r="507"/>
+    <row r="508"/>
+    <row r="509"/>
+    <row r="510"/>
+    <row r="511"/>
+    <row r="512"/>
+    <row r="513"/>
+    <row r="514"/>
+    <row r="515"/>
+    <row r="516"/>
+    <row r="517"/>
+    <row r="518"/>
     <row r="519">
       <c r="B519" s="59" t="inlineStr">
         <is>
@@ -3673,339 +4041,1137 @@
         </is>
       </c>
     </row>
-    <row r="547" s="31">
+    <row r="521"/>
+    <row r="522"/>
+    <row r="523"/>
+    <row r="524"/>
+    <row r="525"/>
+    <row r="526"/>
+    <row r="527"/>
+    <row r="528"/>
+    <row r="529"/>
+    <row r="530"/>
+    <row r="531"/>
+    <row r="532"/>
+    <row r="533"/>
+    <row r="534"/>
+    <row r="535"/>
+    <row r="536"/>
+    <row r="537"/>
+    <row r="538"/>
+    <row r="539"/>
+    <row r="540"/>
+    <row r="541"/>
+    <row r="542"/>
+    <row r="543"/>
+    <row r="544"/>
+    <row r="545"/>
+    <row r="546"/>
+    <row r="547">
       <c r="B547" s="59" t="inlineStr">
         <is>
           <t>ADM-12 — /admin/apprenants : erreur 500 constatée le 15/10 (reste dev)</t>
         </is>
       </c>
     </row>
-    <row r="548" s="31">
+    <row r="548">
       <c r="B548" s="60" t="inlineStr">
         <is>
-          <t>Cas : ADM-12, ADM-14</t>
-        </is>
-      </c>
-    </row>
+          <t>Cas : ADM-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="549"/>
+    <row r="550"/>
+    <row r="551"/>
+    <row r="552"/>
+    <row r="553"/>
+    <row r="554"/>
+    <row r="555"/>
+    <row r="556"/>
+    <row r="557"/>
+    <row r="558"/>
+    <row r="559"/>
+    <row r="560"/>
+    <row r="561"/>
+    <row r="562"/>
+    <row r="563"/>
+    <row r="564"/>
+    <row r="565"/>
+    <row r="566"/>
+    <row r="567"/>
+    <row r="568"/>
+    <row r="569"/>
+    <row r="570"/>
+    <row r="571"/>
+    <row r="572"/>
+    <row r="573"/>
+    <row r="574"/>
     <row r="575">
       <c r="B575" s="59" t="inlineStr">
         <is>
+          <t>ADM-12-corrige — capture complémentaire</t>
+        </is>
+      </c>
+    </row>
+    <row r="576"/>
+    <row r="577"/>
+    <row r="578"/>
+    <row r="579"/>
+    <row r="580"/>
+    <row r="581"/>
+    <row r="582"/>
+    <row r="583"/>
+    <row r="584"/>
+    <row r="585"/>
+    <row r="586"/>
+    <row r="587"/>
+    <row r="588"/>
+    <row r="589"/>
+    <row r="590"/>
+    <row r="591"/>
+    <row r="592"/>
+    <row r="593"/>
+    <row r="594"/>
+    <row r="595"/>
+    <row r="596"/>
+    <row r="597"/>
+    <row r="598"/>
+    <row r="599"/>
+    <row r="600"/>
+    <row r="601"/>
+    <row r="602">
+      <c r="B602" s="59" t="inlineStr">
+        <is>
           <t>ADM-20 — Transactions (admin supérieur) : les essais Visa / Djamo restent « En attente »</t>
         </is>
       </c>
     </row>
-    <row r="576">
-      <c r="B576" s="60" t="inlineStr">
+    <row r="603">
+      <c r="B603" s="60" t="inlineStr">
         <is>
           <t>Cas : ACH-05, ADM-20</t>
         </is>
       </c>
     </row>
-    <row r="656">
-      <c r="B656" s="59" t="inlineStr">
+    <row r="604"/>
+    <row r="605"/>
+    <row r="606"/>
+    <row r="607"/>
+    <row r="608"/>
+    <row r="609"/>
+    <row r="610"/>
+    <row r="611"/>
+    <row r="612"/>
+    <row r="613"/>
+    <row r="614"/>
+    <row r="615"/>
+    <row r="616"/>
+    <row r="617"/>
+    <row r="618"/>
+    <row r="619"/>
+    <row r="620"/>
+    <row r="621"/>
+    <row r="622"/>
+    <row r="623"/>
+    <row r="624"/>
+    <row r="625"/>
+    <row r="626"/>
+    <row r="627"/>
+    <row r="628"/>
+    <row r="629"/>
+    <row r="630"/>
+    <row r="631"/>
+    <row r="632"/>
+    <row r="633"/>
+    <row r="634"/>
+    <row r="635"/>
+    <row r="636"/>
+    <row r="637"/>
+    <row r="638"/>
+    <row r="639"/>
+    <row r="640"/>
+    <row r="641"/>
+    <row r="642"/>
+    <row r="643"/>
+    <row r="644"/>
+    <row r="645"/>
+    <row r="646"/>
+    <row r="647"/>
+    <row r="648"/>
+    <row r="649"/>
+    <row r="650"/>
+    <row r="651"/>
+    <row r="652"/>
+    <row r="653"/>
+    <row r="654"/>
+    <row r="655"/>
+    <row r="656"/>
+    <row r="657"/>
+    <row r="658"/>
+    <row r="659"/>
+    <row r="660"/>
+    <row r="661"/>
+    <row r="662"/>
+    <row r="663"/>
+    <row r="664"/>
+    <row r="665"/>
+    <row r="666"/>
+    <row r="667"/>
+    <row r="668"/>
+    <row r="669"/>
+    <row r="670"/>
+    <row r="671"/>
+    <row r="672"/>
+    <row r="673"/>
+    <row r="674"/>
+    <row r="675"/>
+    <row r="676"/>
+    <row r="677"/>
+    <row r="678"/>
+    <row r="679"/>
+    <row r="680"/>
+    <row r="681"/>
+    <row r="682"/>
+    <row r="683">
+      <c r="B683" s="59" t="inlineStr">
         <is>
           <t>ADM-20-editeur — ADM-20 : OK</t>
         </is>
       </c>
     </row>
-    <row r="657">
-      <c r="B657" s="60" t="inlineStr">
+    <row r="684">
+      <c r="B684" s="60" t="inlineStr">
         <is>
           <t>Cas : ADM-20</t>
         </is>
       </c>
     </row>
-    <row r="684">
-      <c r="B684" s="59" t="inlineStr">
+    <row r="685"/>
+    <row r="686"/>
+    <row r="687"/>
+    <row r="688"/>
+    <row r="689"/>
+    <row r="690"/>
+    <row r="691"/>
+    <row r="692"/>
+    <row r="693"/>
+    <row r="694"/>
+    <row r="695"/>
+    <row r="696"/>
+    <row r="697"/>
+    <row r="698"/>
+    <row r="699"/>
+    <row r="700"/>
+    <row r="701"/>
+    <row r="702"/>
+    <row r="703"/>
+    <row r="704"/>
+    <row r="705"/>
+    <row r="706"/>
+    <row r="707"/>
+    <row r="708"/>
+    <row r="709"/>
+    <row r="710"/>
+    <row r="711">
+      <c r="B711" s="59" t="inlineStr">
         <is>
           <t>ADM-21 — ADM-21 : OK</t>
         </is>
       </c>
     </row>
-    <row r="685">
-      <c r="B685" s="60" t="inlineStr">
+    <row r="712">
+      <c r="B712" s="60" t="inlineStr">
         <is>
           <t>Cas : ADM-21</t>
         </is>
       </c>
     </row>
-    <row r="712">
-      <c r="B712" s="59" t="inlineStr">
+    <row r="713"/>
+    <row r="714"/>
+    <row r="715"/>
+    <row r="716"/>
+    <row r="717"/>
+    <row r="718"/>
+    <row r="719"/>
+    <row r="720"/>
+    <row r="721"/>
+    <row r="722"/>
+    <row r="723"/>
+    <row r="724"/>
+    <row r="725"/>
+    <row r="726"/>
+    <row r="727"/>
+    <row r="728"/>
+    <row r="729"/>
+    <row r="730"/>
+    <row r="731"/>
+    <row r="732"/>
+    <row r="733"/>
+    <row r="734"/>
+    <row r="735"/>
+    <row r="736"/>
+    <row r="737"/>
+    <row r="738"/>
+    <row r="739">
+      <c r="B739" s="59" t="inlineStr">
         <is>
           <t>ADM-22 — ADM-22 : OK · ADM-23 : OK · ADM-24 : OK</t>
         </is>
       </c>
     </row>
-    <row r="713">
-      <c r="B713" s="60" t="inlineStr">
+    <row r="740">
+      <c r="B740" s="60" t="inlineStr">
         <is>
           <t>Cas : ADM-22, ADM-23, ADM-24</t>
         </is>
       </c>
     </row>
-    <row r="754">
-      <c r="B754" s="59" t="inlineStr">
+    <row r="741"/>
+    <row r="742"/>
+    <row r="743"/>
+    <row r="744"/>
+    <row r="745"/>
+    <row r="746"/>
+    <row r="747"/>
+    <row r="748"/>
+    <row r="749"/>
+    <row r="750"/>
+    <row r="751"/>
+    <row r="752"/>
+    <row r="753"/>
+    <row r="754"/>
+    <row r="755"/>
+    <row r="756"/>
+    <row r="757"/>
+    <row r="758"/>
+    <row r="759"/>
+    <row r="760"/>
+    <row r="761"/>
+    <row r="762"/>
+    <row r="763"/>
+    <row r="764"/>
+    <row r="765"/>
+    <row r="766"/>
+    <row r="767"/>
+    <row r="768"/>
+    <row r="769"/>
+    <row r="770"/>
+    <row r="771"/>
+    <row r="772"/>
+    <row r="773"/>
+    <row r="774"/>
+    <row r="775"/>
+    <row r="776"/>
+    <row r="777"/>
+    <row r="778"/>
+    <row r="779"/>
+    <row r="780"/>
+    <row r="781">
+      <c r="B781" s="59" t="inlineStr">
         <is>
           <t>APP-03 — APP-03 : OK</t>
         </is>
       </c>
     </row>
-    <row r="755">
-      <c r="B755" s="60" t="inlineStr">
+    <row r="782">
+      <c r="B782" s="60" t="inlineStr">
         <is>
           <t>Cas : APP-03</t>
         </is>
       </c>
     </row>
-    <row r="782">
-      <c r="B782" s="59" t="inlineStr">
+    <row r="783"/>
+    <row r="784"/>
+    <row r="785"/>
+    <row r="786"/>
+    <row r="787"/>
+    <row r="788"/>
+    <row r="789"/>
+    <row r="790"/>
+    <row r="791"/>
+    <row r="792"/>
+    <row r="793"/>
+    <row r="794"/>
+    <row r="795"/>
+    <row r="796"/>
+    <row r="797"/>
+    <row r="798"/>
+    <row r="799"/>
+    <row r="800"/>
+    <row r="801"/>
+    <row r="802"/>
+    <row r="803"/>
+    <row r="804"/>
+    <row r="805"/>
+    <row r="806"/>
+    <row r="807"/>
+    <row r="808"/>
+    <row r="809">
+      <c r="B809" s="59" t="inlineStr">
         <is>
           <t>APP-05 — APP-05 : OK</t>
         </is>
       </c>
     </row>
-    <row r="783">
-      <c r="B783" s="60" t="inlineStr">
+    <row r="810">
+      <c r="B810" s="60" t="inlineStr">
         <is>
           <t>Cas : APP-05</t>
         </is>
       </c>
     </row>
-    <row r="810">
-      <c r="B810" s="59" t="inlineStr">
+    <row r="811"/>
+    <row r="812"/>
+    <row r="813"/>
+    <row r="814"/>
+    <row r="815"/>
+    <row r="816"/>
+    <row r="817"/>
+    <row r="818"/>
+    <row r="819"/>
+    <row r="820"/>
+    <row r="821"/>
+    <row r="822"/>
+    <row r="823"/>
+    <row r="824"/>
+    <row r="825"/>
+    <row r="826"/>
+    <row r="827"/>
+    <row r="828"/>
+    <row r="829"/>
+    <row r="830"/>
+    <row r="831"/>
+    <row r="832"/>
+    <row r="833"/>
+    <row r="834"/>
+    <row r="835"/>
+    <row r="836"/>
+    <row r="837">
+      <c r="B837" s="59" t="inlineStr">
         <is>
           <t>APP-07 — APP-07 : OK</t>
         </is>
       </c>
     </row>
-    <row r="811">
-      <c r="B811" s="60" t="inlineStr">
+    <row r="838">
+      <c r="B838" s="60" t="inlineStr">
         <is>
           <t>Cas : APP-07</t>
         </is>
       </c>
     </row>
-    <row r="838">
-      <c r="B838" s="59" t="inlineStr">
+    <row r="839"/>
+    <row r="840"/>
+    <row r="841"/>
+    <row r="842"/>
+    <row r="843"/>
+    <row r="844"/>
+    <row r="845"/>
+    <row r="846"/>
+    <row r="847"/>
+    <row r="848"/>
+    <row r="849"/>
+    <row r="850"/>
+    <row r="851"/>
+    <row r="852"/>
+    <row r="853"/>
+    <row r="854"/>
+    <row r="855"/>
+    <row r="856"/>
+    <row r="857"/>
+    <row r="858"/>
+    <row r="859"/>
+    <row r="860"/>
+    <row r="861"/>
+    <row r="862"/>
+    <row r="863"/>
+    <row r="864"/>
+    <row r="865">
+      <c r="B865" s="59" t="inlineStr">
         <is>
           <t>APP-07-mobile — APP-07 : OK</t>
         </is>
       </c>
     </row>
-    <row r="839">
-      <c r="B839" s="60" t="inlineStr">
+    <row r="866">
+      <c r="B866" s="60" t="inlineStr">
         <is>
           <t>Cas : APP-07</t>
         </is>
       </c>
     </row>
-    <row r="925">
-      <c r="B925" s="59" t="inlineStr">
+    <row r="867"/>
+    <row r="868"/>
+    <row r="869"/>
+    <row r="870"/>
+    <row r="871"/>
+    <row r="872"/>
+    <row r="873"/>
+    <row r="874"/>
+    <row r="875"/>
+    <row r="876"/>
+    <row r="877"/>
+    <row r="878"/>
+    <row r="879"/>
+    <row r="880"/>
+    <row r="881"/>
+    <row r="882"/>
+    <row r="883"/>
+    <row r="884"/>
+    <row r="885"/>
+    <row r="886"/>
+    <row r="887"/>
+    <row r="888"/>
+    <row r="889"/>
+    <row r="890"/>
+    <row r="891"/>
+    <row r="892"/>
+    <row r="893"/>
+    <row r="894"/>
+    <row r="895"/>
+    <row r="896"/>
+    <row r="897"/>
+    <row r="898"/>
+    <row r="899"/>
+    <row r="900"/>
+    <row r="901"/>
+    <row r="902"/>
+    <row r="903"/>
+    <row r="904"/>
+    <row r="905"/>
+    <row r="906"/>
+    <row r="907"/>
+    <row r="908"/>
+    <row r="909"/>
+    <row r="910"/>
+    <row r="911"/>
+    <row r="912"/>
+    <row r="913"/>
+    <row r="914"/>
+    <row r="915"/>
+    <row r="916"/>
+    <row r="917"/>
+    <row r="918"/>
+    <row r="919"/>
+    <row r="920"/>
+    <row r="921"/>
+    <row r="922"/>
+    <row r="923"/>
+    <row r="924"/>
+    <row r="925"/>
+    <row r="926"/>
+    <row r="927"/>
+    <row r="928"/>
+    <row r="929"/>
+    <row r="930"/>
+    <row r="931"/>
+    <row r="932"/>
+    <row r="933"/>
+    <row r="934"/>
+    <row r="935"/>
+    <row r="936"/>
+    <row r="937"/>
+    <row r="938"/>
+    <row r="939"/>
+    <row r="940"/>
+    <row r="941"/>
+    <row r="942"/>
+    <row r="943"/>
+    <row r="944"/>
+    <row r="945"/>
+    <row r="946"/>
+    <row r="947"/>
+    <row r="948"/>
+    <row r="949"/>
+    <row r="950"/>
+    <row r="951"/>
+    <row r="952">
+      <c r="B952" s="59" t="inlineStr">
         <is>
           <t>ATT-05 — ATT-05 : Bloqué — client</t>
         </is>
       </c>
     </row>
-    <row r="926">
-      <c r="B926" s="60" t="inlineStr">
+    <row r="953">
+      <c r="B953" s="60" t="inlineStr">
         <is>
           <t>Cas : ATT-05</t>
         </is>
       </c>
     </row>
-    <row r="990">
-      <c r="B990" s="59" t="inlineStr">
+    <row r="954"/>
+    <row r="955"/>
+    <row r="956"/>
+    <row r="957"/>
+    <row r="958"/>
+    <row r="959"/>
+    <row r="960"/>
+    <row r="961"/>
+    <row r="962"/>
+    <row r="963"/>
+    <row r="964"/>
+    <row r="965"/>
+    <row r="966"/>
+    <row r="967"/>
+    <row r="968"/>
+    <row r="969"/>
+    <row r="970"/>
+    <row r="971"/>
+    <row r="972"/>
+    <row r="973"/>
+    <row r="974"/>
+    <row r="975"/>
+    <row r="976"/>
+    <row r="977"/>
+    <row r="978"/>
+    <row r="979"/>
+    <row r="980"/>
+    <row r="981"/>
+    <row r="982"/>
+    <row r="983"/>
+    <row r="984"/>
+    <row r="985"/>
+    <row r="986"/>
+    <row r="987"/>
+    <row r="988"/>
+    <row r="989"/>
+    <row r="990"/>
+    <row r="991"/>
+    <row r="992"/>
+    <row r="993"/>
+    <row r="994"/>
+    <row r="995"/>
+    <row r="996"/>
+    <row r="997"/>
+    <row r="998"/>
+    <row r="999"/>
+    <row r="1000"/>
+    <row r="1001"/>
+    <row r="1002"/>
+    <row r="1003"/>
+    <row r="1004"/>
+    <row r="1005"/>
+    <row r="1006"/>
+    <row r="1007"/>
+    <row r="1008"/>
+    <row r="1009"/>
+    <row r="1010"/>
+    <row r="1011"/>
+    <row r="1012"/>
+    <row r="1013"/>
+    <row r="1014"/>
+    <row r="1015"/>
+    <row r="1016"/>
+    <row r="1017">
+      <c r="B1017" s="59" t="inlineStr">
         <is>
           <t>ATT-07 — ATT-06 : OK · ATT-07 : OK</t>
         </is>
       </c>
     </row>
-    <row r="991">
-      <c r="B991" s="60" t="inlineStr">
+    <row r="1018">
+      <c r="B1018" s="60" t="inlineStr">
         <is>
           <t>Cas : ATT-06, ATT-07</t>
         </is>
       </c>
     </row>
-    <row r="1018">
-      <c r="B1018" s="59" t="inlineStr">
+    <row r="1019"/>
+    <row r="1020"/>
+    <row r="1021"/>
+    <row r="1022"/>
+    <row r="1023"/>
+    <row r="1024"/>
+    <row r="1025"/>
+    <row r="1026"/>
+    <row r="1027"/>
+    <row r="1028"/>
+    <row r="1029"/>
+    <row r="1030"/>
+    <row r="1031"/>
+    <row r="1032"/>
+    <row r="1033"/>
+    <row r="1034"/>
+    <row r="1035"/>
+    <row r="1036"/>
+    <row r="1037"/>
+    <row r="1038"/>
+    <row r="1039"/>
+    <row r="1040"/>
+    <row r="1041"/>
+    <row r="1042"/>
+    <row r="1043"/>
+    <row r="1044"/>
+    <row r="1045">
+      <c r="B1045" s="59" t="inlineStr">
         <is>
           <t>COL-01 — COL-01 : OK · COL-06 : OK</t>
         </is>
       </c>
     </row>
-    <row r="1019">
-      <c r="B1019" s="60" t="inlineStr">
+    <row r="1046">
+      <c r="B1046" s="60" t="inlineStr">
         <is>
           <t>Cas : COL-01, COL-06</t>
         </is>
       </c>
     </row>
-    <row r="1050">
-      <c r="B1050" s="59" t="inlineStr">
+    <row r="1047"/>
+    <row r="1048"/>
+    <row r="1049"/>
+    <row r="1050"/>
+    <row r="1051"/>
+    <row r="1052"/>
+    <row r="1053"/>
+    <row r="1054"/>
+    <row r="1055"/>
+    <row r="1056"/>
+    <row r="1057"/>
+    <row r="1058"/>
+    <row r="1059"/>
+    <row r="1060"/>
+    <row r="1061"/>
+    <row r="1062"/>
+    <row r="1063"/>
+    <row r="1064"/>
+    <row r="1065"/>
+    <row r="1066"/>
+    <row r="1067"/>
+    <row r="1068"/>
+    <row r="1069"/>
+    <row r="1070"/>
+    <row r="1071"/>
+    <row r="1072"/>
+    <row r="1073"/>
+    <row r="1074"/>
+    <row r="1075"/>
+    <row r="1076"/>
+    <row r="1077">
+      <c r="B1077" s="59" t="inlineStr">
         <is>
           <t>COL-03 — COL-03 : À retester</t>
         </is>
       </c>
     </row>
-    <row r="1051">
-      <c r="B1051" s="60" t="inlineStr">
+    <row r="1078">
+      <c r="B1078" s="60" t="inlineStr">
         <is>
           <t>Cas : COL-03</t>
         </is>
       </c>
     </row>
-    <row r="1078">
-      <c r="B1078" s="59" t="inlineStr">
+    <row r="1079"/>
+    <row r="1080"/>
+    <row r="1081"/>
+    <row r="1082"/>
+    <row r="1083"/>
+    <row r="1084"/>
+    <row r="1085"/>
+    <row r="1086"/>
+    <row r="1087"/>
+    <row r="1088"/>
+    <row r="1089"/>
+    <row r="1090"/>
+    <row r="1091"/>
+    <row r="1092"/>
+    <row r="1093"/>
+    <row r="1094"/>
+    <row r="1095"/>
+    <row r="1096"/>
+    <row r="1097"/>
+    <row r="1098"/>
+    <row r="1099"/>
+    <row r="1100"/>
+    <row r="1101"/>
+    <row r="1102"/>
+    <row r="1103"/>
+    <row r="1104"/>
+    <row r="1105">
+      <c r="B1105" s="59" t="inlineStr">
+        <is>
+          <t>COL-05-corrige — capture complémentaire</t>
+        </is>
+      </c>
+    </row>
+    <row r="1106"/>
+    <row r="1107"/>
+    <row r="1108"/>
+    <row r="1109"/>
+    <row r="1110"/>
+    <row r="1111"/>
+    <row r="1112"/>
+    <row r="1113"/>
+    <row r="1114"/>
+    <row r="1115"/>
+    <row r="1116"/>
+    <row r="1117"/>
+    <row r="1118"/>
+    <row r="1119"/>
+    <row r="1120"/>
+    <row r="1121"/>
+    <row r="1122"/>
+    <row r="1123"/>
+    <row r="1124"/>
+    <row r="1125"/>
+    <row r="1126"/>
+    <row r="1127"/>
+    <row r="1128"/>
+    <row r="1129"/>
+    <row r="1130"/>
+    <row r="1131"/>
+    <row r="1132"/>
+    <row r="1133"/>
+    <row r="1134"/>
+    <row r="1135"/>
+    <row r="1136">
+      <c r="B1136" s="59" t="inlineStr">
         <is>
           <t>COL-05-seance-passee — Séance du 19/09 affichée « EN DIRECT · 621 h » (reste dev)</t>
         </is>
       </c>
     </row>
-    <row r="1079">
-      <c r="B1079" s="60" t="inlineStr">
+    <row r="1137">
+      <c r="B1137" s="60" t="inlineStr">
         <is>
           <t>Cas : COL-05</t>
         </is>
       </c>
     </row>
-    <row r="1106">
-      <c r="B1106" s="59" t="inlineStr">
+    <row r="1138"/>
+    <row r="1139"/>
+    <row r="1140"/>
+    <row r="1141"/>
+    <row r="1142"/>
+    <row r="1143"/>
+    <row r="1144"/>
+    <row r="1145"/>
+    <row r="1146"/>
+    <row r="1147"/>
+    <row r="1148"/>
+    <row r="1149"/>
+    <row r="1150"/>
+    <row r="1151"/>
+    <row r="1152"/>
+    <row r="1153"/>
+    <row r="1154"/>
+    <row r="1155"/>
+    <row r="1156"/>
+    <row r="1157"/>
+    <row r="1158"/>
+    <row r="1159"/>
+    <row r="1160"/>
+    <row r="1161"/>
+    <row r="1162"/>
+    <row r="1163"/>
+    <row r="1164">
+      <c r="B1164" s="59" t="inlineStr">
         <is>
           <t>FOR-05 — FOR-05 : OK</t>
         </is>
       </c>
     </row>
-    <row r="1107">
-      <c r="B1107" s="60" t="inlineStr">
+    <row r="1165">
+      <c r="B1165" s="60" t="inlineStr">
         <is>
           <t>Cas : FOR-05</t>
         </is>
       </c>
     </row>
-    <row r="1134">
-      <c r="B1134" s="59" t="inlineStr">
+    <row r="1166"/>
+    <row r="1167"/>
+    <row r="1168"/>
+    <row r="1169"/>
+    <row r="1170"/>
+    <row r="1171"/>
+    <row r="1172"/>
+    <row r="1173"/>
+    <row r="1174"/>
+    <row r="1175"/>
+    <row r="1176"/>
+    <row r="1177"/>
+    <row r="1178"/>
+    <row r="1179"/>
+    <row r="1180"/>
+    <row r="1181"/>
+    <row r="1182"/>
+    <row r="1183"/>
+    <row r="1184"/>
+    <row r="1185"/>
+    <row r="1186"/>
+    <row r="1187"/>
+    <row r="1188"/>
+    <row r="1189"/>
+    <row r="1190"/>
+    <row r="1191"/>
+    <row r="1192">
+      <c r="B1192" s="59" t="inlineStr">
         <is>
           <t>FOR-05-releve — FOR-05 : OK</t>
         </is>
       </c>
     </row>
-    <row r="1135">
-      <c r="B1135" s="60" t="inlineStr">
+    <row r="1193">
+      <c r="B1193" s="60" t="inlineStr">
         <is>
           <t>Cas : FOR-05</t>
         </is>
       </c>
     </row>
-    <row r="1162">
-      <c r="B1162" s="59" t="inlineStr">
+    <row r="1194"/>
+    <row r="1195"/>
+    <row r="1196"/>
+    <row r="1197"/>
+    <row r="1198"/>
+    <row r="1199"/>
+    <row r="1200"/>
+    <row r="1201"/>
+    <row r="1202"/>
+    <row r="1203"/>
+    <row r="1204"/>
+    <row r="1205"/>
+    <row r="1206"/>
+    <row r="1207"/>
+    <row r="1208"/>
+    <row r="1209"/>
+    <row r="1210"/>
+    <row r="1211"/>
+    <row r="1212"/>
+    <row r="1213"/>
+    <row r="1214"/>
+    <row r="1215"/>
+    <row r="1216"/>
+    <row r="1217"/>
+    <row r="1218"/>
+    <row r="1219"/>
+    <row r="1220">
+      <c r="B1220" s="59" t="inlineStr">
         <is>
           <t>PRI-02 — PRI-02 : Pas un bug</t>
         </is>
       </c>
     </row>
-    <row r="1163">
-      <c r="B1163" s="60" t="inlineStr">
+    <row r="1221">
+      <c r="B1221" s="60" t="inlineStr">
         <is>
           <t>Cas : PRI-02</t>
         </is>
       </c>
     </row>
-    <row r="1190">
-      <c r="B1190" s="59" t="inlineStr">
+    <row r="1222"/>
+    <row r="1223"/>
+    <row r="1224"/>
+    <row r="1225"/>
+    <row r="1226"/>
+    <row r="1227"/>
+    <row r="1228"/>
+    <row r="1229"/>
+    <row r="1230"/>
+    <row r="1231"/>
+    <row r="1232"/>
+    <row r="1233"/>
+    <row r="1234"/>
+    <row r="1235"/>
+    <row r="1236"/>
+    <row r="1237"/>
+    <row r="1238"/>
+    <row r="1239"/>
+    <row r="1240"/>
+    <row r="1241"/>
+    <row r="1242"/>
+    <row r="1243"/>
+    <row r="1244"/>
+    <row r="1245"/>
+    <row r="1246"/>
+    <row r="1247"/>
+    <row r="1248">
+      <c r="B1248" s="59" t="inlineStr">
         <is>
           <t>PRI-02-admin — PRI-02 : Pas un bug</t>
         </is>
       </c>
     </row>
-    <row r="1191">
-      <c r="B1191" s="60" t="inlineStr">
+    <row r="1249">
+      <c r="B1249" s="60" t="inlineStr">
         <is>
           <t>Cas : PRI-02</t>
         </is>
       </c>
     </row>
-    <row r="1235">
-      <c r="B1235" s="59" t="inlineStr">
+    <row r="1250"/>
+    <row r="1251"/>
+    <row r="1252"/>
+    <row r="1253"/>
+    <row r="1254"/>
+    <row r="1255"/>
+    <row r="1256"/>
+    <row r="1257"/>
+    <row r="1258"/>
+    <row r="1259"/>
+    <row r="1260"/>
+    <row r="1261"/>
+    <row r="1262"/>
+    <row r="1263"/>
+    <row r="1264"/>
+    <row r="1265"/>
+    <row r="1266"/>
+    <row r="1267"/>
+    <row r="1268"/>
+    <row r="1269"/>
+    <row r="1270"/>
+    <row r="1271"/>
+    <row r="1272"/>
+    <row r="1273"/>
+    <row r="1274"/>
+    <row r="1275"/>
+    <row r="1276"/>
+    <row r="1277"/>
+    <row r="1278"/>
+    <row r="1279"/>
+    <row r="1280"/>
+    <row r="1281"/>
+    <row r="1282"/>
+    <row r="1283"/>
+    <row r="1284"/>
+    <row r="1285"/>
+    <row r="1286"/>
+    <row r="1287"/>
+    <row r="1288"/>
+    <row r="1289"/>
+    <row r="1290"/>
+    <row r="1291"/>
+    <row r="1292"/>
+    <row r="1293">
+      <c r="B1293" s="59" t="inlineStr">
         <is>
           <t>PRI-04 — PRI-04 : Pas un bug</t>
         </is>
       </c>
     </row>
-    <row r="1236">
-      <c r="B1236" s="60" t="inlineStr">
+    <row r="1294">
+      <c r="B1294" s="60" t="inlineStr">
         <is>
           <t>Cas : PRI-04</t>
         </is>
       </c>
     </row>
-    <row r="1263">
-      <c r="B1263" s="59" t="inlineStr">
+    <row r="1295"/>
+    <row r="1296"/>
+    <row r="1297"/>
+    <row r="1298"/>
+    <row r="1299"/>
+    <row r="1300"/>
+    <row r="1301"/>
+    <row r="1302"/>
+    <row r="1303"/>
+    <row r="1304"/>
+    <row r="1305"/>
+    <row r="1306"/>
+    <row r="1307"/>
+    <row r="1308"/>
+    <row r="1309"/>
+    <row r="1310"/>
+    <row r="1311"/>
+    <row r="1312"/>
+    <row r="1313"/>
+    <row r="1314"/>
+    <row r="1315"/>
+    <row r="1316"/>
+    <row r="1317"/>
+    <row r="1318"/>
+    <row r="1319"/>
+    <row r="1320"/>
+    <row r="1321">
+      <c r="B1321" s="59" t="inlineStr">
         <is>
           <t>VIT-11-accueil — VIT-11 : OK</t>
         </is>
       </c>
     </row>
-    <row r="1264">
-      <c r="B1264" s="60" t="inlineStr">
+    <row r="1322">
+      <c r="B1322" s="60" t="inlineStr">
         <is>
           <t>Cas : VIT-11</t>
         </is>
       </c>
     </row>
-    <row r="1291">
-      <c r="B1291" s="59" t="inlineStr">
+    <row r="1323"/>
+    <row r="1324"/>
+    <row r="1325"/>
+    <row r="1326"/>
+    <row r="1327"/>
+    <row r="1328"/>
+    <row r="1329"/>
+    <row r="1330"/>
+    <row r="1331"/>
+    <row r="1332"/>
+    <row r="1333"/>
+    <row r="1334"/>
+    <row r="1335"/>
+    <row r="1336"/>
+    <row r="1337"/>
+    <row r="1338"/>
+    <row r="1339"/>
+    <row r="1340"/>
+    <row r="1341"/>
+    <row r="1342"/>
+    <row r="1343"/>
+    <row r="1344"/>
+    <row r="1345"/>
+    <row r="1346"/>
+    <row r="1347"/>
+    <row r="1348"/>
+    <row r="1349">
+      <c r="B1349" s="59" t="inlineStr">
         <is>
           <t>VIT-12-fiche — VIT-12 : OK</t>
         </is>
       </c>
     </row>
-    <row r="1292">
-      <c r="B1292" s="60" t="inlineStr">
+    <row r="1350">
+      <c r="B1350" s="60" t="inlineStr">
         <is>
           <t>Cas : VIT-12</t>
         </is>
       </c>
     </row>
-    <row r="1319">
-      <c r="B1319" s="59" t="inlineStr">
+    <row r="1351"/>
+    <row r="1352"/>
+    <row r="1353"/>
+    <row r="1354"/>
+    <row r="1355"/>
+    <row r="1356"/>
+    <row r="1357"/>
+    <row r="1358"/>
+    <row r="1359"/>
+    <row r="1360"/>
+    <row r="1361"/>
+    <row r="1362"/>
+    <row r="1363"/>
+    <row r="1364"/>
+    <row r="1365"/>
+    <row r="1366"/>
+    <row r="1367"/>
+    <row r="1368"/>
+    <row r="1369"/>
+    <row r="1370"/>
+    <row r="1371"/>
+    <row r="1372"/>
+    <row r="1373"/>
+    <row r="1374"/>
+    <row r="1375"/>
+    <row r="1376"/>
+    <row r="1377">
+      <c r="B1377" s="59" t="inlineStr">
         <is>
           <t>VIT-15 — VIT-15 : Bloqué — client</t>
         </is>
       </c>
     </row>
-    <row r="1320">
-      <c r="B1320" s="60" t="inlineStr">
+    <row r="1378">
+      <c r="B1378" s="60" t="inlineStr">
         <is>
           <t>Cas : VIT-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="1347">
-      <c r="B1347" s="59" t="inlineStr">
-        <is>
-          <t>ADM-12-corrige — /admin/apprenants s'affiche de nouveau (corrigé le 15/10, 27d835b)</t>
-        </is>
-      </c>
-    </row>
-    <row r="1348">
-      <c r="B1348" s="60" t="inlineStr">
-        <is>
-          <t>Cas : ADM-12, ADM-14</t>
-        </is>
-      </c>
-    </row>
-    <row r="1375">
-      <c r="B1375" s="59" t="inlineStr">
-        <is>
-          <t>COL-05-corrige — Séance du 19/09 affichée « TERMINÉE · 19 septembre à 20:00 » (corrigé le 15/10)</t>
-        </is>
-      </c>
-    </row>
-    <row r="1376">
-      <c r="B1376" s="60" t="inlineStr">
-        <is>
-          <t>Cas : COL-05</t>
         </is>
       </c>
     </row>
@@ -4049,6 +5215,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="48" t="inlineStr">
         <is>
@@ -4137,7 +5304,7 @@
       <c r="H6" s="51" t="inlineStr">
         <is>
           <t>BLQ-KYC → Captures, ligne 155
-ADM-20 → Captures, ligne 575</t>
+ADM-20 → Captures, ligne 602</t>
         </is>
       </c>
     </row>
@@ -4433,7 +5600,7 @@
       </c>
       <c r="H13" s="51" t="inlineStr">
         <is>
-          <t>ATT-05 → Captures, ligne 925</t>
+          <t>ATT-05 → Captures, ligne 952</t>
         </is>
       </c>
     </row>
@@ -4475,7 +5642,7 @@
       </c>
       <c r="H14" s="51" t="inlineStr">
         <is>
-          <t>VIT-15 → Captures, ligne 1319</t>
+          <t>VIT-15 → Captures, ligne 1377</t>
         </is>
       </c>
     </row>
@@ -4518,7 +5685,7 @@
       <c r="H15" s="51" t="inlineStr">
         <is>
           <t>BLQ-GA4 → Captures, ligne 95
-ADM-21 → Captures, ligne 684</t>
+ADM-21 → Captures, ligne 711</t>
         </is>
       </c>
     </row>
@@ -4690,6 +5857,8 @@
         </is>
       </c>
     </row>
+    <row r="20"/>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="48" t="inlineStr">
         <is>
@@ -4747,12 +5916,12 @@
       </c>
       <c r="B24" s="49" t="inlineStr">
         <is>
-          <t>/admin/apprenants plante (erreur 500)</t>
+          <t>/admin/apprenants répondait une erreur 500</t>
         </is>
       </c>
       <c r="C24" s="50" t="inlineStr">
         <is>
-          <t>Corrigé (27d835b)</t>
+          <t>Corrigé</t>
         </is>
       </c>
       <c r="D24" s="50" t="inlineStr">
@@ -4762,7 +5931,7 @@
       </c>
       <c r="E24" s="50" t="inlineStr">
         <is>
-          <t>« Cannot read properties of undefined (reading 'length') », app/pages/admin/apprenants.vue:502. Cause : une fusion a gardé l'API qui renvoie { apprenants, choix } et repris un écran qui attend une simple liste ; l'écran parcourait l'objet au lieu des apprenants. L'écran lit désormais la liste.</t>
+          <t>La page s'affiche de nouveau sans erreur (vérifié le 15/10 sur la base en ligne).</t>
         </is>
       </c>
       <c r="F24" s="50" t="inlineStr">
@@ -4772,13 +5941,12 @@
       </c>
       <c r="G24" s="50" t="inlineStr">
         <is>
-          <t>Vérifié le 15/10 sur la base en ligne : liste des 10 comptes, fiche, historique, export CSV (10 lignes, 13 colonnes), formulaire Prénom / Nom. Reste au testeur : créer un apprenant de test (ADM-12), non rejoué pour ne rien écrire en base.</t>
+          <t>Rejouer la création et l’export.</t>
         </is>
       </c>
       <c r="H24" s="51" t="inlineStr">
         <is>
-          <t>ADM-12 → Captures, ligne 547
-ADM-12-corrige → Captures, ligne 1347</t>
+          <t>ADM-12 → Captures, ligne 547</t>
         </is>
       </c>
     </row>
@@ -4790,12 +5958,12 @@
       </c>
       <c r="B25" s="49" t="inlineStr">
         <is>
-          <t>Mots de passe de démonstration encore actifs (dont l'administrateur principal)</t>
+          <t>Mot de passe de démonstration encore actif sur un administrateur principal</t>
         </is>
       </c>
       <c r="C25" s="50" t="inlineStr">
         <is>
-          <t>Big Five (lancer le script)</t>
+          <t>Développement + Big Five</t>
         </is>
       </c>
       <c r="D25" s="50" t="inlineStr">
@@ -4805,7 +5973,7 @@
       </c>
       <c r="E25" s="50" t="inlineStr">
         <is>
-          <t>Lecture du 15/10 sur la base en ligne : 6 comptes sur 7 acceptent encore le mot de passe commun du jeu de données — cossi@, jeremie.declercq@, houefa@bigfiveabidjan.com, editeur@bigfive.ci, formateur@bigfive.ci, aya@example.ci. Seul jeanluc@ l'a changé.</t>
+          <t>cossi@bigfiveabidjan.com s'ouvre avec le mot de passe publié dans le README.</t>
         </is>
       </c>
       <c r="F25" s="50" t="inlineStr">
@@ -4815,7 +5983,7 @@
       </c>
       <c r="G25" s="50" t="inlineStr">
         <is>
-          <t>Mot de passe retiré du README et du TODO le 15/10. Script prêt : npm run auth:renouveler (lecture seule) puis npm run auth:renouveler -- --appliquer, qui tire un mot de passe aléatoire par compte et l'affiche une seule fois dans le terminal : le reporter dans un gestionnaire, le transmettre à son titulaire. Puis remplacer NUXT_SESSION_PASSWORD sur Vercel pour fermer les sessions ouvertes.</t>
+          <t>Retiré du README le 15/10. Reste à changer le mot de passe de cossi@ et des autres comptes du jeu de données.</t>
         </is>
       </c>
       <c r="H25" s="50" t="inlineStr">
@@ -4837,7 +6005,7 @@
       </c>
       <c r="C26" s="50" t="inlineStr">
         <is>
-          <t>Corrigé (27d835b)</t>
+          <t>Corrigé (dans main)</t>
         </is>
       </c>
       <c r="D26" s="50" t="inlineStr">
@@ -4857,13 +6025,12 @@
       </c>
       <c r="G26" s="50" t="inlineStr">
         <is>
-          <t>Vérifié le 15/10 : la séance du 19/09 affiche « TERMINÉE · 19 septembre à 20:00 » et « Cette séance s'est terminée », bouton d'entrée grisé, y compris pour le formateur et l'administrateur (retouche du bouton à commiter).</t>
+          <t>Corrigé : une séance passée affiche « Terminée ».</t>
         </is>
       </c>
       <c r="H26" s="51" t="inlineStr">
         <is>
-          <t>COL-05-seance-passee → Captures, ligne 1078
-COL-05-corrige → Captures, ligne 1375</t>
+          <t>COL-05-seance-passee → Captures, ligne 1136</t>
         </is>
       </c>
     </row>
@@ -4922,7 +6089,7 @@
       </c>
       <c r="C28" s="50" t="inlineStr">
         <is>
-          <t>Développement</t>
+          <t>Développé (2bc3bcc)</t>
         </is>
       </c>
       <c r="D28" s="50" t="inlineStr">
@@ -4932,7 +6099,7 @@
       </c>
       <c r="E28" s="50" t="inlineStr">
         <is>
-          <t>Aucune tâche ne relit les commandes restées « En attente ».</t>
+          <t>Tâche quotidienne qui relit le statut FeexPay des commandes restées en attente.</t>
         </is>
       </c>
       <c r="F28" s="50" t="inlineStr">
@@ -4942,12 +6109,12 @@
       </c>
       <c r="G28" s="50" t="inlineStr">
         <is>
-          <t>Tâche planifiée de rapprochement.</t>
+          <t>Vérifier après déploiement.</t>
         </is>
       </c>
       <c r="H28" s="51" t="inlineStr">
         <is>
-          <t>ADM-20 → Captures, ligne 575</t>
+          <t>ADM-20 → Captures, ligne 602</t>
         </is>
       </c>
     </row>
@@ -4964,7 +6131,7 @@
       </c>
       <c r="C29" s="50" t="inlineStr">
         <is>
-          <t>Développement</t>
+          <t>Développé (2bc3bcc)</t>
         </is>
       </c>
       <c r="D29" s="50" t="inlineStr">
@@ -4974,7 +6141,7 @@
       </c>
       <c r="E29" s="50" t="inlineStr">
         <is>
-          <t>Ces paiements ne sont suivis que dans la console FeexPay.</t>
+          <t>Les paiements de séance deviennent des transactions.</t>
         </is>
       </c>
       <c r="F29" s="50" t="inlineStr">
@@ -4984,7 +6151,7 @@
       </c>
       <c r="G29" s="50" t="inlineStr">
         <is>
-          <t>Les faire apparaître dans Transactions.</t>
+          <t>Exécuter la migration 38 sur la base hébergée avant de déployer.</t>
         </is>
       </c>
       <c r="H29" s="50" t="inlineStr">
@@ -5006,7 +6173,7 @@
       </c>
       <c r="C30" s="50" t="inlineStr">
         <is>
-          <t>Développement</t>
+          <t>Corrigé (2bc3bcc)</t>
         </is>
       </c>
       <c r="D30" s="50" t="inlineStr">
@@ -5016,7 +6183,7 @@
       </c>
       <c r="E30" s="50" t="inlineStr">
         <is>
-          <t>npm run typecheck : 5 erreurs sur Referentiels.vue (sans effet sur le build).</t>
+          <t>npm run typecheck : 0 erreur.</t>
         </is>
       </c>
       <c r="F30" s="50" t="inlineStr">
@@ -5026,7 +6193,7 @@
       </c>
       <c r="G30" s="50" t="inlineStr">
         <is>
-          <t>Corriger le typage.</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H30" s="50" t="inlineStr">
@@ -5048,7 +6215,7 @@
       </c>
       <c r="C31" s="50" t="inlineStr">
         <is>
-          <t>Développement</t>
+          <t>Développé (2bc3bcc)</t>
         </is>
       </c>
       <c r="D31" s="50" t="inlineStr">
@@ -5058,7 +6225,7 @@
       </c>
       <c r="E31" s="50" t="inlineStr">
         <is>
-          <t>visionnages et reglages_attestation répondent 200 (vide) au lieu de 401.</t>
+          <t>Migration 37 : droits retirés sur toutes les tables.</t>
         </is>
       </c>
       <c r="F31" s="50" t="inlineStr">
@@ -5068,7 +6235,7 @@
       </c>
       <c r="G31" s="50" t="inlineStr">
         <is>
-          <t>Retirer le droit, comme sur les 43 autres tables.</t>
+          <t>Exécuter la migration 37 sur la base hébergée.</t>
         </is>
       </c>
       <c r="H31" s="50" t="inlineStr">
@@ -5090,7 +6257,7 @@
       </c>
       <c r="C32" s="50" t="inlineStr">
         <is>
-          <t>Développé, à fusionner</t>
+          <t>Fusionné dans main</t>
         </is>
       </c>
       <c r="D32" s="50" t="inlineStr">
@@ -5100,7 +6267,7 @@
       </c>
       <c r="E32" s="50" t="inlineStr">
         <is>
-          <t>Les deux modèles sont écrits (commit 5b98316, branche jl/practical-chatelet-e7dbbe) ; ils ne sont pas encore dans main.</t>
+          <t>Les deux modèles sont écrits et fusionnés (5b98316, a06e132).</t>
         </is>
       </c>
       <c r="F32" s="50" t="inlineStr">
@@ -5110,7 +6277,7 @@
       </c>
       <c r="G32" s="50" t="inlineStr">
         <is>
-          <t>Fusionner la branche dans main, déployer, puis vérifier les deux e-mails sur un vrai achat et une vraie délivrance.</t>
+          <t>Déployer, puis vérifier les deux e-mails sur un vrai achat et une vraie délivrance.</t>
         </is>
       </c>
       <c r="H32" s="50" t="inlineStr">
@@ -5119,6 +6286,8 @@
         </is>
       </c>
     </row>
+    <row r="33"/>
+    <row r="34"/>
     <row r="35">
       <c r="A35" s="48" t="inlineStr">
         <is>
@@ -5468,17 +6637,17 @@
     <mergeCell ref="A2:H2"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="H6" location="'Captures'!B155" display="BLQ-KYC → Captures, ligne 155&#10;ADM-20 → Captures, ligne 575"/>
+    <hyperlink ref="H6" location="'Captures'!B155" display="BLQ-KYC → Captures, ligne 155&#10;ADM-20 → Captures, ligne 602"/>
     <hyperlink ref="H10" location="'Captures'!B127" display="BLQ-JURIDIQUE → Captures, ligne 127&#10;ACH-03 → Captures, ligne 272"/>
     <hyperlink ref="H11" location="'Captures'!B184" display="BLQ-VIDEOS → Captures, ligne 184"/>
     <hyperlink ref="H12" location="'Captures'!B4" display="BLQ-CATALOGUE → Captures, ligne 4&#10;ADM-06 → Captures, ligne 519"/>
-    <hyperlink ref="H13" location="'Captures'!B925" display="ATT-05 → Captures, ligne 925"/>
-    <hyperlink ref="H14" location="'Captures'!B1319" display="VIT-15 → Captures, ligne 1319"/>
-    <hyperlink ref="H15" location="'Captures'!B95" display="BLQ-GA4 → Captures, ligne 95&#10;ADM-21 → Captures, ligne 684"/>
+    <hyperlink ref="H13" location="'Captures'!B952" display="ATT-05 → Captures, ligne 952"/>
+    <hyperlink ref="H14" location="'Captures'!B1377" display="VIT-15 → Captures, ligne 1377"/>
+    <hyperlink ref="H15" location="'Captures'!B95" display="BLQ-GA4 → Captures, ligne 95&#10;ADM-21 → Captures, ligne 711"/>
     <hyperlink ref="H17" location="'Captures'!B66" display="BLQ-FEEXPAY → Captures, ligne 66"/>
     <hyperlink ref="H24" location="'Captures'!B547" display="ADM-12 → Captures, ligne 547"/>
-    <hyperlink ref="H26" location="'Captures'!B1078" display="COL-05-seance-passee → Captures, ligne 1078"/>
-    <hyperlink ref="H28" location="'Captures'!B575" display="ADM-20 → Captures, ligne 575"/>
+    <hyperlink ref="H26" location="'Captures'!B1136" display="COL-05-seance-passee → Captures, ligne 1136"/>
+    <hyperlink ref="H28" location="'Captures'!B602" display="ADM-20 → Captures, ligne 602"/>
     <hyperlink ref="H39" location="'Captures'!B378" display="ACH-04-prefill → Captures, ligne 378"/>
     <hyperlink ref="H43" location="'Captures'!B414" display="ACH-04-wave → Captures, ligne 414&#10;ACH-04-carte → Captures, ligne 340"/>
   </hyperlinks>
@@ -5526,6 +6695,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1" s="31">
       <c r="A4" s="32" t="inlineStr">
         <is>
@@ -6206,7 +7376,7 @@
       </c>
       <c r="O15" s="53" t="inlineStr">
         <is>
-          <t>VIT-11-accueil → ligne 1263
+          <t>VIT-11-accueil → ligne 1321
 BLQ-CATALOGUE → ligne 4</t>
         </is>
       </c>
@@ -6272,7 +7442,7 @@
       </c>
       <c r="O16" s="53" t="inlineStr">
         <is>
-          <t>VIT-12-fiche → ligne 1291</t>
+          <t>VIT-12-fiche → ligne 1349</t>
         </is>
       </c>
     </row>
@@ -6456,7 +7626,7 @@
       </c>
       <c r="O19" s="53" t="inlineStr">
         <is>
-          <t>VIT-15 → ligne 1319</t>
+          <t>VIT-15 → ligne 1377</t>
         </is>
       </c>
     </row>
@@ -7351,7 +8521,7 @@
       <c r="O34" s="53" t="inlineStr">
         <is>
           <t>BLQ-FEEXPAY → ligne 66
-ADM-20 → ligne 575</t>
+ADM-20 → ligne 602</t>
         </is>
       </c>
     </row>
@@ -7620,8 +8790,16 @@
           <t>Toujours à faire : aucune tâche planifiée ne relit les commandes restées « en attente » (19 dans la base au 15/10). Seule la vérification commande par commande existe.</t>
         </is>
       </c>
-      <c r="M38" s="33" t="n"/>
-      <c r="N38" s="33" t="n"/>
+      <c r="M38" s="55" t="inlineStr">
+        <is>
+          <t>À retester</t>
+        </is>
+      </c>
+      <c r="N38" s="33" t="inlineStr">
+        <is>
+          <t>Développé le 15/10 : relance quotidienne des commandes restées en attente (cron Vercel 04:00, /api/taches/commandes), qui relit leur statut chez FeexPay. À vérifier après déploiement.</t>
+        </is>
+      </c>
       <c r="O38" s="33" t="n"/>
     </row>
     <row r="39" ht="15.75" customHeight="1" s="31">
@@ -7680,7 +8858,7 @@
       </c>
       <c r="N39" s="33" t="inlineStr">
         <is>
-          <t>Développé le 15/10 (commit 5b98316, branche jl/practical-chatelet-e7dbbe) : e-mail de confirmation d'achat avec module ou séance, montant, moyen et référence, envoyé une seule fois par commande. Pas encore fusionné dans main ni déployé : à retester en ligne après fusion, avec un vrai paiement.</t>
+          <t>Développé le 15/10 (commit 5b98316, fusionné dans main) : e-mail de confirmation d'achat avec module ou séance, montant, moyen et référence, envoyé une seule fois par commande. À retester en ligne après déploiement, avec un vrai paiement.</t>
         </is>
       </c>
       <c r="O39" s="33" t="n"/>
@@ -7994,7 +9172,7 @@
       </c>
       <c r="O44" s="53" t="inlineStr">
         <is>
-          <t>APP-03 → ligne 754</t>
+          <t>APP-03 → ligne 781</t>
         </is>
       </c>
     </row>
@@ -8125,7 +9303,7 @@
       </c>
       <c r="O46" s="53" t="inlineStr">
         <is>
-          <t>APP-05 → ligne 782</t>
+          <t>APP-05 → ligne 809</t>
         </is>
       </c>
     </row>
@@ -8256,8 +9434,8 @@
       </c>
       <c r="O48" s="53" t="inlineStr">
         <is>
-          <t>APP-07 → ligne 810
-APP-07-mobile → ligne 838</t>
+          <t>APP-07 → ligne 837
+APP-07-mobile → ligne 865</t>
         </is>
       </c>
     </row>
@@ -9087,7 +10265,7 @@
       </c>
       <c r="O62" s="53" t="inlineStr">
         <is>
-          <t>COL-01 → ligne 1018</t>
+          <t>COL-01 → ligne 1045</t>
         </is>
       </c>
     </row>
@@ -9217,7 +10395,7 @@
       </c>
       <c r="O64" s="53" t="inlineStr">
         <is>
-          <t>COL-03 → ligne 1050</t>
+          <t>COL-03 → ligne 1077</t>
         </is>
       </c>
     </row>
@@ -9334,12 +10512,12 @@
       </c>
       <c r="N66" s="33" t="inlineStr">
         <is>
-          <t>Zoom en réel depuis le 15/10. Création automatique validée : la session ses-010 créée depuis le site à 19:53 a reçu la réunion 83441083225, présente chez Zoom sous le compte cossi@bigfiveabidjan.com (2 h, salle d'attente). Restent à dérouler : entrée formateur et apprenant depuis la plateforme, report et annulation d'une réunion réelle. Une séance passée s'affichait « EN DIRECT · 621 h » : corrigé (27d835b) et vérifié le 15/10, elle affiche « TERMINÉE · 19 septembre à 20:00 ».</t>
+          <t>Zoom en réel depuis le 15/10. Création automatique validée : la session ses-010 créée depuis le site à 19:53 a reçu la réunion 83441083225, présente chez Zoom sous le compte cossi@bigfiveabidjan.com (2 h, salle d'attente). Restent à dérouler : entrée formateur et apprenant depuis la plateforme, report et annulation d'une réunion réelle. Une séance passée s'affichait « EN DIRECT » : corrigé.</t>
         </is>
       </c>
       <c r="O66" s="53" t="inlineStr">
         <is>
-          <t>COL-05-seance-passee → ligne 1078 · COL-05-corrige → ligne 1375</t>
+          <t>COL-05-seance-passee → ligne 1136</t>
         </is>
       </c>
     </row>
@@ -9404,7 +10582,7 @@
       </c>
       <c r="O67" s="53" t="inlineStr">
         <is>
-          <t>COL-01 → ligne 1018</t>
+          <t>COL-01 → ligne 1045</t>
         </is>
       </c>
     </row>
@@ -9640,8 +10818,8 @@
       </c>
       <c r="O71" s="53" t="inlineStr">
         <is>
-          <t>PRI-02 → ligne 1162
-PRI-02-admin → ligne 1190</t>
+          <t>PRI-02 → ligne 1220
+PRI-02-admin → ligne 1248</t>
         </is>
       </c>
     </row>
@@ -9771,7 +10949,7 @@
       </c>
       <c r="O73" s="53" t="inlineStr">
         <is>
-          <t>PRI-04 → ligne 1235</t>
+          <t>PRI-04 → ligne 1293</t>
         </is>
       </c>
     </row>
@@ -9991,8 +11169,16 @@
           <t>Le coaching privé passe par le même tunnel FeexPay que les modules ; dépend des clés live. Ces paiements ne créent pas de ligne dans /admin/transactions.</t>
         </is>
       </c>
-      <c r="M77" s="33" t="n"/>
-      <c r="N77" s="33" t="n"/>
+      <c r="M77" s="55" t="inlineStr">
+        <is>
+          <t>À retester</t>
+        </is>
+      </c>
+      <c r="N77" s="33" t="inlineStr">
+        <is>
+          <t>Le paiement d'une séance de coaching privé devient une transaction visible dans /admin/transactions et les revenus. Exige la migration 38 sur la base hébergée (pas encore exécutée au 15/10 au soir).</t>
+        </is>
+      </c>
       <c r="O77" s="33" t="n"/>
     </row>
     <row r="78" ht="15.75" customHeight="1" s="31">
@@ -10276,7 +11462,7 @@
       </c>
       <c r="O82" s="53" t="inlineStr">
         <is>
-          <t>ATT-05 → ligne 925</t>
+          <t>ATT-05 → ligne 952</t>
         </is>
       </c>
     </row>
@@ -10353,7 +11539,7 @@
       </c>
       <c r="O83" s="53" t="inlineStr">
         <is>
-          <t>ATT-07 → ligne 990</t>
+          <t>ATT-07 → ligne 1017</t>
         </is>
       </c>
     </row>
@@ -10426,7 +11612,7 @@
       </c>
       <c r="O84" s="53" t="inlineStr">
         <is>
-          <t>ATT-07 → ligne 990</t>
+          <t>ATT-07 → ligne 1017</t>
         </is>
       </c>
     </row>
@@ -10539,7 +11725,7 @@
       </c>
       <c r="N86" s="33" t="inlineStr">
         <is>
-          <t>Développé le 15/10 (commit 5b98316, même branche) : e-mail d'attestation avec le numéro EMBF, le lien vers l'attestation et le lien de vérification, envoyé à la première délivrance. À retester en ligne après fusion.</t>
+          <t>Développé le 15/10 (commit 5b98316, fusionné dans main) : e-mail d'attestation avec le numéro EMBF, le lien vers l'attestation et le lien de vérification, envoyé à la première délivrance. À retester en ligne après déploiement.</t>
         </is>
       </c>
       <c r="O86" s="33" t="n"/>
@@ -10821,8 +12007,8 @@
       </c>
       <c r="O91" s="53" t="inlineStr">
         <is>
-          <t>FOR-05 → ligne 1106
-FOR-05-releve → ligne 1134</t>
+          <t>FOR-05 → ligne 1164
+FOR-05-releve → ligne 1192</t>
         </is>
       </c>
     </row>
@@ -11701,19 +12887,19 @@
           <t>Corrigé le 13/10 : prénom et nom saisis séparément à la création, motif de refus affiché. À retester.</t>
         </is>
       </c>
-      <c r="M106" s="56" t="inlineStr">
+      <c r="M106" s="55" t="inlineStr">
         <is>
           <t>À retester</t>
         </is>
       </c>
       <c r="N106" s="33" t="inlineStr">
         <is>
-          <t>Défaut du 15/10 (500 sur /admin/apprenants) corrigé le soir même (27d835b) et vérifié sur la base en ligne : liste, fiche, historique et formulaire Prénom / Nom s'affichent. La création elle-même reste à rejouer par le testeur avec un compte de test.</t>
+          <t>La page /admin/apprenants s'affiche de nouveau sans erreur (vérifié le 15/10 sur la base en ligne). Reste à rejouer la création d'un apprenant (prénom et nom séparés).</t>
         </is>
       </c>
       <c r="O106" s="53" t="inlineStr">
         <is>
-          <t>ADM-12 → ligne 547 · ADM-12-corrige → ligne 1347</t>
+          <t>ADM-12 → ligne 547</t>
         </is>
       </c>
     </row>
@@ -11823,21 +13009,17 @@
           <t>Développé : export CSV de la liste des apprenants, selon les filtres actifs.</t>
         </is>
       </c>
-      <c r="M108" s="56" t="inlineStr">
-        <is>
-          <t>OK</t>
+      <c r="M108" s="55" t="inlineStr">
+        <is>
+          <t>À retester</t>
         </is>
       </c>
       <c r="N108" s="33" t="inlineStr">
         <is>
-          <t>Corrigé avec ADM-12 : l'export CSV produit les 10 comptes affichés (13 colonnes), filtres respectés. Vérifié le 15/10 au soir.</t>
-        </is>
-      </c>
-      <c r="O108" s="53" t="inlineStr">
-        <is>
-          <t>ADM-12-corrige → ligne 1347</t>
-        </is>
-      </c>
+          <t>La page s'affichant de nouveau, l'export CSV est accessible : à rejouer.</t>
+        </is>
+      </c>
+      <c r="O108" s="33" t="n"/>
     </row>
     <row r="109" ht="27" customHeight="1" s="31">
       <c r="A109" s="33" t="inlineStr">
@@ -12217,8 +13399,8 @@
       </c>
       <c r="O114" s="53" t="inlineStr">
         <is>
-          <t>ADM-20 → ligne 575
-ADM-20-editeur → ligne 656</t>
+          <t>ADM-20 → ligne 602
+ADM-20-editeur → ligne 683</t>
         </is>
       </c>
     </row>
@@ -12295,7 +13477,7 @@
       </c>
       <c r="O115" s="53" t="inlineStr">
         <is>
-          <t>ADM-21 → ligne 684</t>
+          <t>ADM-21 → ligne 711</t>
         </is>
       </c>
     </row>
@@ -12372,7 +13554,7 @@
       </c>
       <c r="O116" s="53" t="inlineStr">
         <is>
-          <t>ADM-22 → ligne 712</t>
+          <t>ADM-22 → ligne 739</t>
         </is>
       </c>
     </row>
@@ -12449,7 +13631,7 @@
       </c>
       <c r="O117" s="53" t="inlineStr">
         <is>
-          <t>ADM-22 → ligne 712</t>
+          <t>ADM-22 → ligne 739</t>
         </is>
       </c>
     </row>
@@ -12526,7 +13708,7 @@
       </c>
       <c r="O118" s="53" t="inlineStr">
         <is>
-          <t>ADM-22 → ligne 712</t>
+          <t>ADM-22 → ligne 739</t>
         </is>
       </c>
     </row>
@@ -13242,8 +14424,16 @@
           <t>Testé le 15/10 sur la base en ligne avec la clé publique : 43 tables sur 45 refusent (401). visionnages et reglages_attestation répondent 200 mais vide (RLS filtre tout) : le droit de lecture n'a pas été retiré comme ailleurs, à aligner.</t>
         </is>
       </c>
-      <c r="M130" s="33" t="n"/>
-      <c r="N130" s="33" t="n"/>
+      <c r="M130" s="55" t="inlineStr">
+        <is>
+          <t>À retester</t>
+        </is>
+      </c>
+      <c r="N130" s="33" t="inlineStr">
+        <is>
+          <t>Migration 37 écrite : RLS activé et droits retirés sur toutes les tables, y compris visionnages et reglages_attestation. À exécuter sur la base hébergée, puis revérifier avec la clé publique.</t>
+        </is>
+      </c>
       <c r="O130" s="33" t="n"/>
     </row>
     <row r="131" ht="15.75" customHeight="1" s="31">
@@ -13371,7 +14561,7 @@
       </c>
       <c r="N132" s="33" t="inlineStr">
         <is>
-          <t>Le 15/10, 6 comptes sur 7 acceptent encore le mot de passe de démonstration, dont l'administrateur principal cossi@bigfiveabidjan.com (seul jeanluc@ a été changé). Retiré du README le 15/10 ; script npm run auth:renouveler prêt, à lancer par Big Five (voir « En attente client », D2).</t>
+          <t>Le 15/10, le compte administrateur principal cossi@bigfiveabidjan.com s'ouvre encore avec le mot de passe de démonstration publié dans le README. À changer immédiatement (jeanluc@ a déjà été changé).</t>
         </is>
       </c>
       <c r="O132" s="33" t="n"/>
@@ -14230,14 +15420,14 @@
           <t>npm run typecheck échoue le 15/10 : 5 erreurs TS2321 « Excessive stack depth » sur app/components/admin/Referentiels.vue:64 (typage des routes de $fetch). Sans effet sur le build.</t>
         </is>
       </c>
-      <c r="M146" s="56" t="inlineStr">
-        <is>
-          <t>KO</t>
+      <c r="M146" s="52" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="N146" s="33" t="inlineStr">
         <is>
-          <t>Inchangé : 5 erreurs TS2321 sur app/components/admin/Referentiels.vue. Sans effet sur le build.</t>
+          <t>npm run typecheck passe sans aucune erreur le 15/10 au soir (Referentiels.vue corrigé).</t>
         </is>
       </c>
       <c r="O146" s="33" t="n"/>
@@ -15347,46 +16537,45 @@
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="O15" location="'Captures'!B1263" display="VIT-11-accueil → ligne 1263&#10;BLQ-CATALOGUE → ligne 4"/>
-    <hyperlink ref="O16" location="'Captures'!B1291" display="VIT-12-fiche → ligne 1291"/>
+    <hyperlink ref="O15" location="'Captures'!B1321" display="VIT-11-accueil → ligne 1321&#10;BLQ-CATALOGUE → ligne 4"/>
+    <hyperlink ref="O16" location="'Captures'!B1349" display="VIT-12-fiche → ligne 1349"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J19" r:id="rId1"/>
-    <hyperlink ref="O19" location="'Captures'!B1319" display="VIT-15 → ligne 1319"/>
+    <hyperlink ref="O19" location="'Captures'!B1377" display="VIT-15 → ligne 1377"/>
     <hyperlink ref="O24" location="'Captures'!B127" display="BLQ-JURIDIQUE → ligne 127"/>
     <hyperlink ref="O32" location="'Captures'!B272" display="ACH-03 → ligne 272"/>
     <hyperlink ref="O33" location="'Captures'!B306" display="ACH-04 → ligne 306&#10;ACH-04-wave → ligne 414&#10;ACH-04-carte → ligne 340&#10;ACH-04-prefill → ligne 378"/>
-    <hyperlink ref="O34" location="'Captures'!B66" display="BLQ-FEEXPAY → ligne 66&#10;ADM-20 → ligne 575"/>
+    <hyperlink ref="O34" location="'Captures'!B66" display="BLQ-FEEXPAY → ligne 66&#10;ADM-20 → ligne 602"/>
     <hyperlink ref="O35" location="'Captures'!B66" display="BLQ-FEEXPAY → ligne 66"/>
     <hyperlink ref="O36" location="'Captures'!B66" display="BLQ-FEEXPAY → ligne 66&#10;BLQ-KYC → ligne 155"/>
     <hyperlink ref="O37" location="'Captures'!B66" display="BLQ-FEEXPAY → ligne 66"/>
     <hyperlink ref="O41" location="'Captures'!B452" display="ACH-12 → ligne 452"/>
-    <hyperlink ref="O44" location="'Captures'!B754" display="APP-03 → ligne 754"/>
+    <hyperlink ref="O44" location="'Captures'!B781" display="APP-03 → ligne 781"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J46" r:id="rId2"/>
-    <hyperlink ref="O46" location="'Captures'!B782" display="APP-05 → ligne 782"/>
+    <hyperlink ref="O46" location="'Captures'!B809" display="APP-05 → ligne 809"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J48" r:id="rId3"/>
-    <hyperlink ref="O48" location="'Captures'!B810" display="APP-07 → ligne 810&#10;APP-07-mobile → ligne 838"/>
+    <hyperlink ref="O48" location="'Captures'!B837" display="APP-07 → ligne 837&#10;APP-07-mobile → ligne 865"/>
     <hyperlink ref="O59" location="'Captures'!B184" display="BLQ-VIDEOS → ligne 184"/>
-    <hyperlink ref="O62" location="'Captures'!B1018" display="COL-01 → ligne 1018"/>
-    <hyperlink ref="O64" location="'Captures'!B1050" display="COL-03 → ligne 1050"/>
-    <hyperlink ref="O66" location="'Captures'!B1078" display="COL-05-seance-passee → ligne 1078"/>
-    <hyperlink ref="O67" location="'Captures'!B1018" display="COL-01 → ligne 1018"/>
-    <hyperlink ref="O71" location="'Captures'!B1162" display="PRI-02 → ligne 1162&#10;PRI-02-admin → ligne 1190"/>
-    <hyperlink ref="O73" location="'Captures'!B1235" display="PRI-04 → ligne 1235"/>
-    <hyperlink ref="O82" location="'Captures'!B925" display="ATT-05 → ligne 925"/>
-    <hyperlink ref="O83" location="'Captures'!B990" display="ATT-07 → ligne 990"/>
-    <hyperlink ref="O84" location="'Captures'!B990" display="ATT-07 → ligne 990"/>
-    <hyperlink ref="O91" location="'Captures'!B1106" display="FOR-05 → ligne 1106&#10;FOR-05-releve → ligne 1134"/>
+    <hyperlink ref="O62" location="'Captures'!B1045" display="COL-01 → ligne 1045"/>
+    <hyperlink ref="O64" location="'Captures'!B1077" display="COL-03 → ligne 1077"/>
+    <hyperlink ref="O66" location="'Captures'!B1136" display="COL-05-seance-passee → ligne 1136"/>
+    <hyperlink ref="O67" location="'Captures'!B1045" display="COL-01 → ligne 1045"/>
+    <hyperlink ref="O71" location="'Captures'!B1220" display="PRI-02 → ligne 1220&#10;PRI-02-admin → ligne 1248"/>
+    <hyperlink ref="O73" location="'Captures'!B1293" display="PRI-04 → ligne 1293"/>
+    <hyperlink ref="O82" location="'Captures'!B952" display="ATT-05 → ligne 952"/>
+    <hyperlink ref="O83" location="'Captures'!B1017" display="ATT-07 → ligne 1017"/>
+    <hyperlink ref="O84" location="'Captures'!B1017" display="ATT-07 → ligne 1017"/>
+    <hyperlink ref="O91" location="'Captures'!B1164" display="FOR-05 → ligne 1164&#10;FOR-05-releve → ligne 1192"/>
     <hyperlink ref="O99" location="'Captures'!B491" display="ADM-05 → ligne 491"/>
     <hyperlink ref="O100" location="'Captures'!B519" display="ADM-06 → ligne 519"/>
     <hyperlink ref="O101" location="'Captures'!B519" display="ADM-06 → ligne 519"/>
     <hyperlink ref="O106" location="'Captures'!B547" display="ADM-12 → ligne 547"/>
-    <hyperlink ref="O108" location="'Captures'!B547" display="ADM-12 → ligne 547"/>
     <hyperlink ref="O111" location="'Captures'!B95" display="BLQ-GA4 → ligne 95"/>
     <hyperlink ref="O112" location="'Captures'!B95" display="BLQ-GA4 → ligne 95"/>
-    <hyperlink ref="O114" location="'Captures'!B575" display="ADM-20 → ligne 575&#10;ADM-20-editeur → ligne 656"/>
-    <hyperlink ref="O115" location="'Captures'!B684" display="ADM-21 → ligne 684"/>
-    <hyperlink ref="O116" location="'Captures'!B712" display="ADM-22 → ligne 712"/>
-    <hyperlink ref="O117" location="'Captures'!B712" display="ADM-22 → ligne 712"/>
-    <hyperlink ref="O118" location="'Captures'!B712" display="ADM-22 → ligne 712"/>
+    <hyperlink ref="O114" location="'Captures'!B602" display="ADM-20 → ligne 602&#10;ADM-20-editeur → ligne 683"/>
+    <hyperlink ref="O115" location="'Captures'!B711" display="ADM-21 → ligne 711"/>
+    <hyperlink ref="O116" location="'Captures'!B739" display="ADM-22 → ligne 739"/>
+    <hyperlink ref="O117" location="'Captures'!B739" display="ADM-22 → ligne 739"/>
+    <hyperlink ref="O118" location="'Captures'!B739" display="ADM-22 → ligne 739"/>
     <hyperlink ref="O120" location="'Captures'!B452" display="ACH-12 → ligne 452"/>
     <hyperlink ref="O142" location="'Captures'!B37" display="BLQ-CONFIG → ligne 37"/>
     <hyperlink ref="O143" location="'Captures'!B95" display="BLQ-GA4 → ligne 95"/>
@@ -15430,6 +16619,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1" s="31">
       <c r="A4" s="32" t="inlineStr">
         <is>
@@ -17932,6 +19122,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1" s="31">
       <c r="A4" s="32" t="inlineStr">
         <is>
@@ -19792,6 +20983,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="32" t="inlineStr">
         <is>
@@ -20821,6 +22013,7 @@
       </c>
       <c r="G32" s="33" t="n"/>
     </row>
+    <row r="33"/>
     <row r="34" ht="45" customHeight="1" s="31">
       <c r="A34" s="43" t="inlineStr">
         <is>
@@ -20828,6 +22021,7 @@
         </is>
       </c>
     </row>
+    <row r="35"/>
     <row r="36">
       <c r="A36" s="58" t="inlineStr">
         <is>
@@ -21077,6 +22271,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1" s="31">
       <c r="A4" s="32" t="inlineStr">
         <is>
@@ -22392,6 +23587,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1" s="31">
       <c r="A4" s="32" t="inlineStr">
         <is>
@@ -24032,6 +25228,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1" s="31">
       <c r="A4" s="16" t="inlineStr">
         <is>
@@ -24267,6 +25464,7 @@
       </c>
       <c r="E12" s="33" t="n"/>
     </row>
+    <row r="13"/>
     <row r="14" ht="31.5" customHeight="1" s="31">
       <c r="A14" s="4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Compte rendu des défauts D1 à D3 du retest du 15/10
- docs/compte-rendu-retest-15-10.md : cause, correctif et vérification de
  l'erreur 500 sur /admin/apprenants, de la séance passée affichée « En
  direct », et procédure de renouvellement des mots de passe de démonstration
  (npm run auth:renouveler).
- Classeur de clôture : D1 et D3 vérifiés sur la base en ligne, D2 passe à
  Big Five avec le script ; ADM-14 OK, ADM-12 à retester (création non
  rejouée), SEC-11 et la Synthèse à jour. Ces textes avaient été perdus par
  la régénération de 7d137ac ; ils sont réappliqués sur sa version.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Recette E-Masterclass BigFive — clôture 15-10.xlsx
+++ b/Recette E-Masterclass BigFive — clôture 15-10.xlsx
@@ -531,6 +531,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -556,6 +559,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -581,6 +587,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -606,6 +615,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -631,6 +643,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -656,6 +671,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -681,6 +699,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -706,6 +727,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -731,6 +755,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -756,6 +783,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -781,6 +811,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -806,6 +839,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -831,6 +867,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -856,6 +895,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -881,6 +923,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -906,6 +951,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -931,6 +979,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -956,6 +1007,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -981,6 +1035,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1006,6 +1063,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1031,6 +1091,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1056,6 +1119,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1081,6 +1147,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1106,6 +1175,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1131,6 +1203,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1156,6 +1231,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1181,6 +1259,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1206,6 +1287,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1231,6 +1315,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1256,6 +1343,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1281,6 +1371,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1306,6 +1399,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1331,6 +1427,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1356,6 +1455,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1381,6 +1483,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1406,6 +1511,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1431,6 +1539,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1456,6 +1567,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1481,6 +1595,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1506,6 +1623,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1804,7 +1924,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
@@ -2209,7 +2328,7 @@
     <row r="44" ht="27.75" customHeight="1" s="31">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>• Mot de passe de démonstration commun encore actif sur tous les comptes et écrit dans le README.</t>
+          <t>• Mot de passe de démonstration commun encore actif sur 6 comptes sur 7 ; retiré du README le 15/10, script de renouvellement prêt (D2).</t>
         </is>
       </c>
     </row>
@@ -2230,14 +2349,14 @@
     <row r="47" ht="27.75" customHeight="1" s="31">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>• /admin/apprenants plante (erreur 500) depuis le 15/10 : création et export d'apprenants indisponibles — reste dev (D1).</t>
+          <t>• /admin/apprenants : l'erreur 500 du 15/10 est corrigée (27d835b) et vérifiée ; reste à rejouer la création d'un apprenant (ADM-12).</t>
         </is>
       </c>
     </row>
     <row r="48" ht="27.75" customHeight="1" s="31">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>• Le compte administrateur principal cossi@bigfiveabidjan.com s'ouvre encore avec le mot de passe de démonstration publié — à changer immédiatement (D2).</t>
+          <t>• Le compte administrateur principal cossi@bigfiveabidjan.com s'ouvre encore avec le mot de passe de démonstration : lancer npm run auth:renouveler -- --appliquer (D2).</t>
         </is>
       </c>
     </row>
@@ -3316,7 +3435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1378"/>
+  <dimension ref="B1:B1378"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" style="31" min="1" max="1"/>
@@ -4110,7 +4229,7 @@
     <row r="575">
       <c r="B575" s="59" t="inlineStr">
         <is>
-          <t>ADM-12-corrige — capture complémentaire</t>
+          <t>ADM-12-corrige — /admin/apprenants s'affiche de nouveau (corrigé le 15/10, 27d835b)</t>
         </is>
       </c>
     </row>
@@ -4790,7 +4909,7 @@
     <row r="1105">
       <c r="B1105" s="59" t="inlineStr">
         <is>
-          <t>COL-05-corrige — capture complémentaire</t>
+          <t>COL-05-corrige — Séance du 19/09 affichée « TERMINÉE · 19 septembre à 20:00 » (corrigé le 15/10)</t>
         </is>
       </c>
     </row>
@@ -5215,7 +5334,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="48" t="inlineStr">
         <is>
@@ -5857,8 +5975,6 @@
         </is>
       </c>
     </row>
-    <row r="20"/>
-    <row r="21"/>
     <row r="22">
       <c r="A22" s="48" t="inlineStr">
         <is>
@@ -5921,7 +6037,7 @@
       </c>
       <c r="C24" s="50" t="inlineStr">
         <is>
-          <t>Corrigé</t>
+          <t>Corrigé (27d835b)</t>
         </is>
       </c>
       <c r="D24" s="50" t="inlineStr">
@@ -5931,7 +6047,7 @@
       </c>
       <c r="E24" s="50" t="inlineStr">
         <is>
-          <t>La page s'affiche de nouveau sans erreur (vérifié le 15/10 sur la base en ligne).</t>
+          <t>La page s'affiche de nouveau sans erreur (vérifié le 15/10 sur la base en ligne). Cause : une fusion a gardé l'API qui renvoie { apprenants, choix } et repris un écran qui attend une simple liste ; l'écran lit désormais la liste.</t>
         </is>
       </c>
       <c r="F24" s="50" t="inlineStr">
@@ -5941,12 +6057,13 @@
       </c>
       <c r="G24" s="50" t="inlineStr">
         <is>
-          <t>Rejouer la création et l’export.</t>
+          <t>Vérifié le 15/10 : liste des 10 comptes, fiche, historique, export CSV (10 lignes, 13 colonnes), formulaire Prénom / Nom. Reste au testeur : créer un apprenant de test (ADM-12), non rejoué pour ne rien écrire en base.</t>
         </is>
       </c>
       <c r="H24" s="51" t="inlineStr">
         <is>
-          <t>ADM-12 → Captures, ligne 547</t>
+          <t>ADM-12 → Captures, ligne 547
+ADM-12-corrige → Captures, ligne 575</t>
         </is>
       </c>
     </row>
@@ -5958,12 +6075,12 @@
       </c>
       <c r="B25" s="49" t="inlineStr">
         <is>
-          <t>Mot de passe de démonstration encore actif sur un administrateur principal</t>
+          <t>Mots de passe de démonstration encore actifs (dont l'administrateur principal)</t>
         </is>
       </c>
       <c r="C25" s="50" t="inlineStr">
         <is>
-          <t>Développement + Big Five</t>
+          <t>Big Five (lancer le script)</t>
         </is>
       </c>
       <c r="D25" s="50" t="inlineStr">
@@ -5973,7 +6090,7 @@
       </c>
       <c r="E25" s="50" t="inlineStr">
         <is>
-          <t>cossi@bigfiveabidjan.com s'ouvre avec le mot de passe publié dans le README.</t>
+          <t>Lecture du 15/10 sur la base en ligne : 6 comptes sur 7 acceptent encore le mot de passe commun du jeu de données — cossi@, jeremie.declercq@, houefa@bigfiveabidjan.com, editeur@bigfive.ci, formateur@bigfive.ci, aya@example.ci. Seul jeanluc@ l'a changé.</t>
         </is>
       </c>
       <c r="F25" s="50" t="inlineStr">
@@ -5983,7 +6100,7 @@
       </c>
       <c r="G25" s="50" t="inlineStr">
         <is>
-          <t>Retiré du README le 15/10. Reste à changer le mot de passe de cossi@ et des autres comptes du jeu de données.</t>
+          <t>Mot de passe retiré du README et du TODO le 15/10. Script prêt : npm run auth:renouveler (lecture seule) puis npm run auth:renouveler -- --appliquer, qui tire un mot de passe aléatoire par compte et l'affiche une seule fois dans le terminal : le reporter dans un gestionnaire, le transmettre à son titulaire. Puis remplacer NUXT_SESSION_PASSWORD sur Vercel pour fermer les sessions ouvertes.</t>
         </is>
       </c>
       <c r="H25" s="50" t="inlineStr">
@@ -6005,7 +6122,7 @@
       </c>
       <c r="C26" s="50" t="inlineStr">
         <is>
-          <t>Corrigé (dans main)</t>
+          <t>Corrigé (27d835b)</t>
         </is>
       </c>
       <c r="D26" s="50" t="inlineStr">
@@ -6025,12 +6142,13 @@
       </c>
       <c r="G26" s="50" t="inlineStr">
         <is>
-          <t>Corrigé : une séance passée affiche « Terminée ».</t>
+          <t>Vérifié le 15/10 : la séance du 19/09 affiche « TERMINÉE · 19 septembre à 20:00 » et « Cette séance s'est terminée », bouton d'entrée grisé, y compris pour le formateur et l'administrateur.</t>
         </is>
       </c>
       <c r="H26" s="51" t="inlineStr">
         <is>
-          <t>COL-05-seance-passee → Captures, ligne 1136</t>
+          <t>COL-05-seance-passee → Captures, ligne 1136
+COL-05-corrige → Captures, ligne 1105</t>
         </is>
       </c>
     </row>
@@ -6286,8 +6404,6 @@
         </is>
       </c>
     </row>
-    <row r="33"/>
-    <row r="34"/>
     <row r="35">
       <c r="A35" s="48" t="inlineStr">
         <is>
@@ -6695,7 +6811,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="30" customHeight="1" s="31">
       <c r="A4" s="32" t="inlineStr">
         <is>
@@ -10512,12 +10627,12 @@
       </c>
       <c r="N66" s="33" t="inlineStr">
         <is>
-          <t>Zoom en réel depuis le 15/10. Création automatique validée : la session ses-010 créée depuis le site à 19:53 a reçu la réunion 83441083225, présente chez Zoom sous le compte cossi@bigfiveabidjan.com (2 h, salle d'attente). Restent à dérouler : entrée formateur et apprenant depuis la plateforme, report et annulation d'une réunion réelle. Une séance passée s'affichait « EN DIRECT » : corrigé.</t>
+          <t>Zoom en réel depuis le 15/10. Création automatique validée : la session ses-010 créée depuis le site à 19:53 a reçu la réunion 83441083225, présente chez Zoom sous le compte cossi@bigfiveabidjan.com (2 h, salle d'attente). Restent à dérouler : entrée formateur et apprenant depuis la plateforme, report et annulation d'une réunion réelle. Une séance passée s'affichait « EN DIRECT · 621 h » : corrigé (27d835b) et vérifié le 15/10, elle affiche « TERMINÉE · 19 septembre à 20:00 ».</t>
         </is>
       </c>
       <c r="O66" s="53" t="inlineStr">
         <is>
-          <t>COL-05-seance-passee → ligne 1136</t>
+          <t>COL-05-seance-passee → ligne 1136 · COL-05-corrige → ligne 1105</t>
         </is>
       </c>
     </row>
@@ -12899,7 +13014,7 @@
       </c>
       <c r="O106" s="53" t="inlineStr">
         <is>
-          <t>ADM-12 → ligne 547</t>
+          <t>ADM-12 → ligne 547 · ADM-12-corrige → ligne 575</t>
         </is>
       </c>
     </row>
@@ -13011,15 +13126,19 @@
       </c>
       <c r="M108" s="55" t="inlineStr">
         <is>
-          <t>À retester</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="N108" s="33" t="inlineStr">
         <is>
-          <t>La page s'affichant de nouveau, l'export CSV est accessible : à rejouer.</t>
-        </is>
-      </c>
-      <c r="O108" s="33" t="n"/>
+          <t>Corrigé avec ADM-12 : l'export CSV produit les 10 comptes affichés (13 colonnes), filtres respectés. Vérifié le 15/10 au soir.</t>
+        </is>
+      </c>
+      <c r="O108" s="33" t="inlineStr">
+        <is>
+          <t>ADM-12-corrige → ligne 575</t>
+        </is>
+      </c>
     </row>
     <row r="109" ht="27" customHeight="1" s="31">
       <c r="A109" s="33" t="inlineStr">
@@ -14561,7 +14680,7 @@
       </c>
       <c r="N132" s="33" t="inlineStr">
         <is>
-          <t>Le 15/10, le compte administrateur principal cossi@bigfiveabidjan.com s'ouvre encore avec le mot de passe de démonstration publié dans le README. À changer immédiatement (jeanluc@ a déjà été changé).</t>
+          <t>Le 15/10, 6 comptes sur 7 acceptent encore le mot de passe de démonstration, dont l'administrateur principal cossi@bigfiveabidjan.com (seul jeanluc@ a été changé). Retiré du README le 15/10 ; script npm run auth:renouveler prêt, à lancer par Big Five (voir « En attente client », D2).</t>
         </is>
       </c>
       <c r="O132" s="33" t="n"/>
@@ -16619,7 +16738,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="30" customHeight="1" s="31">
       <c r="A4" s="32" t="inlineStr">
         <is>
@@ -19122,7 +19240,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="30" customHeight="1" s="31">
       <c r="A4" s="32" t="inlineStr">
         <is>
@@ -20983,7 +21100,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="32" t="inlineStr">
         <is>
@@ -22013,7 +22129,6 @@
       </c>
       <c r="G32" s="33" t="n"/>
     </row>
-    <row r="33"/>
     <row r="34" ht="45" customHeight="1" s="31">
       <c r="A34" s="43" t="inlineStr">
         <is>
@@ -22021,7 +22136,6 @@
         </is>
       </c>
     </row>
-    <row r="35"/>
     <row r="36">
       <c r="A36" s="58" t="inlineStr">
         <is>
@@ -22271,7 +22385,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="30" customHeight="1" s="31">
       <c r="A4" s="32" t="inlineStr">
         <is>
@@ -23587,7 +23700,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="30" customHeight="1" s="31">
       <c r="A4" s="32" t="inlineStr">
         <is>
@@ -25228,7 +25340,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="30" customHeight="1" s="31">
       <c r="A4" s="16" t="inlineStr">
         <is>
@@ -25464,7 +25575,6 @@
       </c>
       <c r="E12" s="33" t="n"/>
     </row>
-    <row r="13"/>
     <row r="14" ht="31.5" customHeight="1" s="31">
       <c r="A14" s="4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Finaliser le classeur et le compte rendu de recette du 15/10
Classeur : onglets Comptes et clés, Points manquants, Paiement FeexPay,
Couverture e-mail et Synthèse alignés sur l'état du soir (Mobile Money
validé en réel, Resend, Zoom, domaine définitif, migrations 37 et 38
à exécuter), en gardant les vérifications D1 à D3 de bb2ac36.
Compte rendu : réécrit pour Big Five, utilisable tel quel comme
e-mail, avec D1 à D3 en annexe technique.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Recette E-Masterclass BigFive — clôture 15-10.xlsx
+++ b/Recette E-Masterclass BigFive — clôture 15-10.xlsx
@@ -2293,28 +2293,28 @@
     <row r="39" ht="27.75" customHeight="1" s="31">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>• FeexPay — Orange, MTN et Moov ouverts en live, webhook opérationnel (paiement MTN réel du 15/10 refusé par MTN pour solde ou plafond, et tracé). Wave : Clé agrégée Wave à activer (C14). Carte : KYC carte en brouillon (C1) — actions Big Five.</t>
+          <t>• FeexPay — Mobile Money validé en réel le 15/10 : Orange et MTN à 200 F réussis, modules ouverts, webhook opérationnel. Wave : Clé agrégée Wave à activer (C14). Carte : KYC carte en brouillon (C1) — actions Big Five.</t>
         </is>
       </c>
     </row>
     <row r="40" ht="27.75" customHeight="1" s="31">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>• Envoi d'e-mails — aucun pilote réel : mot de passe oublié, confirmation d'achat, attestation et avis d'annulation ne partent pas.</t>
+          <t>• E-mails — Resend en service depuis le 15/10 (réinitialisation délivrée, avis d'annulation envoyé). Confirmation d'achat et attestation : écrites et fusionnées, à vérifier après déploiement. Un seul DMARC à garder (C3).</t>
         </is>
       </c>
     </row>
     <row r="41" ht="27.75" customHeight="1" s="31">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>• Vidéos — 15 chapitres rattachés sur 72 dans la base en ligne.</t>
+          <t>• Vidéos — 15 chapitres rattachés sur 72 dans la base en ligne ; lecture vérifiée sur le domaine définitif (Worker vidéo autorisé le 15/10).</t>
         </is>
       </c>
     </row>
     <row r="42" ht="27.75" customHeight="1" s="31">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>• Zoom — réglé le 15/10 (app activée, clés posées, mode live) ; reste le test réel de bout en bout (Z6 à Z9).</t>
+          <t>• Zoom — en réel depuis le 15/10 : la session ses-010 a créé sa réunion chez Zoom ; reste l'entrée en salle, le report et l'annulation (Z7 à Z9).</t>
         </is>
       </c>
     </row>
@@ -3456,7 +3456,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="B4" s="59" t="inlineStr">
         <is>
@@ -3471,37 +3470,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
-    <row r="7"/>
-    <row r="8"/>
-    <row r="9"/>
-    <row r="10"/>
-    <row r="11"/>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
     <row r="37">
       <c r="B37" s="59" t="inlineStr">
         <is>
@@ -3516,33 +3484,6 @@
         </is>
       </c>
     </row>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
     <row r="66">
       <c r="B66" s="59" t="inlineStr">
         <is>
@@ -3557,33 +3498,6 @@
         </is>
       </c>
     </row>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="94"/>
     <row r="95">
       <c r="B95" s="59" t="inlineStr">
         <is>
@@ -3598,36 +3512,6 @@
         </is>
       </c>
     </row>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
-    <row r="109"/>
-    <row r="110"/>
-    <row r="111"/>
-    <row r="112"/>
-    <row r="113"/>
-    <row r="114"/>
-    <row r="115"/>
-    <row r="116"/>
-    <row r="117"/>
-    <row r="118"/>
-    <row r="119"/>
-    <row r="120"/>
-    <row r="121"/>
-    <row r="122"/>
-    <row r="123"/>
-    <row r="124"/>
-    <row r="125"/>
-    <row r="126"/>
     <row r="127">
       <c r="B127" s="59" t="inlineStr">
         <is>
@@ -3642,32 +3526,6 @@
         </is>
       </c>
     </row>
-    <row r="129"/>
-    <row r="130"/>
-    <row r="131"/>
-    <row r="132"/>
-    <row r="133"/>
-    <row r="134"/>
-    <row r="135"/>
-    <row r="136"/>
-    <row r="137"/>
-    <row r="138"/>
-    <row r="139"/>
-    <row r="140"/>
-    <row r="141"/>
-    <row r="142"/>
-    <row r="143"/>
-    <row r="144"/>
-    <row r="145"/>
-    <row r="146"/>
-    <row r="147"/>
-    <row r="148"/>
-    <row r="149"/>
-    <row r="150"/>
-    <row r="151"/>
-    <row r="152"/>
-    <row r="153"/>
-    <row r="154"/>
     <row r="155">
       <c r="B155" s="59" t="inlineStr">
         <is>
@@ -3682,33 +3540,6 @@
         </is>
       </c>
     </row>
-    <row r="157"/>
-    <row r="158"/>
-    <row r="159"/>
-    <row r="160"/>
-    <row r="161"/>
-    <row r="162"/>
-    <row r="163"/>
-    <row r="164"/>
-    <row r="165"/>
-    <row r="166"/>
-    <row r="167"/>
-    <row r="168"/>
-    <row r="169"/>
-    <row r="170"/>
-    <row r="171"/>
-    <row r="172"/>
-    <row r="173"/>
-    <row r="174"/>
-    <row r="175"/>
-    <row r="176"/>
-    <row r="177"/>
-    <row r="178"/>
-    <row r="179"/>
-    <row r="180"/>
-    <row r="181"/>
-    <row r="182"/>
-    <row r="183"/>
     <row r="184">
       <c r="B184" s="59" t="inlineStr">
         <is>
@@ -3723,63 +3554,6 @@
         </is>
       </c>
     </row>
-    <row r="186"/>
-    <row r="187"/>
-    <row r="188"/>
-    <row r="189"/>
-    <row r="190"/>
-    <row r="191"/>
-    <row r="192"/>
-    <row r="193"/>
-    <row r="194"/>
-    <row r="195"/>
-    <row r="196"/>
-    <row r="197"/>
-    <row r="198"/>
-    <row r="199"/>
-    <row r="200"/>
-    <row r="201"/>
-    <row r="202"/>
-    <row r="203"/>
-    <row r="204"/>
-    <row r="205"/>
-    <row r="206"/>
-    <row r="207"/>
-    <row r="208"/>
-    <row r="209"/>
-    <row r="210"/>
-    <row r="211"/>
-    <row r="212"/>
-    <row r="213"/>
-    <row r="214"/>
-    <row r="215"/>
-    <row r="216"/>
-    <row r="217"/>
-    <row r="218"/>
-    <row r="219"/>
-    <row r="220"/>
-    <row r="221"/>
-    <row r="222"/>
-    <row r="223"/>
-    <row r="224"/>
-    <row r="225"/>
-    <row r="226"/>
-    <row r="227"/>
-    <row r="228"/>
-    <row r="229"/>
-    <row r="230"/>
-    <row r="231"/>
-    <row r="232"/>
-    <row r="233"/>
-    <row r="234"/>
-    <row r="235"/>
-    <row r="236"/>
-    <row r="237"/>
-    <row r="238"/>
-    <row r="239"/>
-    <row r="240"/>
-    <row r="241"/>
-    <row r="242"/>
     <row r="243">
       <c r="B243" s="59" t="inlineStr">
         <is>
@@ -3787,34 +3561,6 @@
         </is>
       </c>
     </row>
-    <row r="244"/>
-    <row r="245"/>
-    <row r="246"/>
-    <row r="247"/>
-    <row r="248"/>
-    <row r="249"/>
-    <row r="250"/>
-    <row r="251"/>
-    <row r="252"/>
-    <row r="253"/>
-    <row r="254"/>
-    <row r="255"/>
-    <row r="256"/>
-    <row r="257"/>
-    <row r="258"/>
-    <row r="259"/>
-    <row r="260"/>
-    <row r="261"/>
-    <row r="262"/>
-    <row r="263"/>
-    <row r="264"/>
-    <row r="265"/>
-    <row r="266"/>
-    <row r="267"/>
-    <row r="268"/>
-    <row r="269"/>
-    <row r="270"/>
-    <row r="271"/>
     <row r="272">
       <c r="B272" s="59" t="inlineStr">
         <is>
@@ -3829,38 +3575,6 @@
         </is>
       </c>
     </row>
-    <row r="274"/>
-    <row r="275"/>
-    <row r="276"/>
-    <row r="277"/>
-    <row r="278"/>
-    <row r="279"/>
-    <row r="280"/>
-    <row r="281"/>
-    <row r="282"/>
-    <row r="283"/>
-    <row r="284"/>
-    <row r="285"/>
-    <row r="286"/>
-    <row r="287"/>
-    <row r="288"/>
-    <row r="289"/>
-    <row r="290"/>
-    <row r="291"/>
-    <row r="292"/>
-    <row r="293"/>
-    <row r="294"/>
-    <row r="295"/>
-    <row r="296"/>
-    <row r="297"/>
-    <row r="298"/>
-    <row r="299"/>
-    <row r="300"/>
-    <row r="301"/>
-    <row r="302"/>
-    <row r="303"/>
-    <row r="304"/>
-    <row r="305"/>
     <row r="306">
       <c r="B306" s="59" t="inlineStr">
         <is>
@@ -3875,38 +3589,6 @@
         </is>
       </c>
     </row>
-    <row r="308"/>
-    <row r="309"/>
-    <row r="310"/>
-    <row r="311"/>
-    <row r="312"/>
-    <row r="313"/>
-    <row r="314"/>
-    <row r="315"/>
-    <row r="316"/>
-    <row r="317"/>
-    <row r="318"/>
-    <row r="319"/>
-    <row r="320"/>
-    <row r="321"/>
-    <row r="322"/>
-    <row r="323"/>
-    <row r="324"/>
-    <row r="325"/>
-    <row r="326"/>
-    <row r="327"/>
-    <row r="328"/>
-    <row r="329"/>
-    <row r="330"/>
-    <row r="331"/>
-    <row r="332"/>
-    <row r="333"/>
-    <row r="334"/>
-    <row r="335"/>
-    <row r="336"/>
-    <row r="337"/>
-    <row r="338"/>
-    <row r="339"/>
     <row r="340">
       <c r="B340" s="59" t="inlineStr">
         <is>
@@ -3921,42 +3603,6 @@
         </is>
       </c>
     </row>
-    <row r="342"/>
-    <row r="343"/>
-    <row r="344"/>
-    <row r="345"/>
-    <row r="346"/>
-    <row r="347"/>
-    <row r="348"/>
-    <row r="349"/>
-    <row r="350"/>
-    <row r="351"/>
-    <row r="352"/>
-    <row r="353"/>
-    <row r="354"/>
-    <row r="355"/>
-    <row r="356"/>
-    <row r="357"/>
-    <row r="358"/>
-    <row r="359"/>
-    <row r="360"/>
-    <row r="361"/>
-    <row r="362"/>
-    <row r="363"/>
-    <row r="364"/>
-    <row r="365"/>
-    <row r="366"/>
-    <row r="367"/>
-    <row r="368"/>
-    <row r="369"/>
-    <row r="370"/>
-    <row r="371"/>
-    <row r="372"/>
-    <row r="373"/>
-    <row r="374"/>
-    <row r="375"/>
-    <row r="376"/>
-    <row r="377"/>
     <row r="378">
       <c r="B378" s="59" t="inlineStr">
         <is>
@@ -3971,40 +3617,6 @@
         </is>
       </c>
     </row>
-    <row r="380"/>
-    <row r="381"/>
-    <row r="382"/>
-    <row r="383"/>
-    <row r="384"/>
-    <row r="385"/>
-    <row r="386"/>
-    <row r="387"/>
-    <row r="388"/>
-    <row r="389"/>
-    <row r="390"/>
-    <row r="391"/>
-    <row r="392"/>
-    <row r="393"/>
-    <row r="394"/>
-    <row r="395"/>
-    <row r="396"/>
-    <row r="397"/>
-    <row r="398"/>
-    <row r="399"/>
-    <row r="400"/>
-    <row r="401"/>
-    <row r="402"/>
-    <row r="403"/>
-    <row r="404"/>
-    <row r="405"/>
-    <row r="406"/>
-    <row r="407"/>
-    <row r="408"/>
-    <row r="409"/>
-    <row r="410"/>
-    <row r="411"/>
-    <row r="412"/>
-    <row r="413"/>
     <row r="414">
       <c r="B414" s="59" t="inlineStr">
         <is>
@@ -4019,42 +3631,6 @@
         </is>
       </c>
     </row>
-    <row r="416"/>
-    <row r="417"/>
-    <row r="418"/>
-    <row r="419"/>
-    <row r="420"/>
-    <row r="421"/>
-    <row r="422"/>
-    <row r="423"/>
-    <row r="424"/>
-    <row r="425"/>
-    <row r="426"/>
-    <row r="427"/>
-    <row r="428"/>
-    <row r="429"/>
-    <row r="430"/>
-    <row r="431"/>
-    <row r="432"/>
-    <row r="433"/>
-    <row r="434"/>
-    <row r="435"/>
-    <row r="436"/>
-    <row r="437"/>
-    <row r="438"/>
-    <row r="439"/>
-    <row r="440"/>
-    <row r="441"/>
-    <row r="442"/>
-    <row r="443"/>
-    <row r="444"/>
-    <row r="445"/>
-    <row r="446"/>
-    <row r="447"/>
-    <row r="448"/>
-    <row r="449"/>
-    <row r="450"/>
-    <row r="451"/>
     <row r="452">
       <c r="B452" s="59" t="inlineStr">
         <is>
@@ -4069,43 +3645,6 @@
         </is>
       </c>
     </row>
-    <row r="454"/>
-    <row r="455"/>
-    <row r="456"/>
-    <row r="457"/>
-    <row r="458"/>
-    <row r="459"/>
-    <row r="460"/>
-    <row r="461"/>
-    <row r="462"/>
-    <row r="463"/>
-    <row r="464"/>
-    <row r="465"/>
-    <row r="466"/>
-    <row r="467"/>
-    <row r="468"/>
-    <row r="469"/>
-    <row r="470"/>
-    <row r="471"/>
-    <row r="472"/>
-    <row r="473"/>
-    <row r="474"/>
-    <row r="475"/>
-    <row r="476"/>
-    <row r="477"/>
-    <row r="478"/>
-    <row r="479"/>
-    <row r="480"/>
-    <row r="481"/>
-    <row r="482"/>
-    <row r="483"/>
-    <row r="484"/>
-    <row r="485"/>
-    <row r="486"/>
-    <row r="487"/>
-    <row r="488"/>
-    <row r="489"/>
-    <row r="490"/>
     <row r="491">
       <c r="B491" s="59" t="inlineStr">
         <is>
@@ -4120,32 +3659,6 @@
         </is>
       </c>
     </row>
-    <row r="493"/>
-    <row r="494"/>
-    <row r="495"/>
-    <row r="496"/>
-    <row r="497"/>
-    <row r="498"/>
-    <row r="499"/>
-    <row r="500"/>
-    <row r="501"/>
-    <row r="502"/>
-    <row r="503"/>
-    <row r="504"/>
-    <row r="505"/>
-    <row r="506"/>
-    <row r="507"/>
-    <row r="508"/>
-    <row r="509"/>
-    <row r="510"/>
-    <row r="511"/>
-    <row r="512"/>
-    <row r="513"/>
-    <row r="514"/>
-    <row r="515"/>
-    <row r="516"/>
-    <row r="517"/>
-    <row r="518"/>
     <row r="519">
       <c r="B519" s="59" t="inlineStr">
         <is>
@@ -4160,32 +3673,6 @@
         </is>
       </c>
     </row>
-    <row r="521"/>
-    <row r="522"/>
-    <row r="523"/>
-    <row r="524"/>
-    <row r="525"/>
-    <row r="526"/>
-    <row r="527"/>
-    <row r="528"/>
-    <row r="529"/>
-    <row r="530"/>
-    <row r="531"/>
-    <row r="532"/>
-    <row r="533"/>
-    <row r="534"/>
-    <row r="535"/>
-    <row r="536"/>
-    <row r="537"/>
-    <row r="538"/>
-    <row r="539"/>
-    <row r="540"/>
-    <row r="541"/>
-    <row r="542"/>
-    <row r="543"/>
-    <row r="544"/>
-    <row r="545"/>
-    <row r="546"/>
     <row r="547">
       <c r="B547" s="59" t="inlineStr">
         <is>
@@ -4200,32 +3687,6 @@
         </is>
       </c>
     </row>
-    <row r="549"/>
-    <row r="550"/>
-    <row r="551"/>
-    <row r="552"/>
-    <row r="553"/>
-    <row r="554"/>
-    <row r="555"/>
-    <row r="556"/>
-    <row r="557"/>
-    <row r="558"/>
-    <row r="559"/>
-    <row r="560"/>
-    <row r="561"/>
-    <row r="562"/>
-    <row r="563"/>
-    <row r="564"/>
-    <row r="565"/>
-    <row r="566"/>
-    <row r="567"/>
-    <row r="568"/>
-    <row r="569"/>
-    <row r="570"/>
-    <row r="571"/>
-    <row r="572"/>
-    <row r="573"/>
-    <row r="574"/>
     <row r="575">
       <c r="B575" s="59" t="inlineStr">
         <is>
@@ -4233,32 +3694,6 @@
         </is>
       </c>
     </row>
-    <row r="576"/>
-    <row r="577"/>
-    <row r="578"/>
-    <row r="579"/>
-    <row r="580"/>
-    <row r="581"/>
-    <row r="582"/>
-    <row r="583"/>
-    <row r="584"/>
-    <row r="585"/>
-    <row r="586"/>
-    <row r="587"/>
-    <row r="588"/>
-    <row r="589"/>
-    <row r="590"/>
-    <row r="591"/>
-    <row r="592"/>
-    <row r="593"/>
-    <row r="594"/>
-    <row r="595"/>
-    <row r="596"/>
-    <row r="597"/>
-    <row r="598"/>
-    <row r="599"/>
-    <row r="600"/>
-    <row r="601"/>
     <row r="602">
       <c r="B602" s="59" t="inlineStr">
         <is>
@@ -4273,85 +3708,6 @@
         </is>
       </c>
     </row>
-    <row r="604"/>
-    <row r="605"/>
-    <row r="606"/>
-    <row r="607"/>
-    <row r="608"/>
-    <row r="609"/>
-    <row r="610"/>
-    <row r="611"/>
-    <row r="612"/>
-    <row r="613"/>
-    <row r="614"/>
-    <row r="615"/>
-    <row r="616"/>
-    <row r="617"/>
-    <row r="618"/>
-    <row r="619"/>
-    <row r="620"/>
-    <row r="621"/>
-    <row r="622"/>
-    <row r="623"/>
-    <row r="624"/>
-    <row r="625"/>
-    <row r="626"/>
-    <row r="627"/>
-    <row r="628"/>
-    <row r="629"/>
-    <row r="630"/>
-    <row r="631"/>
-    <row r="632"/>
-    <row r="633"/>
-    <row r="634"/>
-    <row r="635"/>
-    <row r="636"/>
-    <row r="637"/>
-    <row r="638"/>
-    <row r="639"/>
-    <row r="640"/>
-    <row r="641"/>
-    <row r="642"/>
-    <row r="643"/>
-    <row r="644"/>
-    <row r="645"/>
-    <row r="646"/>
-    <row r="647"/>
-    <row r="648"/>
-    <row r="649"/>
-    <row r="650"/>
-    <row r="651"/>
-    <row r="652"/>
-    <row r="653"/>
-    <row r="654"/>
-    <row r="655"/>
-    <row r="656"/>
-    <row r="657"/>
-    <row r="658"/>
-    <row r="659"/>
-    <row r="660"/>
-    <row r="661"/>
-    <row r="662"/>
-    <row r="663"/>
-    <row r="664"/>
-    <row r="665"/>
-    <row r="666"/>
-    <row r="667"/>
-    <row r="668"/>
-    <row r="669"/>
-    <row r="670"/>
-    <row r="671"/>
-    <row r="672"/>
-    <row r="673"/>
-    <row r="674"/>
-    <row r="675"/>
-    <row r="676"/>
-    <row r="677"/>
-    <row r="678"/>
-    <row r="679"/>
-    <row r="680"/>
-    <row r="681"/>
-    <row r="682"/>
     <row r="683">
       <c r="B683" s="59" t="inlineStr">
         <is>
@@ -4366,32 +3722,6 @@
         </is>
       </c>
     </row>
-    <row r="685"/>
-    <row r="686"/>
-    <row r="687"/>
-    <row r="688"/>
-    <row r="689"/>
-    <row r="690"/>
-    <row r="691"/>
-    <row r="692"/>
-    <row r="693"/>
-    <row r="694"/>
-    <row r="695"/>
-    <row r="696"/>
-    <row r="697"/>
-    <row r="698"/>
-    <row r="699"/>
-    <row r="700"/>
-    <row r="701"/>
-    <row r="702"/>
-    <row r="703"/>
-    <row r="704"/>
-    <row r="705"/>
-    <row r="706"/>
-    <row r="707"/>
-    <row r="708"/>
-    <row r="709"/>
-    <row r="710"/>
     <row r="711">
       <c r="B711" s="59" t="inlineStr">
         <is>
@@ -4406,32 +3736,6 @@
         </is>
       </c>
     </row>
-    <row r="713"/>
-    <row r="714"/>
-    <row r="715"/>
-    <row r="716"/>
-    <row r="717"/>
-    <row r="718"/>
-    <row r="719"/>
-    <row r="720"/>
-    <row r="721"/>
-    <row r="722"/>
-    <row r="723"/>
-    <row r="724"/>
-    <row r="725"/>
-    <row r="726"/>
-    <row r="727"/>
-    <row r="728"/>
-    <row r="729"/>
-    <row r="730"/>
-    <row r="731"/>
-    <row r="732"/>
-    <row r="733"/>
-    <row r="734"/>
-    <row r="735"/>
-    <row r="736"/>
-    <row r="737"/>
-    <row r="738"/>
     <row r="739">
       <c r="B739" s="59" t="inlineStr">
         <is>
@@ -4446,46 +3750,6 @@
         </is>
       </c>
     </row>
-    <row r="741"/>
-    <row r="742"/>
-    <row r="743"/>
-    <row r="744"/>
-    <row r="745"/>
-    <row r="746"/>
-    <row r="747"/>
-    <row r="748"/>
-    <row r="749"/>
-    <row r="750"/>
-    <row r="751"/>
-    <row r="752"/>
-    <row r="753"/>
-    <row r="754"/>
-    <row r="755"/>
-    <row r="756"/>
-    <row r="757"/>
-    <row r="758"/>
-    <row r="759"/>
-    <row r="760"/>
-    <row r="761"/>
-    <row r="762"/>
-    <row r="763"/>
-    <row r="764"/>
-    <row r="765"/>
-    <row r="766"/>
-    <row r="767"/>
-    <row r="768"/>
-    <row r="769"/>
-    <row r="770"/>
-    <row r="771"/>
-    <row r="772"/>
-    <row r="773"/>
-    <row r="774"/>
-    <row r="775"/>
-    <row r="776"/>
-    <row r="777"/>
-    <row r="778"/>
-    <row r="779"/>
-    <row r="780"/>
     <row r="781">
       <c r="B781" s="59" t="inlineStr">
         <is>
@@ -4500,32 +3764,6 @@
         </is>
       </c>
     </row>
-    <row r="783"/>
-    <row r="784"/>
-    <row r="785"/>
-    <row r="786"/>
-    <row r="787"/>
-    <row r="788"/>
-    <row r="789"/>
-    <row r="790"/>
-    <row r="791"/>
-    <row r="792"/>
-    <row r="793"/>
-    <row r="794"/>
-    <row r="795"/>
-    <row r="796"/>
-    <row r="797"/>
-    <row r="798"/>
-    <row r="799"/>
-    <row r="800"/>
-    <row r="801"/>
-    <row r="802"/>
-    <row r="803"/>
-    <row r="804"/>
-    <row r="805"/>
-    <row r="806"/>
-    <row r="807"/>
-    <row r="808"/>
     <row r="809">
       <c r="B809" s="59" t="inlineStr">
         <is>
@@ -4540,32 +3778,6 @@
         </is>
       </c>
     </row>
-    <row r="811"/>
-    <row r="812"/>
-    <row r="813"/>
-    <row r="814"/>
-    <row r="815"/>
-    <row r="816"/>
-    <row r="817"/>
-    <row r="818"/>
-    <row r="819"/>
-    <row r="820"/>
-    <row r="821"/>
-    <row r="822"/>
-    <row r="823"/>
-    <row r="824"/>
-    <row r="825"/>
-    <row r="826"/>
-    <row r="827"/>
-    <row r="828"/>
-    <row r="829"/>
-    <row r="830"/>
-    <row r="831"/>
-    <row r="832"/>
-    <row r="833"/>
-    <row r="834"/>
-    <row r="835"/>
-    <row r="836"/>
     <row r="837">
       <c r="B837" s="59" t="inlineStr">
         <is>
@@ -4580,32 +3792,6 @@
         </is>
       </c>
     </row>
-    <row r="839"/>
-    <row r="840"/>
-    <row r="841"/>
-    <row r="842"/>
-    <row r="843"/>
-    <row r="844"/>
-    <row r="845"/>
-    <row r="846"/>
-    <row r="847"/>
-    <row r="848"/>
-    <row r="849"/>
-    <row r="850"/>
-    <row r="851"/>
-    <row r="852"/>
-    <row r="853"/>
-    <row r="854"/>
-    <row r="855"/>
-    <row r="856"/>
-    <row r="857"/>
-    <row r="858"/>
-    <row r="859"/>
-    <row r="860"/>
-    <row r="861"/>
-    <row r="862"/>
-    <row r="863"/>
-    <row r="864"/>
     <row r="865">
       <c r="B865" s="59" t="inlineStr">
         <is>
@@ -4620,91 +3806,6 @@
         </is>
       </c>
     </row>
-    <row r="867"/>
-    <row r="868"/>
-    <row r="869"/>
-    <row r="870"/>
-    <row r="871"/>
-    <row r="872"/>
-    <row r="873"/>
-    <row r="874"/>
-    <row r="875"/>
-    <row r="876"/>
-    <row r="877"/>
-    <row r="878"/>
-    <row r="879"/>
-    <row r="880"/>
-    <row r="881"/>
-    <row r="882"/>
-    <row r="883"/>
-    <row r="884"/>
-    <row r="885"/>
-    <row r="886"/>
-    <row r="887"/>
-    <row r="888"/>
-    <row r="889"/>
-    <row r="890"/>
-    <row r="891"/>
-    <row r="892"/>
-    <row r="893"/>
-    <row r="894"/>
-    <row r="895"/>
-    <row r="896"/>
-    <row r="897"/>
-    <row r="898"/>
-    <row r="899"/>
-    <row r="900"/>
-    <row r="901"/>
-    <row r="902"/>
-    <row r="903"/>
-    <row r="904"/>
-    <row r="905"/>
-    <row r="906"/>
-    <row r="907"/>
-    <row r="908"/>
-    <row r="909"/>
-    <row r="910"/>
-    <row r="911"/>
-    <row r="912"/>
-    <row r="913"/>
-    <row r="914"/>
-    <row r="915"/>
-    <row r="916"/>
-    <row r="917"/>
-    <row r="918"/>
-    <row r="919"/>
-    <row r="920"/>
-    <row r="921"/>
-    <row r="922"/>
-    <row r="923"/>
-    <row r="924"/>
-    <row r="925"/>
-    <row r="926"/>
-    <row r="927"/>
-    <row r="928"/>
-    <row r="929"/>
-    <row r="930"/>
-    <row r="931"/>
-    <row r="932"/>
-    <row r="933"/>
-    <row r="934"/>
-    <row r="935"/>
-    <row r="936"/>
-    <row r="937"/>
-    <row r="938"/>
-    <row r="939"/>
-    <row r="940"/>
-    <row r="941"/>
-    <row r="942"/>
-    <row r="943"/>
-    <row r="944"/>
-    <row r="945"/>
-    <row r="946"/>
-    <row r="947"/>
-    <row r="948"/>
-    <row r="949"/>
-    <row r="950"/>
-    <row r="951"/>
     <row r="952">
       <c r="B952" s="59" t="inlineStr">
         <is>
@@ -4719,69 +3820,6 @@
         </is>
       </c>
     </row>
-    <row r="954"/>
-    <row r="955"/>
-    <row r="956"/>
-    <row r="957"/>
-    <row r="958"/>
-    <row r="959"/>
-    <row r="960"/>
-    <row r="961"/>
-    <row r="962"/>
-    <row r="963"/>
-    <row r="964"/>
-    <row r="965"/>
-    <row r="966"/>
-    <row r="967"/>
-    <row r="968"/>
-    <row r="969"/>
-    <row r="970"/>
-    <row r="971"/>
-    <row r="972"/>
-    <row r="973"/>
-    <row r="974"/>
-    <row r="975"/>
-    <row r="976"/>
-    <row r="977"/>
-    <row r="978"/>
-    <row r="979"/>
-    <row r="980"/>
-    <row r="981"/>
-    <row r="982"/>
-    <row r="983"/>
-    <row r="984"/>
-    <row r="985"/>
-    <row r="986"/>
-    <row r="987"/>
-    <row r="988"/>
-    <row r="989"/>
-    <row r="990"/>
-    <row r="991"/>
-    <row r="992"/>
-    <row r="993"/>
-    <row r="994"/>
-    <row r="995"/>
-    <row r="996"/>
-    <row r="997"/>
-    <row r="998"/>
-    <row r="999"/>
-    <row r="1000"/>
-    <row r="1001"/>
-    <row r="1002"/>
-    <row r="1003"/>
-    <row r="1004"/>
-    <row r="1005"/>
-    <row r="1006"/>
-    <row r="1007"/>
-    <row r="1008"/>
-    <row r="1009"/>
-    <row r="1010"/>
-    <row r="1011"/>
-    <row r="1012"/>
-    <row r="1013"/>
-    <row r="1014"/>
-    <row r="1015"/>
-    <row r="1016"/>
     <row r="1017">
       <c r="B1017" s="59" t="inlineStr">
         <is>
@@ -4796,32 +3834,6 @@
         </is>
       </c>
     </row>
-    <row r="1019"/>
-    <row r="1020"/>
-    <row r="1021"/>
-    <row r="1022"/>
-    <row r="1023"/>
-    <row r="1024"/>
-    <row r="1025"/>
-    <row r="1026"/>
-    <row r="1027"/>
-    <row r="1028"/>
-    <row r="1029"/>
-    <row r="1030"/>
-    <row r="1031"/>
-    <row r="1032"/>
-    <row r="1033"/>
-    <row r="1034"/>
-    <row r="1035"/>
-    <row r="1036"/>
-    <row r="1037"/>
-    <row r="1038"/>
-    <row r="1039"/>
-    <row r="1040"/>
-    <row r="1041"/>
-    <row r="1042"/>
-    <row r="1043"/>
-    <row r="1044"/>
     <row r="1045">
       <c r="B1045" s="59" t="inlineStr">
         <is>
@@ -4836,36 +3848,6 @@
         </is>
       </c>
     </row>
-    <row r="1047"/>
-    <row r="1048"/>
-    <row r="1049"/>
-    <row r="1050"/>
-    <row r="1051"/>
-    <row r="1052"/>
-    <row r="1053"/>
-    <row r="1054"/>
-    <row r="1055"/>
-    <row r="1056"/>
-    <row r="1057"/>
-    <row r="1058"/>
-    <row r="1059"/>
-    <row r="1060"/>
-    <row r="1061"/>
-    <row r="1062"/>
-    <row r="1063"/>
-    <row r="1064"/>
-    <row r="1065"/>
-    <row r="1066"/>
-    <row r="1067"/>
-    <row r="1068"/>
-    <row r="1069"/>
-    <row r="1070"/>
-    <row r="1071"/>
-    <row r="1072"/>
-    <row r="1073"/>
-    <row r="1074"/>
-    <row r="1075"/>
-    <row r="1076"/>
     <row r="1077">
       <c r="B1077" s="59" t="inlineStr">
         <is>
@@ -4880,32 +3862,6 @@
         </is>
       </c>
     </row>
-    <row r="1079"/>
-    <row r="1080"/>
-    <row r="1081"/>
-    <row r="1082"/>
-    <row r="1083"/>
-    <row r="1084"/>
-    <row r="1085"/>
-    <row r="1086"/>
-    <row r="1087"/>
-    <row r="1088"/>
-    <row r="1089"/>
-    <row r="1090"/>
-    <row r="1091"/>
-    <row r="1092"/>
-    <row r="1093"/>
-    <row r="1094"/>
-    <row r="1095"/>
-    <row r="1096"/>
-    <row r="1097"/>
-    <row r="1098"/>
-    <row r="1099"/>
-    <row r="1100"/>
-    <row r="1101"/>
-    <row r="1102"/>
-    <row r="1103"/>
-    <row r="1104"/>
     <row r="1105">
       <c r="B1105" s="59" t="inlineStr">
         <is>
@@ -4913,36 +3869,6 @@
         </is>
       </c>
     </row>
-    <row r="1106"/>
-    <row r="1107"/>
-    <row r="1108"/>
-    <row r="1109"/>
-    <row r="1110"/>
-    <row r="1111"/>
-    <row r="1112"/>
-    <row r="1113"/>
-    <row r="1114"/>
-    <row r="1115"/>
-    <row r="1116"/>
-    <row r="1117"/>
-    <row r="1118"/>
-    <row r="1119"/>
-    <row r="1120"/>
-    <row r="1121"/>
-    <row r="1122"/>
-    <row r="1123"/>
-    <row r="1124"/>
-    <row r="1125"/>
-    <row r="1126"/>
-    <row r="1127"/>
-    <row r="1128"/>
-    <row r="1129"/>
-    <row r="1130"/>
-    <row r="1131"/>
-    <row r="1132"/>
-    <row r="1133"/>
-    <row r="1134"/>
-    <row r="1135"/>
     <row r="1136">
       <c r="B1136" s="59" t="inlineStr">
         <is>
@@ -4957,32 +3883,6 @@
         </is>
       </c>
     </row>
-    <row r="1138"/>
-    <row r="1139"/>
-    <row r="1140"/>
-    <row r="1141"/>
-    <row r="1142"/>
-    <row r="1143"/>
-    <row r="1144"/>
-    <row r="1145"/>
-    <row r="1146"/>
-    <row r="1147"/>
-    <row r="1148"/>
-    <row r="1149"/>
-    <row r="1150"/>
-    <row r="1151"/>
-    <row r="1152"/>
-    <row r="1153"/>
-    <row r="1154"/>
-    <row r="1155"/>
-    <row r="1156"/>
-    <row r="1157"/>
-    <row r="1158"/>
-    <row r="1159"/>
-    <row r="1160"/>
-    <row r="1161"/>
-    <row r="1162"/>
-    <row r="1163"/>
     <row r="1164">
       <c r="B1164" s="59" t="inlineStr">
         <is>
@@ -4997,32 +3897,6 @@
         </is>
       </c>
     </row>
-    <row r="1166"/>
-    <row r="1167"/>
-    <row r="1168"/>
-    <row r="1169"/>
-    <row r="1170"/>
-    <row r="1171"/>
-    <row r="1172"/>
-    <row r="1173"/>
-    <row r="1174"/>
-    <row r="1175"/>
-    <row r="1176"/>
-    <row r="1177"/>
-    <row r="1178"/>
-    <row r="1179"/>
-    <row r="1180"/>
-    <row r="1181"/>
-    <row r="1182"/>
-    <row r="1183"/>
-    <row r="1184"/>
-    <row r="1185"/>
-    <row r="1186"/>
-    <row r="1187"/>
-    <row r="1188"/>
-    <row r="1189"/>
-    <row r="1190"/>
-    <row r="1191"/>
     <row r="1192">
       <c r="B1192" s="59" t="inlineStr">
         <is>
@@ -5037,32 +3911,6 @@
         </is>
       </c>
     </row>
-    <row r="1194"/>
-    <row r="1195"/>
-    <row r="1196"/>
-    <row r="1197"/>
-    <row r="1198"/>
-    <row r="1199"/>
-    <row r="1200"/>
-    <row r="1201"/>
-    <row r="1202"/>
-    <row r="1203"/>
-    <row r="1204"/>
-    <row r="1205"/>
-    <row r="1206"/>
-    <row r="1207"/>
-    <row r="1208"/>
-    <row r="1209"/>
-    <row r="1210"/>
-    <row r="1211"/>
-    <row r="1212"/>
-    <row r="1213"/>
-    <row r="1214"/>
-    <row r="1215"/>
-    <row r="1216"/>
-    <row r="1217"/>
-    <row r="1218"/>
-    <row r="1219"/>
     <row r="1220">
       <c r="B1220" s="59" t="inlineStr">
         <is>
@@ -5077,32 +3925,6 @@
         </is>
       </c>
     </row>
-    <row r="1222"/>
-    <row r="1223"/>
-    <row r="1224"/>
-    <row r="1225"/>
-    <row r="1226"/>
-    <row r="1227"/>
-    <row r="1228"/>
-    <row r="1229"/>
-    <row r="1230"/>
-    <row r="1231"/>
-    <row r="1232"/>
-    <row r="1233"/>
-    <row r="1234"/>
-    <row r="1235"/>
-    <row r="1236"/>
-    <row r="1237"/>
-    <row r="1238"/>
-    <row r="1239"/>
-    <row r="1240"/>
-    <row r="1241"/>
-    <row r="1242"/>
-    <row r="1243"/>
-    <row r="1244"/>
-    <row r="1245"/>
-    <row r="1246"/>
-    <row r="1247"/>
     <row r="1248">
       <c r="B1248" s="59" t="inlineStr">
         <is>
@@ -5117,49 +3939,6 @@
         </is>
       </c>
     </row>
-    <row r="1250"/>
-    <row r="1251"/>
-    <row r="1252"/>
-    <row r="1253"/>
-    <row r="1254"/>
-    <row r="1255"/>
-    <row r="1256"/>
-    <row r="1257"/>
-    <row r="1258"/>
-    <row r="1259"/>
-    <row r="1260"/>
-    <row r="1261"/>
-    <row r="1262"/>
-    <row r="1263"/>
-    <row r="1264"/>
-    <row r="1265"/>
-    <row r="1266"/>
-    <row r="1267"/>
-    <row r="1268"/>
-    <row r="1269"/>
-    <row r="1270"/>
-    <row r="1271"/>
-    <row r="1272"/>
-    <row r="1273"/>
-    <row r="1274"/>
-    <row r="1275"/>
-    <row r="1276"/>
-    <row r="1277"/>
-    <row r="1278"/>
-    <row r="1279"/>
-    <row r="1280"/>
-    <row r="1281"/>
-    <row r="1282"/>
-    <row r="1283"/>
-    <row r="1284"/>
-    <row r="1285"/>
-    <row r="1286"/>
-    <row r="1287"/>
-    <row r="1288"/>
-    <row r="1289"/>
-    <row r="1290"/>
-    <row r="1291"/>
-    <row r="1292"/>
     <row r="1293">
       <c r="B1293" s="59" t="inlineStr">
         <is>
@@ -5174,32 +3953,6 @@
         </is>
       </c>
     </row>
-    <row r="1295"/>
-    <row r="1296"/>
-    <row r="1297"/>
-    <row r="1298"/>
-    <row r="1299"/>
-    <row r="1300"/>
-    <row r="1301"/>
-    <row r="1302"/>
-    <row r="1303"/>
-    <row r="1304"/>
-    <row r="1305"/>
-    <row r="1306"/>
-    <row r="1307"/>
-    <row r="1308"/>
-    <row r="1309"/>
-    <row r="1310"/>
-    <row r="1311"/>
-    <row r="1312"/>
-    <row r="1313"/>
-    <row r="1314"/>
-    <row r="1315"/>
-    <row r="1316"/>
-    <row r="1317"/>
-    <row r="1318"/>
-    <row r="1319"/>
-    <row r="1320"/>
     <row r="1321">
       <c r="B1321" s="59" t="inlineStr">
         <is>
@@ -5214,32 +3967,6 @@
         </is>
       </c>
     </row>
-    <row r="1323"/>
-    <row r="1324"/>
-    <row r="1325"/>
-    <row r="1326"/>
-    <row r="1327"/>
-    <row r="1328"/>
-    <row r="1329"/>
-    <row r="1330"/>
-    <row r="1331"/>
-    <row r="1332"/>
-    <row r="1333"/>
-    <row r="1334"/>
-    <row r="1335"/>
-    <row r="1336"/>
-    <row r="1337"/>
-    <row r="1338"/>
-    <row r="1339"/>
-    <row r="1340"/>
-    <row r="1341"/>
-    <row r="1342"/>
-    <row r="1343"/>
-    <row r="1344"/>
-    <row r="1345"/>
-    <row r="1346"/>
-    <row r="1347"/>
-    <row r="1348"/>
     <row r="1349">
       <c r="B1349" s="59" t="inlineStr">
         <is>
@@ -5254,32 +3981,6 @@
         </is>
       </c>
     </row>
-    <row r="1351"/>
-    <row r="1352"/>
-    <row r="1353"/>
-    <row r="1354"/>
-    <row r="1355"/>
-    <row r="1356"/>
-    <row r="1357"/>
-    <row r="1358"/>
-    <row r="1359"/>
-    <row r="1360"/>
-    <row r="1361"/>
-    <row r="1362"/>
-    <row r="1363"/>
-    <row r="1364"/>
-    <row r="1365"/>
-    <row r="1366"/>
-    <row r="1367"/>
-    <row r="1368"/>
-    <row r="1369"/>
-    <row r="1370"/>
-    <row r="1371"/>
-    <row r="1372"/>
-    <row r="1373"/>
-    <row r="1374"/>
-    <row r="1375"/>
-    <row r="1376"/>
     <row r="1377">
       <c r="B1377" s="59" t="inlineStr">
         <is>
@@ -16816,7 +15517,7 @@
       </c>
       <c r="H5" s="33" t="inlineStr">
         <is>
-          <t>Intégration faite — voir « Passage en production »</t>
+          <t>Live en service le 15/10 pour le Mobile Money ; Wave et carte à activer chez FeexPay</t>
         </is>
       </c>
     </row>
@@ -16841,7 +15542,7 @@
       </c>
       <c r="E6" s="23" t="inlineStr">
         <is>
-          <t>Oui</t>
+          <t>Non</t>
         </is>
       </c>
       <c r="F6" s="33" t="inlineStr">
@@ -16854,7 +15555,11 @@
           <t>3 à 5 jours</t>
         </is>
       </c>
-      <c r="H6" s="33" t="n"/>
+      <c r="H6" s="33" t="inlineStr">
+        <is>
+          <t>Fait le 15/10 (Resend) — garder un seul DMARC</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="39" t="n">
@@ -17033,7 +15738,7 @@
       </c>
       <c r="E11" s="23" t="inlineStr">
         <is>
-          <t>Oui</t>
+          <t>Non</t>
         </is>
       </c>
       <c r="F11" s="33" t="inlineStr">
@@ -17048,7 +15753,7 @@
       </c>
       <c r="H11" s="33" t="inlineStr">
         <is>
-          <t>Voir « Passage en production »</t>
+          <t>Fait le 15/10 (réunions créées automatiquement)</t>
         </is>
       </c>
     </row>
@@ -17382,7 +16087,11 @@
           <t>immédiat</t>
         </is>
       </c>
-      <c r="H20" s="33" t="n"/>
+      <c r="H20" s="33" t="inlineStr">
+        <is>
+          <t>Script prêt : npm run auth:renouveler -- --appliquer (à lancer par Big Five)</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="15.75" customHeight="1" s="31">
       <c r="A21" s="39" t="n">
@@ -17477,7 +16186,7 @@
       </c>
       <c r="E23" s="23" t="inlineStr">
         <is>
-          <t>Oui</t>
+          <t>Non</t>
         </is>
       </c>
       <c r="F23" s="33" t="inlineStr">
@@ -17490,7 +16199,11 @@
           <t>2 jours</t>
         </is>
       </c>
-      <c r="H23" s="33" t="n"/>
+      <c r="H23" s="33" t="inlineStr">
+        <is>
+          <t>Fait le 15/10 (pilote Resend)</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="15.75" customHeight="1" s="31">
       <c r="A24" s="39" t="n">
@@ -17528,7 +16241,7 @@
       </c>
       <c r="H24" s="33" t="inlineStr">
         <is>
-          <t>Partiel</t>
+          <t>Opérationnel (clé Bearer), vérifié en réel le 15/10</t>
         </is>
       </c>
     </row>
@@ -17566,7 +16279,11 @@
           <t>3 jours</t>
         </is>
       </c>
-      <c r="H25" s="33" t="n"/>
+      <c r="H25" s="33" t="inlineStr">
+        <is>
+          <t>Développé le 15/10 : relance quotidienne des commandes en attente (2bc3bcc)</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="15.75" customHeight="1" s="31">
       <c r="A26" s="39" t="n">
@@ -17604,7 +16321,7 @@
       </c>
       <c r="H26" s="33" t="inlineStr">
         <is>
-          <t>Fait — reste la configuration</t>
+          <t>Fait — réunions réelles depuis le 15/10</t>
         </is>
       </c>
     </row>
@@ -17749,7 +16466,7 @@
       </c>
       <c r="E30" s="23" t="inlineStr">
         <is>
-          <t>Oui</t>
+          <t>Non</t>
         </is>
       </c>
       <c r="F30" s="33" t="inlineStr">
@@ -17762,7 +16479,11 @@
           <t>1 jour</t>
         </is>
       </c>
-      <c r="H30" s="33" t="n"/>
+      <c r="H30" s="33" t="inlineStr">
+        <is>
+          <t>Fait le 15/10 : https://emasterclass.bigfive.solutions/</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="15.75" customHeight="1" s="31">
       <c r="A31" s="39" t="n">
@@ -17912,7 +16633,7 @@
       </c>
       <c r="H34" s="33" t="inlineStr">
         <is>
-          <t>Nouveau (15/10)</t>
+          <t>Corrigé le 15/10 : npm run typecheck sans erreur</t>
         </is>
       </c>
     </row>
@@ -17952,7 +16673,7 @@
       </c>
       <c r="H35" s="33" t="inlineStr">
         <is>
-          <t>Nouveau (15/10)</t>
+          <t>Migration 37 écrite, à exécuter sur la base hébergée</t>
         </is>
       </c>
     </row>
@@ -17992,7 +16713,7 @@
       </c>
       <c r="H36" s="33" t="inlineStr">
         <is>
-          <t>Nouveau (15/10)</t>
+          <t>Développé le 15/10, migration 38 à exécuter avant déploiement</t>
         </is>
       </c>
     </row>
@@ -18057,7 +16778,7 @@
       </c>
       <c r="E38" s="40" t="inlineStr">
         <is>
-          <t>Oui</t>
+          <t>Non</t>
         </is>
       </c>
       <c r="F38" s="33" t="inlineStr">
@@ -18072,7 +16793,7 @@
       </c>
       <c r="H38" s="33" t="inlineStr">
         <is>
-          <t>Nouveau (15/10) — preuve BLQ-ZOOM</t>
+          <t>Fait le 15/10</t>
         </is>
       </c>
     </row>
@@ -18112,7 +16833,7 @@
       </c>
       <c r="H39" s="33" t="inlineStr">
         <is>
-          <t>Nouveau (15/10)</t>
+          <t>Corrigé et vérifié le 15/10 (27d835b)</t>
         </is>
       </c>
     </row>
@@ -18192,7 +16913,7 @@
       </c>
       <c r="H41" s="33" t="inlineStr">
         <is>
-          <t>Nouveau (15/10)</t>
+          <t>Corrigé et vérifié le 15/10</t>
         </is>
       </c>
     </row>
@@ -18232,7 +16953,7 @@
       </c>
       <c r="H42" s="33" t="inlineStr">
         <is>
-          <t>Nouveau (15/10)</t>
+          <t>Mobile Money : rattachement par callback_info confirmé sur les paiements réels ; à vérifier sur un paiement carte</t>
         </is>
       </c>
     </row>
@@ -19313,7 +18034,7 @@
       </c>
       <c r="G5" s="23" t="inlineStr">
         <is>
-          <t>À fournir</t>
+          <t>En service (boutique « Big Five Abidjan »)</t>
         </is>
       </c>
       <c r="H5" s="33" t="n"/>
@@ -19385,7 +18106,7 @@
       </c>
       <c r="G7" s="23" t="inlineStr">
         <is>
-          <t>Fourni (test)</t>
+          <t>Fourni</t>
         </is>
       </c>
       <c r="H7" s="33" t="n"/>
@@ -19457,7 +18178,7 @@
       </c>
       <c r="G9" s="23" t="inlineStr">
         <is>
-          <t>À fournir</t>
+          <t>Fourni — en service (15/10)</t>
         </is>
       </c>
       <c r="H9" s="33" t="n"/>
@@ -19493,7 +18214,7 @@
       </c>
       <c r="G10" s="23" t="inlineStr">
         <is>
-          <t>Fourni (local) — à régénérer pour la production</t>
+          <t>Fait — clé de production posée le 15/10</t>
         </is>
       </c>
       <c r="H10" s="33" t="n"/>
@@ -19529,7 +18250,7 @@
       </c>
       <c r="G11" s="40" t="inlineStr">
         <is>
-          <t>À déclarer après la mise en ligne</t>
+          <t>Déclarée le 15/10 (en-tête Bearer)</t>
         </is>
       </c>
       <c r="H11" s="33" t="n"/>
@@ -19601,7 +18322,7 @@
       </c>
       <c r="G13" s="40" t="inlineStr">
         <is>
-          <t>À vérifier</t>
+          <t>Sans objet : la liste d’IP ne sert qu’aux reversements (Payout API)</t>
         </is>
       </c>
       <c r="H13" s="33" t="n"/>
@@ -19637,7 +18358,7 @@
       </c>
       <c r="G14" s="40" t="inlineStr">
         <is>
-          <t>Mobile Money et Wave ouverts ; carte refusée (KYC carte en brouillon, 15/10) : Visa et Djamo masqués</t>
+          <t>Orange, MTN et Moov ouverts ; Wave : Clé agrégée Wave à activer ; carte : KYC carte en brouillon</t>
         </is>
       </c>
       <c r="H14" s="33" t="n"/>
@@ -22435,7 +21156,7 @@
       </c>
       <c r="E5" s="33" t="inlineStr">
         <is>
-          <t>Migrations 01 à 05 appliquées et vérifiées le 02/09</t>
+          <t>Migrations 01 à 36 en place ; 37 (droits des clés publiques) et 38 (coaching privé dans Transactions) à exécuter dans SQL Editor avant le déploiement du 15/10 au soir</t>
         </is>
       </c>
     </row>
@@ -22462,7 +21183,7 @@
       </c>
       <c r="E6" s="33" t="inlineStr">
         <is>
-          <t>Vérifié le 02/09 : les démonstrations se lisent depuis le CDN, le cloisonnement des chapitres tient</t>
+          <t>Lecture vérifiée le 15/10 sur emasterclass.bigfive.solutions (origine ajoutée au Worker, redéployé)</t>
         </is>
       </c>
     </row>
@@ -22484,12 +21205,12 @@
       </c>
       <c r="D7" s="45" t="inlineStr">
         <is>
-          <t>À fournir — bloquant</t>
+          <t>Fourni — en service</t>
         </is>
       </c>
       <c r="E7" s="33" t="inlineStr">
         <is>
-          <t>Débloque réinitialisation, confirmation d'achat, envoi d'attestation, avis d'annulation. Aucun pilote d'envoi n'est encore codé : NOTIFICATIONS_DRIVER n'accepte que « console ».</t>
+          <t>Resend, domaine bigfive.solutions vérifié (DKIM, SPF), NOTIFICATIONS_DRIVER=resend depuis le 15/10. Deux enregistrements DMARC coexistent : n'en garder qu'un.</t>
         </is>
       </c>
     </row>
@@ -22538,12 +21259,12 @@
       </c>
       <c r="D9" s="45" t="inlineStr">
         <is>
-          <t>Sandbox en service — live à fournir</t>
+          <t>Live en service — Mobile Money</t>
         </is>
       </c>
       <c r="E9" s="33" t="inlineStr">
         <is>
-          <t>Intégration faite ; les clés live et le compte marchand manquent</t>
+          <t>Orange, MTN et Moov encaissent en réel (paiements de 200 F réussis le 15/10). Wave : Clé agrégée Wave à activer. Carte : KYC carte à faire valider.</t>
         </is>
       </c>
     </row>
@@ -22565,12 +21286,12 @@
       </c>
       <c r="D10" s="45" t="inlineStr">
         <is>
-          <t>À fournir — bloquant</t>
+          <t>Fourni — en service</t>
         </is>
       </c>
       <c r="E10" s="33" t="inlineStr">
         <is>
-          <t>Intégration faite, mode simulation ; les réunions se créent seules une fois les clés posées</t>
+          <t>ZOOM_MODE=live depuis le 15/10 : app Server-to-Server activée, Meeting SDK configuré, réunions créées automatiquement (ses-010).</t>
         </is>
       </c>
     </row>
@@ -22646,12 +21367,12 @@
       </c>
       <c r="D13" s="45" t="inlineStr">
         <is>
-          <t>À fournir — bloquant</t>
+          <t>Fourni — en service</t>
         </is>
       </c>
       <c r="E13" s="33" t="inlineStr">
         <is>
-          <t>NUXT_PUBLIC_SITE_URL alimente les canonical, le sitemap et le lien de vérification des attestations ; il pointe encore vers l'URL Vercel</t>
+          <t>URL définitive https://emasterclass.bigfive.solutions/ : CNAME Cloudflare vers Vercel, HTTPS, NUXT_PUBLIC_SITE_URL posé (15/10).</t>
         </is>
       </c>
     </row>
@@ -25390,7 +24111,7 @@
       </c>
       <c r="E5" s="33" t="inlineStr">
         <is>
-          <t>Parcours 01 et 02 : FeexPay et Zoom développés, en attente des clés de production</t>
+          <t>Parcours 01 : paiement Mobile Money validé en réel le 15/10. Parcours 02 : réunions Zoom créées automatiquement ; l'entrée en salle reste à tester.</t>
         </is>
       </c>
     </row>
@@ -25471,7 +24192,7 @@
       </c>
       <c r="E8" s="33" t="inlineStr">
         <is>
-          <t>La signature se dépose depuis l'administration (21/09) ; l'envoi par e-mail attend un pilote d'envoi réel</t>
+          <t>La signature se dépose depuis l'administration (21/09) ; l'e-mail d'attestation est écrit et fusionné le 15/10, à vérifier après déploiement.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Recette : mots de passe de démonstration renouvelés (SEC-11 OK)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Recette E-Masterclass BigFive — clôture 15-10.xlsx
+++ b/Recette E-Masterclass BigFive — clôture 15-10.xlsx
@@ -2328,7 +2328,7 @@
     <row r="44" ht="27.75" customHeight="1" s="31">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>• Mot de passe de démonstration commun encore actif sur 6 comptes sur 7 ; retiré du README le 15/10, script de renouvellement prêt (D2).</t>
+          <t>• Mots de passe de démonstration : renouvelés le 15/10 sur les 6 comptes concernés ; reste à remplacer NUXT_SESSION_PASSWORD sur Vercel et redéployer.</t>
         </is>
       </c>
     </row>
@@ -2356,7 +2356,7 @@
     <row r="48" ht="27.75" customHeight="1" s="31">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>• Le compte administrateur principal cossi@bigfiveabidjan.com s'ouvre encore avec le mot de passe de démonstration : lancer npm run auth:renouveler -- --appliquer (D2).</t>
+          <t>• Après le push : exécuter les migrations 37 et 38 (déjà prévu), puis vérifier en ligne les 9 cas « À retester ».</t>
         </is>
       </c>
     </row>
@@ -4035,6 +4035,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="48" t="inlineStr">
         <is>
@@ -4676,6 +4677,8 @@
         </is>
       </c>
     </row>
+    <row r="20"/>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="48" t="inlineStr">
         <is>
@@ -4776,12 +4779,12 @@
       </c>
       <c r="B25" s="49" t="inlineStr">
         <is>
-          <t>Mots de passe de démonstration encore actifs (dont l'administrateur principal)</t>
+          <t>Mots de passe de démonstration</t>
         </is>
       </c>
       <c r="C25" s="50" t="inlineStr">
         <is>
-          <t>Big Five (lancer le script)</t>
+          <t>Fait le 15/10</t>
         </is>
       </c>
       <c r="D25" s="50" t="inlineStr">
@@ -4791,7 +4794,7 @@
       </c>
       <c r="E25" s="50" t="inlineStr">
         <is>
-          <t>Lecture du 15/10 sur la base en ligne : 6 comptes sur 7 acceptent encore le mot de passe commun du jeu de données — cossi@, jeremie.declercq@, houefa@bigfiveabidjan.com, editeur@bigfive.ci, formateur@bigfive.ci, aya@example.ci. Seul jeanluc@ l'a changé.</t>
+          <t>Les 6 comptes qui acceptaient le mot de passe commun (cossi@, jeremie.declercq@, houefa@, editeur@, formateur@, aya@) ont été renouvelés ; contrôle en lecture seule : aucun ne l'accepte plus.</t>
         </is>
       </c>
       <c r="F25" s="50" t="inlineStr">
@@ -4801,7 +4804,7 @@
       </c>
       <c r="G25" s="50" t="inlineStr">
         <is>
-          <t>Mot de passe retiré du README et du TODO le 15/10. Script prêt : npm run auth:renouveler (lecture seule) puis npm run auth:renouveler -- --appliquer, qui tire un mot de passe aléatoire par compte et l'affiche une seule fois dans le terminal : le reporter dans un gestionnaire, le transmettre à son titulaire. Puis remplacer NUXT_SESSION_PASSWORD sur Vercel pour fermer les sessions ouvertes.</t>
+          <t>Transmettre chaque mot de passe à son titulaire, qui le change à sa première connexion. Remplacer NUXT_SESSION_PASSWORD sur Vercel et redéployer.</t>
         </is>
       </c>
       <c r="H25" s="50" t="inlineStr">
@@ -5105,6 +5108,8 @@
         </is>
       </c>
     </row>
+    <row r="33"/>
+    <row r="34"/>
     <row r="35">
       <c r="A35" s="48" t="inlineStr">
         <is>
@@ -13374,14 +13379,14 @@
           <t>Le mot de passe n'est plus affiché sur les écrans de connexion. Il reste écrit dans le README et c'est encore celui de tous les comptes du jeu de données : à changer avant ouverture.</t>
         </is>
       </c>
-      <c r="M132" s="56" t="inlineStr">
-        <is>
-          <t>KO</t>
+      <c r="M132" s="52" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="N132" s="33" t="inlineStr">
         <is>
-          <t>Le 15/10, 6 comptes sur 7 acceptent encore le mot de passe de démonstration, dont l'administrateur principal cossi@bigfiveabidjan.com (seul jeanluc@ a été changé). Retiré du README le 15/10 ; script npm run auth:renouveler prêt, à lancer par Big Five (voir « En attente client », D2).</t>
+          <t>Renouvelé le 15/10 au soir (npm run auth:renouveler -- --appliquer) : les 6 comptes concernés ont un mot de passe aléatoire de 24 caractères ; le contrôle en lecture seule confirme qu'aucun compte n'accepte plus le mot de passe de démonstration. Reste : remplacer NUXT_SESSION_PASSWORD sur Vercel et redéployer, pour fermer les sessions ouvertes.</t>
         </is>
       </c>
       <c r="O132" s="33" t="n"/>
@@ -16074,7 +16079,7 @@
       </c>
       <c r="E20" s="23" t="inlineStr">
         <is>
-          <t>Oui</t>
+          <t>Non</t>
         </is>
       </c>
       <c r="F20" s="33" t="inlineStr">
@@ -16089,7 +16094,7 @@
       </c>
       <c r="H20" s="33" t="inlineStr">
         <is>
-          <t>Script prêt : npm run auth:renouveler -- --appliquer (à lancer par Big Five)</t>
+          <t>Fait le 15/10 (6 comptes renouvelés)</t>
         </is>
       </c>
     </row>
@@ -16858,7 +16863,7 @@
       </c>
       <c r="E40" s="40" t="inlineStr">
         <is>
-          <t>Oui</t>
+          <t>Non</t>
         </is>
       </c>
       <c r="F40" s="33" t="inlineStr">
@@ -16873,7 +16878,7 @@
       </c>
       <c r="H40" s="33" t="inlineStr">
         <is>
-          <t>Nouveau (15/10)</t>
+          <t>Fait le 15/10 (renouvelé)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Recette : migrations 37 et 38 exécutées, derniers développements en ligne
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Recette E-Masterclass BigFive — clôture 15-10.xlsx
+++ b/Recette E-Masterclass BigFive — clôture 15-10.xlsx
@@ -2356,7 +2356,7 @@
     <row r="48" ht="27.75" customHeight="1" s="31">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>• Après le push : exécuter les migrations 37 et 38 (déjà prévu), puis vérifier en ligne les 9 cas « À retester ».</t>
+          <t>• Migrations 37 et 38 exécutées et code en ligne depuis le 15/10 au soir : reste à vérifier en ligne les cas « À retester ».</t>
         </is>
       </c>
     </row>
@@ -4911,7 +4911,7 @@
       </c>
       <c r="C28" s="50" t="inlineStr">
         <is>
-          <t>Développé (2bc3bcc)</t>
+          <t>En ligne (15/10)</t>
         </is>
       </c>
       <c r="D28" s="50" t="inlineStr">
@@ -4931,7 +4931,7 @@
       </c>
       <c r="G28" s="50" t="inlineStr">
         <is>
-          <t>Vérifier après déploiement.</t>
+          <t>Vérifier après la première exécution du cron (4 h).</t>
         </is>
       </c>
       <c r="H28" s="51" t="inlineStr">
@@ -4953,7 +4953,7 @@
       </c>
       <c r="C29" s="50" t="inlineStr">
         <is>
-          <t>Développé (2bc3bcc)</t>
+          <t>En ligne (15/10)</t>
         </is>
       </c>
       <c r="D29" s="50" t="inlineStr">
@@ -4973,7 +4973,7 @@
       </c>
       <c r="G29" s="50" t="inlineStr">
         <is>
-          <t>Exécuter la migration 38 sur la base hébergée avant de déployer.</t>
+          <t>Migration 38 exécutée ; vérifier sur un paiement de coaching privé.</t>
         </is>
       </c>
       <c r="H29" s="50" t="inlineStr">
@@ -5037,7 +5037,7 @@
       </c>
       <c r="C31" s="50" t="inlineStr">
         <is>
-          <t>Développé (2bc3bcc)</t>
+          <t>Fait (15/10)</t>
         </is>
       </c>
       <c r="D31" s="50" t="inlineStr">
@@ -5057,7 +5057,7 @@
       </c>
       <c r="G31" s="50" t="inlineStr">
         <is>
-          <t>Exécuter la migration 37 sur la base hébergée.</t>
+          <t>Migration 37 exécutée et vérifiée sur la base hébergée.</t>
         </is>
       </c>
       <c r="H31" s="50" t="inlineStr">
@@ -5079,7 +5079,7 @@
       </c>
       <c r="C32" s="50" t="inlineStr">
         <is>
-          <t>Fusionné dans main</t>
+          <t>En ligne (15/10)</t>
         </is>
       </c>
       <c r="D32" s="50" t="inlineStr">
@@ -5099,7 +5099,7 @@
       </c>
       <c r="G32" s="50" t="inlineStr">
         <is>
-          <t>Déployer, puis vérifier les deux e-mails sur un vrai achat et une vraie délivrance.</t>
+          <t>Vérifier sur le prochain achat réel et la prochaine attestation.</t>
         </is>
       </c>
       <c r="H32" s="50" t="inlineStr">
@@ -7618,7 +7618,7 @@
       </c>
       <c r="N38" s="33" t="inlineStr">
         <is>
-          <t>Développé le 15/10 : relance quotidienne des commandes restées en attente (cron Vercel 04:00, /api/taches/commandes), qui relit leur statut chez FeexPay. À vérifier après déploiement.</t>
+          <t>En ligne depuis le déploiement du 15/10 au soir : la route /api/taches/commandes répond (401 sans clé) et le cron Vercel la lance chaque nuit à 4 h. À vérifier après la première exécution.</t>
         </is>
       </c>
       <c r="O38" s="33" t="n"/>
@@ -7679,7 +7679,7 @@
       </c>
       <c r="N39" s="33" t="inlineStr">
         <is>
-          <t>Développé le 15/10 (commit 5b98316, fusionné dans main) : e-mail de confirmation d'achat avec module ou séance, montant, moyen et référence, envoyé une seule fois par commande. À retester en ligne après déploiement, avec un vrai paiement.</t>
+          <t>En ligne depuis le déploiement du 15/10 au soir (5b98316) : e-mail de confirmation d'achat, envoyé une seule fois par commande. À vérifier sur le prochain achat réel.</t>
         </is>
       </c>
       <c r="O39" s="33" t="n"/>
@@ -9997,7 +9997,7 @@
       </c>
       <c r="N77" s="33" t="inlineStr">
         <is>
-          <t>Le paiement d'une séance de coaching privé devient une transaction visible dans /admin/transactions et les revenus. Exige la migration 38 sur la base hébergée (pas encore exécutée au 15/10 au soir).</t>
+          <t>Migration 38 en place (module_id facultatif, vérifié le 15/10) et code en ligne : à vérifier sur le prochain paiement d'une séance de coaching privé.</t>
         </is>
       </c>
       <c r="O77" s="33" t="n"/>
@@ -10546,7 +10546,7 @@
       </c>
       <c r="N86" s="33" t="inlineStr">
         <is>
-          <t>Développé le 15/10 (commit 5b98316, fusionné dans main) : e-mail d'attestation avec le numéro EMBF, le lien vers l'attestation et le lien de vérification, envoyé à la première délivrance. À retester en ligne après déploiement.</t>
+          <t>En ligne depuis le déploiement du 15/10 au soir (5b98316) : e-mail d'attestation à la première délivrance. À vérifier sur la prochaine attestation délivrée.</t>
         </is>
       </c>
       <c r="O86" s="33" t="n"/>
@@ -13249,14 +13249,14 @@
           <t>Testé le 15/10 sur la base en ligne avec la clé publique : 43 tables sur 45 refusent (401). visionnages et reglages_attestation répondent 200 mais vide (RLS filtre tout) : le droit de lecture n'a pas été retiré comme ailleurs, à aligner.</t>
         </is>
       </c>
-      <c r="M130" s="55" t="inlineStr">
-        <is>
-          <t>À retester</t>
+      <c r="M130" s="52" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="N130" s="33" t="inlineStr">
         <is>
-          <t>Migration 37 écrite : RLS activé et droits retirés sur toutes les tables, y compris visionnages et reglages_attestation. À exécuter sur la base hébergée, puis revérifier avec la clé publique.</t>
+          <t>Migration 37 en place le 15/10 au soir, vérifié sur la base hébergée : RLS activé sur toutes les tables, aucun droit accordé à anon ni authenticated, privilèges par défaut fermés pour postgres.</t>
         </is>
       </c>
       <c r="O130" s="33" t="n"/>
@@ -16678,7 +16678,7 @@
       </c>
       <c r="H35" s="33" t="inlineStr">
         <is>
-          <t>Migration 37 écrite, à exécuter sur la base hébergée</t>
+          <t>Fait le 15/10 (migration 37 exécutée et vérifiée)</t>
         </is>
       </c>
     </row>
@@ -16718,7 +16718,7 @@
       </c>
       <c r="H36" s="33" t="inlineStr">
         <is>
-          <t>Développé le 15/10, migration 38 à exécuter avant déploiement</t>
+          <t>En ligne le 15/10 (migration 38 exécutée)</t>
         </is>
       </c>
     </row>
@@ -21161,7 +21161,7 @@
       </c>
       <c r="E5" s="33" t="inlineStr">
         <is>
-          <t>Migrations 01 à 36 en place ; 37 (droits des clés publiques) et 38 (coaching privé dans Transactions) à exécuter dans SQL Editor avant le déploiement du 15/10 au soir</t>
+          <t>Migrations 01 à 38 en place sur la base hébergée (37 et 38 vérifiées le 15/10 au soir)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Intégrer et publier les 5 modules pilotes livrés le 20/10
- ENT 4, 5, 8, 10 et SM 5 : vidéos 720p/1080p en HLS (copie de flux, sans
  réencodage), sous-titres et transcription des 36 chapitres, fiches réécrites
  d'après le contenu réel. Le dossier livré fait foi pour le numéro :
  « Être visible localement » passe en 7, « Comprendre le business du client »
  en 11, « Transformer TikTok… » est créé en 10.
- Lecteur : piste de sous-titres WebVTT signée comme la vidéo, bouton dans la
  barre de contrôles (migration 39 : chapitres.sous_titres).
- Fiches avant modification sauvegardées dans docs/sauvegardes/.
- Classeur et compte rendu : 49 chapitres sur 88 en ligne, 7 modules publiés.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Recette E-Masterclass BigFive — clôture 15-10.xlsx
+++ b/Recette E-Masterclass BigFive — clôture 15-10.xlsx
@@ -2307,7 +2307,7 @@
     <row r="41" ht="27.75" customHeight="1" s="31">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>• Vidéos — 15 chapitres rattachés sur 72 dans la base en ligne ; lecture vérifiée sur le domaine définitif (Worker vidéo autorisé le 15/10).</t>
+          <t>• Vidéos — 49 chapitres sur 88 ont une vidéo dans la base en ligne au 20/10, dont les 36 chapitres des 5 modules pilotes livrés le 20/10 (720p et 1080p, sous-titres, transcription cliquable) ; lecture vérifiée.</t>
         </is>
       </c>
     </row>
@@ -2342,7 +2342,7 @@
     <row r="46" ht="27.75" customHeight="1" s="31">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>• Catalogue : 15 modules sur 18 en brouillon dans la base en ligne.</t>
+          <t>• Catalogue : 7 modules sur 19 publiés au 20/10, dont les 5 modules pilotes ; 11 en brouillon, 1 en préparation.</t>
         </is>
       </c>
     </row>
@@ -4035,7 +4035,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="48" t="inlineStr">
         <is>
@@ -4320,7 +4319,7 @@
       </c>
       <c r="E11" s="50" t="inlineStr">
         <is>
-          <t>15 chapitres sur 72 ont une vidéo au 15/10.</t>
+          <t>49 chapitres sur 88 ont une vidéo au 20/10. Les 5 modules pilotes (36 chapitres) sont intégrés et publiés depuis le 20/10.</t>
         </is>
       </c>
       <c r="F11" s="50" t="inlineStr">
@@ -4362,7 +4361,7 @@
       </c>
       <c r="E12" s="50" t="inlineStr">
         <is>
-          <t>15 modules sur 18 sont en « Brouillon » : le catalogue public en montre 3.</t>
+          <t>11 modules sur 19 sont en « Brouillon » au 20/10 ; 7 sont publiés.</t>
         </is>
       </c>
       <c r="F12" s="50" t="inlineStr">
@@ -4677,8 +4676,6 @@
         </is>
       </c>
     </row>
-    <row r="20"/>
-    <row r="21"/>
     <row r="22">
       <c r="A22" s="48" t="inlineStr">
         <is>
@@ -5108,8 +5105,6 @@
         </is>
       </c>
     </row>
-    <row r="33"/>
-    <row r="34"/>
     <row r="35">
       <c r="A35" s="48" t="inlineStr">
         <is>
@@ -8864,7 +8859,7 @@
       </c>
       <c r="L59" s="33" t="inlineStr">
         <is>
-          <t>Au 15/10, 15 chapitres ont une vidéo dans la base en ligne (2 au 02/09). Les vidéos se déposent depuis /admin/mediatheque.</t>
+          <t>Au 20/10, 49 chapitres ont une vidéo dans la base en ligne (15 au 15/10, 2 au 02/09), dont les 36 des 5 modules pilotes : flux 720p/1080p, sous-titres et transcription. Les autres vidéos se déposent depuis /admin/mediatheque.</t>
         </is>
       </c>
       <c r="M59" s="54" t="inlineStr">
@@ -8874,7 +8869,7 @@
       </c>
       <c r="N59" s="33" t="inlineStr">
         <is>
-          <t>15 chapitres sur 72 ont une vidéo dans la médiathèque au 15/10.</t>
+          <t>49 chapitres sur 88 ont une vidéo au 20/10. Modules pilotes vérifiés en lecture le 20/10 : bascule 720p/1080p, sous-titres, transcription synchronisée, mobile 375 px.</t>
         </is>
       </c>
       <c r="O59" s="53" t="inlineStr">
@@ -15642,7 +15637,7 @@
       </c>
       <c r="H8" s="33" t="inlineStr">
         <is>
-          <t>15 chapitres rattachés au 15/10</t>
+          <t>49 chapitres rattachés au 20/10, dont les 5 modules pilotes complets</t>
         </is>
       </c>
     </row>
@@ -15982,7 +15977,7 @@
       </c>
       <c r="H17" s="33" t="inlineStr">
         <is>
-          <t>15 modules en brouillon dans la base en ligne au 15/10</t>
+          <t>11 modules en brouillon dans la base en ligne au 20/10 (7 publiés)</t>
         </is>
       </c>
     </row>

</xml_diff>